<commit_message>
Update 2 terms in BCIO_Population.xlsx
</commit_message>
<xml_diff>
--- a/Population/BCIO_Population.xlsx
+++ b/Population/BCIO_Population.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -44,12 +44,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ffffff"/>
+        <fgColor rgb="00ffe4b5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002f4f4f"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ffffff"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,12 +70,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3958,11 +3964,11 @@
           <t>quality</t>
         </is>
       </c>
-      <c r="E63" s="3" t="inlineStr"/>
+      <c r="E63" s="3" t="n"/>
       <c r="F63" s="3" t="n"/>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>SDGIO:00010029</t>
+          <t>Sustainable Development Goals Interface Ontology (SDGIO:00010029)</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
@@ -3977,7 +3983,7 @@
         </is>
       </c>
       <c r="J63" s="3" t="n"/>
-      <c r="K63" s="3" t="n"/>
+      <c r="K63" s="3" t="inlineStr"/>
       <c r="L63" s="3" t="n"/>
       <c r="M63" s="3" t="n"/>
       <c r="N63" s="3" t="inlineStr">
@@ -3992,7 +3998,7 @@
       </c>
       <c r="P63" s="3" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Discussed</t>
         </is>
       </c>
       <c r="Q63" s="3" t="n"/>
@@ -6405,7 +6411,7 @@
         </is>
       </c>
       <c r="Q107" s="2" t="n"/>
-      <c r="R107" s="2" t="inlineStr"/>
+      <c r="R107" s="2" t="n"/>
       <c r="S107" s="2" t="n"/>
       <c r="T107" s="2" t="n"/>
       <c r="U107" s="2" t="n"/>
@@ -8377,7 +8383,7 @@
         </is>
       </c>
       <c r="E143" s="2" t="n"/>
-      <c r="F143" s="2" t="inlineStr"/>
+      <c r="F143" s="2" t="n"/>
       <c r="G143" s="2" t="n"/>
       <c r="H143" s="2" t="n"/>
       <c r="I143" s="2" t="inlineStr">
@@ -8466,51 +8472,51 @@
       <c r="U144" s="2" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="3" t="inlineStr">
+      <c r="A145" s="5" t="inlineStr">
         <is>
           <t>BCIO:050976</t>
         </is>
       </c>
-      <c r="B145" s="3" t="inlineStr">
+      <c r="B145" s="5" t="inlineStr">
         <is>
           <t>number of people in a population</t>
         </is>
       </c>
-      <c r="C145" s="3" t="inlineStr">
+      <c r="C145" s="5" t="inlineStr">
         <is>
           <t>A data item about the number of people in a population.</t>
         </is>
       </c>
-      <c r="D145" s="3" t="inlineStr">
+      <c r="D145" s="5" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E145" s="3" t="n"/>
-      <c r="F145" s="3" t="n"/>
-      <c r="G145" s="3" t="n"/>
-      <c r="H145" s="3" t="n"/>
-      <c r="I145" s="3" t="inlineStr">
-        <is>
-          <t>population</t>
-        </is>
-      </c>
-      <c r="J145" s="3" t="n"/>
-      <c r="K145" s="3" t="n"/>
-      <c r="L145" s="3" t="n"/>
-      <c r="M145" s="3" t="n"/>
-      <c r="N145" s="3" t="n"/>
-      <c r="O145" s="3" t="n"/>
-      <c r="P145" s="3" t="inlineStr">
+      <c r="E145" s="5" t="n"/>
+      <c r="F145" s="5" t="n"/>
+      <c r="G145" s="5" t="n"/>
+      <c r="H145" s="5" t="n"/>
+      <c r="I145" s="5" t="inlineStr">
+        <is>
+          <t>population</t>
+        </is>
+      </c>
+      <c r="J145" s="5" t="n"/>
+      <c r="K145" s="5" t="n"/>
+      <c r="L145" s="5" t="n"/>
+      <c r="M145" s="5" t="n"/>
+      <c r="N145" s="5" t="n"/>
+      <c r="O145" s="5" t="n"/>
+      <c r="P145" s="5" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="Q145" s="3" t="n"/>
-      <c r="R145" s="3" t="n"/>
-      <c r="S145" s="3" t="n"/>
-      <c r="T145" s="3" t="n"/>
-      <c r="U145" s="3" t="n"/>
+      <c r="Q145" s="5" t="n"/>
+      <c r="R145" s="5" t="n"/>
+      <c r="S145" s="5" t="n"/>
+      <c r="T145" s="5" t="n"/>
+      <c r="U145" s="5" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -8922,7 +8928,7 @@
       <c r="F153" s="3" t="n"/>
       <c r="G153" s="3" t="inlineStr">
         <is>
-          <t>SDGIO:00010028</t>
+          <t>owner in the Sustainable Development Goals Interface Ontology (SDGIO:00010028)</t>
         </is>
       </c>
       <c r="H153" s="3" t="inlineStr">
@@ -8951,7 +8957,7 @@
       </c>
       <c r="P153" s="3" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Discussed</t>
         </is>
       </c>
       <c r="Q153" s="3" t="n"/>
@@ -9279,52 +9285,52 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="3" t="inlineStr">
+      <c r="A160" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">BCIO:050975
 </t>
         </is>
       </c>
-      <c r="B160" s="3" t="inlineStr">
+      <c r="B160" s="5" t="inlineStr">
         <is>
           <t>people with intervention source role</t>
         </is>
       </c>
-      <c r="C160" s="3" t="inlineStr">
+      <c r="C160" s="5" t="inlineStr">
         <is>
           <t>A &lt;human population&gt; whose members are people with an intervention source role for a specified intervention.</t>
         </is>
       </c>
-      <c r="D160" s="3" t="inlineStr">
+      <c r="D160" s="5" t="inlineStr">
         <is>
           <t>human population</t>
         </is>
       </c>
-      <c r="E160" s="3" t="n"/>
-      <c r="F160" s="3" t="n"/>
-      <c r="G160" s="3" t="n"/>
-      <c r="H160" s="3" t="n"/>
-      <c r="I160" s="3" t="inlineStr">
-        <is>
-          <t>population</t>
-        </is>
-      </c>
-      <c r="J160" s="3" t="n"/>
-      <c r="K160" s="3" t="n"/>
-      <c r="L160" s="3" t="n"/>
-      <c r="M160" s="3" t="n"/>
-      <c r="N160" s="3" t="n"/>
-      <c r="O160" s="3" t="n"/>
-      <c r="P160" s="3" t="inlineStr">
+      <c r="E160" s="5" t="n"/>
+      <c r="F160" s="5" t="n"/>
+      <c r="G160" s="5" t="n"/>
+      <c r="H160" s="5" t="n"/>
+      <c r="I160" s="5" t="inlineStr">
+        <is>
+          <t>population</t>
+        </is>
+      </c>
+      <c r="J160" s="5" t="n"/>
+      <c r="K160" s="5" t="n"/>
+      <c r="L160" s="5" t="n"/>
+      <c r="M160" s="5" t="n"/>
+      <c r="N160" s="5" t="n"/>
+      <c r="O160" s="5" t="n"/>
+      <c r="P160" s="5" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="Q160" s="3" t="n"/>
-      <c r="R160" s="3" t="n"/>
-      <c r="S160" s="3" t="n"/>
-      <c r="T160" s="3" t="n"/>
-      <c r="U160" s="3" t="n"/>
+      <c r="Q160" s="5" t="n"/>
+      <c r="R160" s="5" t="n"/>
+      <c r="S160" s="5" t="n"/>
+      <c r="T160" s="5" t="n"/>
+      <c r="U160" s="5" t="n"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -10265,52 +10271,52 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="3" t="inlineStr">
+      <c r="A179" s="5" t="inlineStr">
         <is>
           <t>BCIO:050978</t>
         </is>
       </c>
-      <c r="B179" s="3" t="inlineStr">
+      <c r="B179" s="5" t="inlineStr">
         <is>
           <t>population statistic</t>
         </is>
       </c>
-      <c r="C179" s="3" t="inlineStr">
+      <c r="C179" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">A data item that is about the number or extent of something in a population. </t>
         </is>
       </c>
-      <c r="D179" s="3" t="inlineStr">
+      <c r="D179" s="5" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E179" s="3" t="n"/>
-      <c r="F179" s="3" t="inlineStr">
+      <c r="E179" s="5" t="n"/>
+      <c r="F179" s="5" t="inlineStr">
         <is>
           <t>Percentage of highly educated individuals in a population. 
 Mean age in a population.</t>
         </is>
       </c>
-      <c r="G179" s="3" t="n"/>
-      <c r="H179" s="3" t="n"/>
-      <c r="I179" s="3" t="n"/>
-      <c r="J179" s="3" t="n"/>
-      <c r="K179" s="3" t="n"/>
-      <c r="L179" s="3" t="n"/>
-      <c r="M179" s="3" t="n"/>
-      <c r="N179" s="3" t="n"/>
-      <c r="O179" s="3" t="n"/>
-      <c r="P179" s="3" t="inlineStr">
+      <c r="G179" s="5" t="n"/>
+      <c r="H179" s="5" t="n"/>
+      <c r="I179" s="5" t="n"/>
+      <c r="J179" s="5" t="n"/>
+      <c r="K179" s="5" t="n"/>
+      <c r="L179" s="5" t="n"/>
+      <c r="M179" s="5" t="n"/>
+      <c r="N179" s="5" t="n"/>
+      <c r="O179" s="5" t="n"/>
+      <c r="P179" s="5" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="Q179" s="3" t="n"/>
-      <c r="R179" s="3" t="n"/>
-      <c r="S179" s="3" t="n"/>
-      <c r="T179" s="3" t="n"/>
-      <c r="U179" s="3" t="n"/>
+      <c r="Q179" s="5" t="n"/>
+      <c r="R179" s="5" t="n"/>
+      <c r="S179" s="5" t="n"/>
+      <c r="T179" s="5" t="n"/>
+      <c r="U179" s="5" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update 11 terms in BCIO_Population.xlsx
</commit_message>
<xml_diff>
--- a/Population/BCIO_Population.xlsx
+++ b/Population/BCIO_Population.xlsx
@@ -49,7 +49,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ffffff"/>
+        <fgColor rgb="00ffe4b5"/>
       </patternFill>
     </fill>
   </fills>
@@ -3628,19 +3628,19 @@
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr"/>
-      <c r="F57" s="4" t="inlineStr"/>
-      <c r="G57" s="4" t="inlineStr"/>
-      <c r="H57" s="4" t="inlineStr"/>
-      <c r="I57" s="4" t="inlineStr"/>
-      <c r="J57" s="4" t="inlineStr"/>
+      <c r="E57" s="4" t="n"/>
+      <c r="F57" s="4" t="n"/>
+      <c r="G57" s="4" t="n"/>
+      <c r="H57" s="4" t="n"/>
+      <c r="I57" s="4" t="n"/>
+      <c r="J57" s="4" t="n"/>
       <c r="K57" s="4" t="inlineStr">
         <is>
           <t>population</t>
         </is>
       </c>
-      <c r="L57" s="4" t="inlineStr"/>
-      <c r="M57" s="4" t="inlineStr"/>
+      <c r="L57" s="4" t="n"/>
+      <c r="M57" s="4" t="n"/>
       <c r="N57" s="4" t="inlineStr">
         <is>
           <t>roles</t>
@@ -3651,16 +3651,16 @@
           <t>percentage; proportion</t>
         </is>
       </c>
-      <c r="P57" s="4" t="inlineStr"/>
-      <c r="Q57" s="4" t="inlineStr"/>
+      <c r="P57" s="4" t="n"/>
+      <c r="Q57" s="4" t="n"/>
       <c r="R57" s="4" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="S57" s="4" t="inlineStr"/>
-      <c r="T57" s="4" t="inlineStr"/>
-      <c r="U57" s="4" t="inlineStr"/>
+          <t>Discussed</t>
+        </is>
+      </c>
+      <c r="S57" s="4" t="n"/>
+      <c r="T57" s="4" t="n"/>
+      <c r="U57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -5130,19 +5130,19 @@
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E84" s="4" t="inlineStr"/>
-      <c r="F84" s="4" t="inlineStr"/>
-      <c r="G84" s="4" t="inlineStr"/>
-      <c r="H84" s="4" t="inlineStr"/>
-      <c r="I84" s="4" t="inlineStr"/>
-      <c r="J84" s="4" t="inlineStr"/>
+      <c r="E84" s="4" t="n"/>
+      <c r="F84" s="4" t="n"/>
+      <c r="G84" s="4" t="n"/>
+      <c r="H84" s="4" t="n"/>
+      <c r="I84" s="4" t="n"/>
+      <c r="J84" s="4" t="n"/>
       <c r="K84" s="4" t="inlineStr">
         <is>
           <t>population</t>
         </is>
       </c>
-      <c r="L84" s="4" t="inlineStr"/>
-      <c r="M84" s="4" t="inlineStr"/>
+      <c r="L84" s="4" t="n"/>
+      <c r="M84" s="4" t="n"/>
       <c r="N84" s="4" t="inlineStr">
         <is>
           <t>roles</t>
@@ -5153,16 +5153,16 @@
           <t>percentage; proportion</t>
         </is>
       </c>
-      <c r="P84" s="4" t="inlineStr"/>
-      <c r="Q84" s="4" t="inlineStr"/>
+      <c r="P84" s="4" t="n"/>
+      <c r="Q84" s="4" t="n"/>
       <c r="R84" s="4" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="S84" s="4" t="inlineStr"/>
-      <c r="T84" s="4" t="inlineStr"/>
-      <c r="U84" s="4" t="inlineStr"/>
+          <t>Discussed</t>
+        </is>
+      </c>
+      <c r="S84" s="4" t="n"/>
+      <c r="T84" s="4" t="n"/>
+      <c r="U84" s="4" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -5634,7 +5634,7 @@
         </is>
       </c>
       <c r="E93" s="3" t="n"/>
-      <c r="F93" s="3" t="inlineStr"/>
+      <c r="F93" s="3" t="n"/>
       <c r="G93" s="3" t="n"/>
       <c r="H93" s="3" t="n"/>
       <c r="I93" s="3" t="n"/>
@@ -5688,23 +5688,23 @@
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E94" s="4" t="inlineStr"/>
+      <c r="E94" s="4" t="n"/>
       <c r="F94" s="4" t="inlineStr">
         <is>
           <t>completing a university bachelor's or master's course of study, medical school or other professional school.</t>
         </is>
       </c>
-      <c r="G94" s="4" t="inlineStr"/>
-      <c r="H94" s="4" t="inlineStr"/>
-      <c r="I94" s="4" t="inlineStr"/>
-      <c r="J94" s="4" t="inlineStr"/>
+      <c r="G94" s="4" t="n"/>
+      <c r="H94" s="4" t="n"/>
+      <c r="I94" s="4" t="n"/>
+      <c r="J94" s="4" t="n"/>
       <c r="K94" s="4" t="inlineStr">
         <is>
           <t>population</t>
         </is>
       </c>
-      <c r="L94" s="4" t="inlineStr"/>
-      <c r="M94" s="4" t="inlineStr"/>
+      <c r="L94" s="4" t="n"/>
+      <c r="M94" s="4" t="n"/>
       <c r="N94" s="4" t="inlineStr">
         <is>
           <t>roles</t>
@@ -5715,16 +5715,16 @@
           <t>percentage; proportion</t>
         </is>
       </c>
-      <c r="P94" s="4" t="inlineStr"/>
-      <c r="Q94" s="4" t="inlineStr"/>
+      <c r="P94" s="4" t="n"/>
+      <c r="Q94" s="4" t="n"/>
       <c r="R94" s="4" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="S94" s="4" t="inlineStr"/>
-      <c r="T94" s="4" t="inlineStr"/>
-      <c r="U94" s="4" t="inlineStr"/>
+          <t>Discussed</t>
+        </is>
+      </c>
+      <c r="S94" s="4" t="n"/>
+      <c r="T94" s="4" t="n"/>
+      <c r="U94" s="4" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -7048,19 +7048,19 @@
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E119" s="4" t="inlineStr"/>
-      <c r="F119" s="4" t="inlineStr"/>
-      <c r="G119" s="4" t="inlineStr"/>
-      <c r="H119" s="4" t="inlineStr"/>
-      <c r="I119" s="4" t="inlineStr"/>
-      <c r="J119" s="4" t="inlineStr"/>
+      <c r="E119" s="4" t="n"/>
+      <c r="F119" s="4" t="n"/>
+      <c r="G119" s="4" t="n"/>
+      <c r="H119" s="4" t="n"/>
+      <c r="I119" s="4" t="n"/>
+      <c r="J119" s="4" t="n"/>
       <c r="K119" s="4" t="inlineStr">
         <is>
           <t>population</t>
         </is>
       </c>
-      <c r="L119" s="4" t="inlineStr"/>
-      <c r="M119" s="4" t="inlineStr"/>
+      <c r="L119" s="4" t="n"/>
+      <c r="M119" s="4" t="n"/>
       <c r="N119" s="4" t="inlineStr">
         <is>
           <t>roles</t>
@@ -7071,16 +7071,16 @@
           <t>percentage; proportion</t>
         </is>
       </c>
-      <c r="P119" s="4" t="inlineStr"/>
-      <c r="Q119" s="4" t="inlineStr"/>
+      <c r="P119" s="4" t="n"/>
+      <c r="Q119" s="4" t="n"/>
       <c r="R119" s="4" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="S119" s="4" t="inlineStr"/>
-      <c r="T119" s="4" t="inlineStr"/>
-      <c r="U119" s="4" t="inlineStr"/>
+          <t>Discussed</t>
+        </is>
+      </c>
+      <c r="S119" s="4" t="n"/>
+      <c r="T119" s="4" t="n"/>
+      <c r="U119" s="4" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -7827,7 +7827,7 @@
         </is>
       </c>
       <c r="P133" s="3" t="n"/>
-      <c r="Q133" s="3" t="inlineStr"/>
+      <c r="Q133" s="3" t="n"/>
       <c r="R133" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
@@ -7858,19 +7858,19 @@
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E134" s="4" t="inlineStr"/>
-      <c r="F134" s="4" t="inlineStr"/>
-      <c r="G134" s="4" t="inlineStr"/>
-      <c r="H134" s="4" t="inlineStr"/>
-      <c r="I134" s="4" t="inlineStr"/>
-      <c r="J134" s="4" t="inlineStr"/>
+      <c r="E134" s="4" t="n"/>
+      <c r="F134" s="4" t="n"/>
+      <c r="G134" s="4" t="n"/>
+      <c r="H134" s="4" t="n"/>
+      <c r="I134" s="4" t="n"/>
+      <c r="J134" s="4" t="n"/>
       <c r="K134" s="4" t="inlineStr">
         <is>
           <t>population</t>
         </is>
       </c>
-      <c r="L134" s="4" t="inlineStr"/>
-      <c r="M134" s="4" t="inlineStr"/>
+      <c r="L134" s="4" t="n"/>
+      <c r="M134" s="4" t="n"/>
       <c r="N134" s="4" t="inlineStr">
         <is>
           <t>roles</t>
@@ -7881,16 +7881,16 @@
           <t>percentage; proportion</t>
         </is>
       </c>
-      <c r="P134" s="4" t="inlineStr"/>
-      <c r="Q134" s="4" t="inlineStr"/>
+      <c r="P134" s="4" t="n"/>
+      <c r="Q134" s="4" t="n"/>
       <c r="R134" s="4" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="S134" s="4" t="inlineStr"/>
-      <c r="T134" s="4" t="inlineStr"/>
-      <c r="U134" s="4" t="inlineStr"/>
+          <t>Discussed</t>
+        </is>
+      </c>
+      <c r="S134" s="4" t="n"/>
+      <c r="T134" s="4" t="n"/>
+      <c r="U134" s="4" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -8788,7 +8788,7 @@
       <c r="Q150" s="4" t="n"/>
       <c r="R150" s="4" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Discussed</t>
         </is>
       </c>
       <c r="S150" s="4" t="n"/>
@@ -9602,7 +9602,7 @@
       <c r="Q165" s="4" t="n"/>
       <c r="R165" s="4" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Discussed</t>
         </is>
       </c>
       <c r="S165" s="4" t="n"/>
@@ -10588,7 +10588,7 @@
       <c r="Q184" s="4" t="n"/>
       <c r="R184" s="4" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Discussed</t>
         </is>
       </c>
       <c r="S184" s="4" t="n"/>
@@ -11486,19 +11486,19 @@
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E201" s="4" t="inlineStr"/>
-      <c r="F201" s="4" t="inlineStr"/>
-      <c r="G201" s="4" t="inlineStr"/>
-      <c r="H201" s="4" t="inlineStr"/>
-      <c r="I201" s="4" t="inlineStr"/>
-      <c r="J201" s="4" t="inlineStr"/>
+      <c r="E201" s="4" t="n"/>
+      <c r="F201" s="4" t="n"/>
+      <c r="G201" s="4" t="n"/>
+      <c r="H201" s="4" t="n"/>
+      <c r="I201" s="4" t="n"/>
+      <c r="J201" s="4" t="n"/>
       <c r="K201" s="4" t="inlineStr">
         <is>
           <t>population</t>
         </is>
       </c>
-      <c r="L201" s="4" t="inlineStr"/>
-      <c r="M201" s="4" t="inlineStr"/>
+      <c r="L201" s="4" t="n"/>
+      <c r="M201" s="4" t="n"/>
       <c r="N201" s="4" t="inlineStr">
         <is>
           <t>roles</t>
@@ -11509,16 +11509,16 @@
           <t>percentage; proportion</t>
         </is>
       </c>
-      <c r="P201" s="4" t="inlineStr"/>
-      <c r="Q201" s="4" t="inlineStr"/>
+      <c r="P201" s="4" t="n"/>
+      <c r="Q201" s="4" t="n"/>
       <c r="R201" s="4" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="S201" s="4" t="inlineStr"/>
-      <c r="T201" s="4" t="inlineStr"/>
-      <c r="U201" s="4" t="inlineStr"/>
+          <t>Discussed</t>
+        </is>
+      </c>
+      <c r="S201" s="4" t="n"/>
+      <c r="T201" s="4" t="n"/>
+      <c r="U201" s="4" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -13247,19 +13247,19 @@
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E234" s="4" t="inlineStr"/>
-      <c r="F234" s="4" t="inlineStr"/>
-      <c r="G234" s="4" t="inlineStr"/>
-      <c r="H234" s="4" t="inlineStr"/>
-      <c r="I234" s="4" t="inlineStr"/>
-      <c r="J234" s="4" t="inlineStr"/>
+      <c r="E234" s="4" t="n"/>
+      <c r="F234" s="4" t="n"/>
+      <c r="G234" s="4" t="n"/>
+      <c r="H234" s="4" t="n"/>
+      <c r="I234" s="4" t="n"/>
+      <c r="J234" s="4" t="n"/>
       <c r="K234" s="4" t="inlineStr">
         <is>
           <t>population</t>
         </is>
       </c>
-      <c r="L234" s="4" t="inlineStr"/>
-      <c r="M234" s="4" t="inlineStr"/>
+      <c r="L234" s="4" t="n"/>
+      <c r="M234" s="4" t="n"/>
       <c r="N234" s="4" t="inlineStr">
         <is>
           <t>roles</t>
@@ -13270,16 +13270,16 @@
           <t>percentage; proportion</t>
         </is>
       </c>
-      <c r="P234" s="4" t="inlineStr"/>
-      <c r="Q234" s="4" t="inlineStr"/>
+      <c r="P234" s="4" t="n"/>
+      <c r="Q234" s="4" t="n"/>
       <c r="R234" s="4" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="S234" s="4" t="inlineStr"/>
-      <c r="T234" s="4" t="inlineStr"/>
-      <c r="U234" s="4" t="inlineStr"/>
+          <t>Discussed</t>
+        </is>
+      </c>
+      <c r="S234" s="4" t="n"/>
+      <c r="T234" s="4" t="n"/>
+      <c r="U234" s="4" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
@@ -13589,19 +13589,19 @@
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E240" s="4" t="inlineStr"/>
-      <c r="F240" s="4" t="inlineStr"/>
-      <c r="G240" s="4" t="inlineStr"/>
-      <c r="H240" s="4" t="inlineStr"/>
-      <c r="I240" s="4" t="inlineStr"/>
-      <c r="J240" s="4" t="inlineStr"/>
+      <c r="E240" s="4" t="n"/>
+      <c r="F240" s="4" t="n"/>
+      <c r="G240" s="4" t="n"/>
+      <c r="H240" s="4" t="n"/>
+      <c r="I240" s="4" t="n"/>
+      <c r="J240" s="4" t="n"/>
       <c r="K240" s="4" t="inlineStr">
         <is>
           <t>population</t>
         </is>
       </c>
-      <c r="L240" s="4" t="inlineStr"/>
-      <c r="M240" s="4" t="inlineStr"/>
+      <c r="L240" s="4" t="n"/>
+      <c r="M240" s="4" t="n"/>
       <c r="N240" s="4" t="inlineStr">
         <is>
           <t>roles</t>
@@ -13612,16 +13612,16 @@
           <t>percentage; proportion</t>
         </is>
       </c>
-      <c r="P240" s="4" t="inlineStr"/>
-      <c r="Q240" s="4" t="inlineStr"/>
+      <c r="P240" s="4" t="n"/>
+      <c r="Q240" s="4" t="n"/>
       <c r="R240" s="4" t="inlineStr">
         <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="S240" s="4" t="inlineStr"/>
-      <c r="T240" s="4" t="inlineStr"/>
-      <c r="U240" s="4" t="inlineStr"/>
+          <t>Discussed</t>
+        </is>
+      </c>
+      <c r="S240" s="4" t="n"/>
+      <c r="T240" s="4" t="n"/>
+      <c r="U240" s="4" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update 9 terms in BCIO_Population.xlsx
</commit_message>
<xml_diff>
--- a/Population/BCIO_Population.xlsx
+++ b/Population/BCIO_Population.xlsx
@@ -451,17 +451,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Examples</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Parent</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Logical definition</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Examples</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -558,15 +558,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Comprehend the German language</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">linguistic capability </t>
         </is>
       </c>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Comprehend the German language</t>
-        </is>
-      </c>
+      <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
@@ -617,15 +617,15 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>The exclusion criteria were an inability to read English</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">linguistic capability </t>
         </is>
       </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>The exclusion criteria were an inability to read English</t>
-        </is>
-      </c>
+      <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="n"/>
@@ -676,15 +676,15 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>Able to speak Chinese.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">linguistic capability </t>
         </is>
       </c>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Able to speak Chinese.</t>
-        </is>
-      </c>
+      <c r="F4" s="2" t="n"/>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
@@ -735,15 +735,15 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>Fluency in written English.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">linguistic capability </t>
         </is>
       </c>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Fluency in written English.</t>
-        </is>
-      </c>
+      <c r="F5" s="2" t="n"/>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="n"/>
@@ -792,12 +792,12 @@
           <t>A highest level of formal education qualification achieved after participating in an education process intended to result in the acquisition and development of skills and knowledge in a specialised discipline that culminated in the award of an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>highest level of formal educational qualification achieved</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -837,7 +837,7 @@
       </c>
       <c r="S6" s="2" t="n"/>
       <c r="T6" s="2" t="n"/>
-      <c r="U6" s="2" t="inlineStr"/>
+      <c r="U6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -855,12 +855,12 @@
           <t xml:space="preserve">A highest level of formal educational qualification achieved after participating in an education process devoted to advanced study and original research that led to the award of a PhD or equivalent level qualification. </t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>highest level of formal educational qualification achieved</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="n"/>
@@ -914,12 +914,12 @@
           <t xml:space="preserve">A highest level of formal educational qualification achieved after participating in an education process intended to introduce very young children to a school-type environment. </t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>highest level of formal educational qualification achieved</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
@@ -973,12 +973,12 @@
           <t>A highest level of formal educational qualification achieved after participating in an education process intended to result in the acquisition and development of skills and knowledge in subject areas more specialised than basic reading, writing and mathematics, with the overall goal of laying the foundation for lifelong learning and human development on which education systems may systematically expand further educational opportunities.</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>highest level of formal educational qualification achieved</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
@@ -1036,12 +1036,12 @@
           <t>A highest level of formal educational qualification achieved after participating in an education process which has as a prerequisite an undergraduate degree and which is intended to result in the acquisition and development of advanced academic or professional skills and knowledge in a specialised discipline, that culminated in the award of a Master's or equivalent degree.</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>highest level of formal educational qualification achieved</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
@@ -1095,12 +1095,12 @@
           <t>A highest level of formal educational qualification achieved after participating in an education process intended to result in the acquisition of fundamental skills in reading, writing and mathematics.</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>highest level of formal educational qualification achieved</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -1160,15 +1160,15 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
+          <t>graduated high school, International Baccaulaureate, A Levels</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
           <t>highest level of formal educational qualification achieved</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>graduated high school, International Baccaulaureate, A Levels</t>
-        </is>
-      </c>
+      <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>OMRSE_00002040</t>
@@ -1225,12 +1225,12 @@
           <t>An adoptive sibling who is male gender.</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>adoptive sibling</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="n"/>
       <c r="H13" s="2" t="n"/>
@@ -1280,12 +1280,12 @@
           <t xml:space="preserve">A child relation in a parent-child relationship established by a legal adoption process. </t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>child relation</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -1339,12 +1339,12 @@
           <t>An adoptive child who is female gender.</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>adoptive child</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
       <c r="H15" s="2" t="n"/>
@@ -1394,12 +1394,12 @@
           <t>An adoptive parent who is male gender.</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>adoptive parent</t>
         </is>
       </c>
-      <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="n"/>
@@ -1449,12 +1449,12 @@
           <t>An adoptive parent who is female gender.</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>adoptive parent</t>
         </is>
       </c>
-      <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="n"/>
       <c r="H17" s="2" t="n"/>
@@ -1504,12 +1504,12 @@
           <t>A parent in a parent-child relationship established by a legal adoption process.</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>parent</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -1563,12 +1563,12 @@
           <t>A sibling with whom the subject shares a parent through a parent-child relationship established by a legal adoption process.</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>sibling</t>
         </is>
       </c>
-      <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="n"/>
@@ -1618,12 +1618,12 @@
           <t>An adoptive sibling who is female gender.</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>adoptive sibling</t>
         </is>
       </c>
-      <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
@@ -1673,12 +1673,12 @@
           <t>An adoptive child who is male gender.</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>adoptive child</t>
         </is>
       </c>
-      <c r="E21" s="2" t="n"/>
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="n"/>
@@ -1728,7 +1728,7 @@
           <t>A person who has reached maturity.</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>person</t>
         </is>
@@ -1775,12 +1775,12 @@
           <t>A rent-free occupier who lives in the residential facility with the agreement of the residential facility owner.</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>rent-free occupier</t>
         </is>
       </c>
-      <c r="E23" s="2" t="n"/>
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
       <c r="H23" s="2" t="n"/>
@@ -1830,12 +1830,12 @@
           <t xml:space="preserve">A sexual orientation of an individual who does not experience sexual attraction. </t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>sexual orientation</t>
         </is>
       </c>
-      <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
@@ -1889,12 +1889,12 @@
           <t>A family member who is the sister of one's parent.</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E25" s="2" t="n"/>
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
@@ -1944,12 +1944,12 @@
           <t>An intervention participant who is exposed to a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>intervention participant</t>
         </is>
       </c>
-      <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="n"/>
@@ -1995,12 +1995,12 @@
           <t>An intervention population who are exposed to a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>intervention population</t>
         </is>
       </c>
-      <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="n"/>
@@ -2042,12 +2042,12 @@
           <t>A data item that is about the rate of individual human behaviour change.</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
@@ -2093,12 +2093,12 @@
           <t>A person who has formed an intention to enact a specified behaviour, and has enacted that behaviour.</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="inlineStr">
@@ -2117,7 +2117,11 @@
       <c r="L29" s="2" t="n"/>
       <c r="M29" s="2" t="n"/>
       <c r="N29" s="2" t="n"/>
-      <c r="O29" s="2" t="n"/>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>percentage; proportion</t>
+        </is>
+      </c>
       <c r="P29" s="2" t="n"/>
       <c r="Q29" s="2" t="n"/>
       <c r="R29" s="2" t="inlineStr">
@@ -2145,12 +2149,12 @@
           <t>A person who has formed an intention to enact a specified behaviour, but has not acted on this intention.</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="n"/>
@@ -2165,7 +2169,11 @@
       <c r="L30" s="2" t="n"/>
       <c r="M30" s="2" t="n"/>
       <c r="N30" s="2" t="n"/>
-      <c r="O30" s="2" t="n"/>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>percentage; proportion</t>
+        </is>
+      </c>
       <c r="P30" s="2" t="n"/>
       <c r="Q30" s="2" t="n"/>
       <c r="R30" s="2" t="inlineStr">
@@ -2193,12 +2201,12 @@
           <t>A person who has not formed an intention to enact a specified behaviour.</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">person </t>
         </is>
       </c>
-      <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="n"/>
@@ -2213,7 +2221,11 @@
       <c r="L31" s="2" t="n"/>
       <c r="M31" s="2" t="n"/>
       <c r="N31" s="2" t="n"/>
-      <c r="O31" s="2" t="n"/>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>percentage; proportion</t>
+        </is>
+      </c>
       <c r="P31" s="2" t="n"/>
       <c r="Q31" s="2" t="n"/>
       <c r="R31" s="2" t="inlineStr">
@@ -2241,12 +2253,12 @@
           <t xml:space="preserve">A data item that is about the number of times a behaviour occurs in a time period. </t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="n"/>
       <c r="H32" s="2" t="n"/>
@@ -2263,8 +2275,16 @@
       </c>
       <c r="L32" s="2" t="n"/>
       <c r="M32" s="2" t="n"/>
-      <c r="N32" s="2" t="n"/>
-      <c r="O32" s="2" t="n"/>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median; percentage; proportion</t>
+        </is>
+      </c>
       <c r="P32" s="2" t="n"/>
       <c r="Q32" s="2" t="n"/>
       <c r="R32" s="2" t="inlineStr">
@@ -2292,12 +2312,12 @@
           <t>A biological sibling who is male gender.</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>biological sibling</t>
         </is>
       </c>
-      <c r="E33" s="2" t="n"/>
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="n"/>
       <c r="H33" s="2" t="n"/>
@@ -2347,12 +2367,12 @@
           <t>A child relation who is genetically related to their parent.</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>child relation</t>
         </is>
       </c>
-      <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="n"/>
       <c r="H34" s="2" t="n"/>
@@ -2402,12 +2422,12 @@
           <t>A biological child who is female gender.</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>biological child</t>
         </is>
       </c>
-      <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="n"/>
       <c r="H35" s="2" t="n"/>
@@ -2457,12 +2477,12 @@
           <t>A biological parent who provided the sperm.</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>biological parent</t>
         </is>
       </c>
-      <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="n"/>
       <c r="H36" s="2" t="n"/>
@@ -2512,12 +2532,12 @@
           <t>A biological parent who provided an egg.</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>biological parent</t>
         </is>
       </c>
-      <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="n"/>
       <c r="H37" s="2" t="n"/>
@@ -2567,12 +2587,12 @@
           <t>A parent who provided one of the gametes that resulted in one's conception.</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>parent</t>
         </is>
       </c>
-      <c r="E38" s="2" t="n"/>
       <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
@@ -2626,12 +2646,12 @@
           <t>A bodily quality based on reproductive function or organs.</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>bodily quality</t>
         </is>
       </c>
-      <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="n"/>
       <c r="H39" s="2" t="n"/>
@@ -2681,12 +2701,12 @@
           <t>A sibling with whom the subject shares a biological parent.</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>sibling</t>
         </is>
       </c>
-      <c r="E40" s="2" t="n"/>
       <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="n"/>
       <c r="H40" s="2" t="n"/>
@@ -2736,12 +2756,12 @@
           <t>A biological sibling who is female gender.</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>biological sibling</t>
         </is>
       </c>
-      <c r="E41" s="2" t="n"/>
       <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="n"/>
       <c r="H41" s="2" t="n"/>
@@ -2791,12 +2811,12 @@
           <t>A biological child who is male gender.</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>biological child</t>
         </is>
       </c>
-      <c r="E42" s="2" t="n"/>
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="n"/>
       <c r="H42" s="2" t="n"/>
@@ -2846,12 +2866,12 @@
           <t>A sexual orientation of an individual who experiences sexual attraction to members of more than one sex.</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>sexual orientation</t>
         </is>
       </c>
-      <c r="E43" s="2" t="n"/>
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
@@ -2905,7 +2925,7 @@
           <t>A quality that inheres in some extended organism.</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>quality</t>
         </is>
@@ -2937,12 +2957,12 @@
           <t>A role which inheres in a person and is realised by the person assuming responsibility for the physical and emotional needs of another who has difficulties with self care.</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="E45" s="2" t="n"/>
       <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="n"/>
       <c r="H45" s="2" t="n"/>
@@ -2992,12 +3012,12 @@
           <t>A personal attribute as belonging to a group within a stratified system of categorisation based on a status conferred at birth based on descent, in which individuals have limited or no mobility due to custom or law.</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="n"/>
       <c r="H46" s="2" t="n"/>
@@ -3024,7 +3044,7 @@
           <t>percentage; proportion</t>
         </is>
       </c>
-      <c r="P46" s="2" t="inlineStr"/>
+      <c r="P46" s="2" t="n"/>
       <c r="Q46" s="2" t="n"/>
       <c r="R46" s="2" t="inlineStr">
         <is>
@@ -3051,12 +3071,12 @@
           <t xml:space="preserve">A person who has not yet reached maturity. </t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="n"/>
       <c r="H47" s="2" t="n"/>
@@ -3110,12 +3130,12 @@
           <t>A family member who is a person's first generation offspring.</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="n"/>
       <c r="H48" s="2" t="n"/>
@@ -3165,12 +3185,12 @@
           <t>A gender identity that matches the person's assigned sex at birth.</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>gender identity</t>
         </is>
       </c>
-      <c r="E49" s="2" t="n"/>
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
@@ -3224,12 +3244,12 @@
           <t xml:space="preserve">A geographic location that is the country in which a person was born. </t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>geographic location</t>
         </is>
       </c>
-      <c r="E50" s="2" t="n"/>
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
@@ -3283,12 +3303,12 @@
           <t>A family member who is a child relation of one's aunt or uncle.</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E51" s="2" t="n"/>
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="n"/>
       <c r="H51" s="2" t="n"/>
@@ -3338,15 +3358,15 @@
           <t>A personal attribute in which the person has impaired physical or mental functioning that has a notable effect on their ability to do typical daily activities.</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D52" s="2" t="n"/>
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E52" s="2" t="n"/>
       <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="n"/>
-      <c r="H52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="n"/>
       <c r="I52" s="2" t="n"/>
       <c r="J52" s="2" t="n"/>
       <c r="K52" s="2" t="inlineStr">
@@ -3367,7 +3387,7 @@
         </is>
       </c>
       <c r="P52" s="2" t="n"/>
-      <c r="Q52" s="2" t="inlineStr"/>
+      <c r="Q52" s="2" t="n"/>
       <c r="R52" s="2" t="inlineStr">
         <is>
           <t>Published</t>
@@ -3395,15 +3415,15 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
+          <t>psychology, counselling, public health</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
           <t>expertise discipline</t>
         </is>
       </c>
-      <c r="E53" s="2" t="n"/>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>psychology, counselling, public health</t>
-        </is>
-      </c>
+      <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="n"/>
       <c r="H53" s="2" t="n"/>
       <c r="I53" s="2" t="n"/>
@@ -3458,15 +3478,15 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
+          <t>Mathematics, English, hairdressing skills, vehicle engineering, nursing, astrophysics, accountancy</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
           <t>expertise discipline</t>
         </is>
       </c>
-      <c r="E54" s="2" t="n"/>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>Mathematics, English, hairdressing skills, vehicle engineering, nursing, astrophysics, accountancy</t>
-        </is>
-      </c>
+      <c r="F54" s="2" t="n"/>
       <c r="G54" s="2" t="n"/>
       <c r="H54" s="2" t="n"/>
       <c r="I54" s="2" t="n"/>
@@ -3515,12 +3535,12 @@
           <t>A relationship status where the individual was previously in a legally formalised relationship and this relationship has now ended or dissolved.</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D55" s="2" t="n"/>
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>relationship status</t>
         </is>
       </c>
-      <c r="E55" s="2" t="n"/>
       <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="n"/>
       <c r="H55" s="2" t="n"/>
@@ -3570,12 +3590,12 @@
           <t>A higher education student  role realised by currently studying for a doctoral degree.</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="D56" s="3" t="n"/>
+      <c r="E56" s="3" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E56" s="3" t="n"/>
       <c r="F56" s="3" t="n"/>
       <c r="G56" s="3" t="n"/>
       <c r="H56" s="3" t="n"/>
@@ -3625,12 +3645,12 @@
           <t>A higher education student  role realised by currently studying for a doctoral degree.</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E57" s="2" t="n"/>
       <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="n"/>
       <c r="H57" s="2" t="n"/>
@@ -3680,12 +3700,12 @@
           <t>A &lt;social group&gt; of two people who interact and influence each other.</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D58" s="2" t="n"/>
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>social group</t>
         </is>
       </c>
-      <c r="E58" s="2" t="n"/>
       <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="n"/>
       <c r="H58" s="2" t="n"/>
@@ -3727,12 +3747,12 @@
           <t>A planned process wherein knowledge and skills is imparted.</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D59" s="2" t="n"/>
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="E59" s="2" t="n"/>
       <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
@@ -3778,12 +3798,12 @@
           <t>An employment status realised by an individual being engaged in an activity or service for wages or salary.</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D60" s="2" t="n"/>
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E60" s="2" t="n"/>
       <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
@@ -3837,12 +3857,12 @@
           <t>An employment status realised by an individual working a standard number of hours defined as full-time by their employer.</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D61" s="2" t="n"/>
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E61" s="2" t="n"/>
       <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
@@ -3896,12 +3916,12 @@
           <t>An employment status realised by an individual working for recurring periods in which different groups of workers do the same jobs in relay.</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D62" s="2" t="n"/>
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E62" s="2" t="n"/>
       <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="n"/>
       <c r="H62" s="2" t="n"/>
@@ -3951,12 +3971,12 @@
           <t>An employment status realised by an individual whose working hours involving less than the standard or customary working time.</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D63" s="2" t="n"/>
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E63" s="2" t="n"/>
       <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
@@ -4010,12 +4030,12 @@
           <t>A quality inhering in a person by virtue of that person bearing a role realised in an employment process.</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="D64" s="2" t="n"/>
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>quality</t>
         </is>
       </c>
-      <c r="E64" s="2" t="n"/>
       <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
@@ -4074,12 +4094,12 @@
           <t>A self-identity as belonging to a social group or groups whose members have a common cultural or ancestral heritage.</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="D65" s="2" t="n"/>
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>self-identity</t>
         </is>
       </c>
-      <c r="E65" s="2" t="n"/>
       <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
@@ -4137,12 +4157,12 @@
           <t>An attribute that is a field of knowledge or practice.</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D66" s="2" t="n"/>
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>specifically dependent continuant</t>
         </is>
       </c>
-      <c r="E66" s="2" t="n"/>
       <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="n"/>
       <c r="H66" s="2" t="n"/>
@@ -4192,12 +4212,12 @@
           <t>A data item that is the extent to which the person’s past behaviour has reached or exceeded a standard.</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="D67" s="2" t="n"/>
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E67" s="2" t="n"/>
       <c r="F67" s="2" t="n"/>
       <c r="G67" s="2" t="n"/>
       <c r="H67" s="2" t="n"/>
@@ -4209,7 +4229,7 @@
         </is>
       </c>
       <c r="L67" s="2" t="n"/>
-      <c r="M67" s="2" t="inlineStr"/>
+      <c r="M67" s="2" t="n"/>
       <c r="N67" s="2" t="inlineStr">
         <is>
           <t>value</t>
@@ -4247,12 +4267,12 @@
           <t>A person who is a member of a group of persons united by blood, or by marriage or other legal arrangement, or by self-identity as belonging to the same family.</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="D68" s="2" t="n"/>
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E68" s="2" t="n"/>
       <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
@@ -4306,12 +4326,12 @@
           <t>A parent who is male gender.</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="D69" s="2" t="n"/>
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>parent</t>
         </is>
       </c>
-      <c r="E69" s="2" t="n"/>
       <c r="F69" s="2" t="n"/>
       <c r="G69" s="2" t="n"/>
       <c r="H69" s="2" t="n"/>
@@ -4361,12 +4381,12 @@
           <t>A biological sex associated with the ability to produce female gametes.</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="D70" s="2" t="n"/>
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>biological sex</t>
         </is>
       </c>
-      <c r="E70" s="2" t="n"/>
       <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="n"/>
       <c r="H70" s="2" t="n"/>
@@ -4416,12 +4436,12 @@
           <t>A gender identity as being female.</t>
         </is>
       </c>
-      <c r="D71" s="2" t="inlineStr">
+      <c r="D71" s="2" t="n"/>
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>gender identity</t>
         </is>
       </c>
-      <c r="E71" s="2" t="n"/>
       <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
@@ -4479,12 +4499,12 @@
           <t>A foster sibling who is male gender.</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="D72" s="2" t="n"/>
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>foster sibling</t>
         </is>
       </c>
-      <c r="E72" s="2" t="n"/>
       <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="n"/>
       <c r="H72" s="2" t="n"/>
@@ -4534,12 +4554,12 @@
           <t xml:space="preserve">A child relation in a parent-child relationship created by a foster care arrangement. </t>
         </is>
       </c>
-      <c r="D73" s="2" t="inlineStr">
+      <c r="D73" s="2" t="n"/>
+      <c r="E73" s="2" t="inlineStr">
         <is>
           <t>child relation</t>
         </is>
       </c>
-      <c r="E73" s="2" t="n"/>
       <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="n"/>
       <c r="H73" s="2" t="n"/>
@@ -4589,12 +4609,12 @@
           <t>A foster child who is female gender.</t>
         </is>
       </c>
-      <c r="D74" s="2" t="inlineStr">
+      <c r="D74" s="2" t="n"/>
+      <c r="E74" s="2" t="inlineStr">
         <is>
           <t>foster child</t>
         </is>
       </c>
-      <c r="E74" s="2" t="n"/>
       <c r="F74" s="2" t="n"/>
       <c r="G74" s="2" t="n"/>
       <c r="H74" s="2" t="n"/>
@@ -4644,12 +4664,12 @@
           <t>A foster parent who is male gender.</t>
         </is>
       </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="D75" s="2" t="n"/>
+      <c r="E75" s="2" t="inlineStr">
         <is>
           <t>foster parent</t>
         </is>
       </c>
-      <c r="E75" s="2" t="n"/>
       <c r="F75" s="2" t="n"/>
       <c r="G75" s="2" t="n"/>
       <c r="H75" s="2" t="n"/>
@@ -4699,12 +4719,12 @@
           <t>A foster parent who is female gender.</t>
         </is>
       </c>
-      <c r="D76" s="2" t="inlineStr">
+      <c r="D76" s="2" t="n"/>
+      <c r="E76" s="2" t="inlineStr">
         <is>
           <t>foster parent</t>
         </is>
       </c>
-      <c r="E76" s="2" t="n"/>
       <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="n"/>
       <c r="H76" s="2" t="n"/>
@@ -4754,12 +4774,12 @@
           <t>A parent who cares for a child who has been placed with them in a foster care arrangement.</t>
         </is>
       </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="D77" s="2" t="n"/>
+      <c r="E77" s="2" t="inlineStr">
         <is>
           <t>parent</t>
         </is>
       </c>
-      <c r="E77" s="2" t="n"/>
       <c r="F77" s="2" t="n"/>
       <c r="G77" s="2" t="inlineStr">
         <is>
@@ -4813,12 +4833,12 @@
           <t>A sibling who shares a parent through a parent-child relationship created by a foster care agreement.</t>
         </is>
       </c>
-      <c r="D78" s="2" t="inlineStr">
+      <c r="D78" s="2" t="n"/>
+      <c r="E78" s="2" t="inlineStr">
         <is>
           <t>sibling</t>
         </is>
       </c>
-      <c r="E78" s="2" t="n"/>
       <c r="F78" s="2" t="n"/>
       <c r="G78" s="2" t="n"/>
       <c r="H78" s="2" t="n"/>
@@ -4868,12 +4888,12 @@
           <t>A foster sibling who is female gender.</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
+      <c r="D79" s="2" t="n"/>
+      <c r="E79" s="2" t="inlineStr">
         <is>
           <t>foster sibling</t>
         </is>
       </c>
-      <c r="E79" s="2" t="n"/>
       <c r="F79" s="2" t="n"/>
       <c r="G79" s="2" t="n"/>
       <c r="H79" s="2" t="n"/>
@@ -4923,12 +4943,12 @@
           <t>A foster child who is male gender.</t>
         </is>
       </c>
-      <c r="D80" s="2" t="inlineStr">
+      <c r="D80" s="2" t="n"/>
+      <c r="E80" s="2" t="inlineStr">
         <is>
           <t>foster child</t>
         </is>
       </c>
-      <c r="E80" s="2" t="n"/>
       <c r="F80" s="2" t="n"/>
       <c r="G80" s="2" t="n"/>
       <c r="H80" s="2" t="n"/>
@@ -4978,12 +4998,12 @@
           <t>A behavioural frequency about the number of times a person has enacted a behaviour per unit of time.</t>
         </is>
       </c>
-      <c r="D81" s="2" t="inlineStr">
+      <c r="D81" s="2" t="n"/>
+      <c r="E81" s="2" t="inlineStr">
         <is>
           <t>behavioural frequency</t>
         </is>
       </c>
-      <c r="E81" s="2" t="n"/>
       <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="n"/>
       <c r="H81" s="2" t="n"/>
@@ -4996,8 +5016,16 @@
       </c>
       <c r="L81" s="2" t="n"/>
       <c r="M81" s="2" t="n"/>
-      <c r="N81" s="2" t="n"/>
-      <c r="O81" s="2" t="n"/>
+      <c r="N81" s="2" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median; percentage; proportion</t>
+        </is>
+      </c>
       <c r="P81" s="2" t="n"/>
       <c r="Q81" s="2" t="n"/>
       <c r="R81" s="2" t="inlineStr">
@@ -5025,12 +5053,12 @@
           <t>A self-identity as having a particular gender, which may or may not correspond with sex assigned at birth.</t>
         </is>
       </c>
-      <c r="D82" s="2" t="inlineStr">
+      <c r="D82" s="2" t="n"/>
+      <c r="E82" s="2" t="inlineStr">
         <is>
           <t>self-identity</t>
         </is>
       </c>
-      <c r="E82" s="2" t="n"/>
       <c r="F82" s="2" t="n"/>
       <c r="G82" s="2" t="n"/>
       <c r="H82" s="2" t="n"/>
@@ -5080,12 +5108,12 @@
           <t>A higher education student role realised by currently studying for a more advanced degree after completing an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D83" s="3" t="inlineStr">
+      <c r="D83" s="3" t="n"/>
+      <c r="E83" s="3" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E83" s="3" t="n"/>
       <c r="F83" s="3" t="n"/>
       <c r="G83" s="3" t="n"/>
       <c r="H83" s="3" t="n"/>
@@ -5135,12 +5163,12 @@
           <t>A higher education student role realised by currently studying for a more advanced degree after completing an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D84" s="2" t="inlineStr">
+      <c r="D84" s="2" t="n"/>
+      <c r="E84" s="2" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E84" s="2" t="n"/>
       <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="n"/>
       <c r="H84" s="2" t="n"/>
@@ -5190,12 +5218,12 @@
           <t>A grandparent who is male gender.</t>
         </is>
       </c>
-      <c r="D85" s="2" t="inlineStr">
+      <c r="D85" s="2" t="n"/>
+      <c r="E85" s="2" t="inlineStr">
         <is>
           <t>grandparent</t>
         </is>
       </c>
-      <c r="E85" s="2" t="n"/>
       <c r="F85" s="2" t="n"/>
       <c r="G85" s="2" t="n"/>
       <c r="H85" s="2" t="n"/>
@@ -5245,12 +5273,12 @@
           <t>A grandparent who is female gender.</t>
         </is>
       </c>
-      <c r="D86" s="2" t="inlineStr">
+      <c r="D86" s="2" t="n"/>
+      <c r="E86" s="2" t="inlineStr">
         <is>
           <t>grandparent</t>
         </is>
       </c>
-      <c r="E86" s="2" t="n"/>
       <c r="F86" s="2" t="n"/>
       <c r="G86" s="2" t="n"/>
       <c r="H86" s="2" t="n"/>
@@ -5300,12 +5328,12 @@
           <t>A family member who is the parent of one's parent.</t>
         </is>
       </c>
-      <c r="D87" s="2" t="inlineStr">
+      <c r="D87" s="2" t="n"/>
+      <c r="E87" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E87" s="2" t="n"/>
       <c r="F87" s="2" t="n"/>
       <c r="G87" s="2" t="n"/>
       <c r="H87" s="2" t="n"/>
@@ -5355,12 +5383,12 @@
           <t xml:space="preserve">A personal history part that includes previously performing a behaviour. </t>
         </is>
       </c>
-      <c r="D88" s="2" t="inlineStr">
+      <c r="D88" s="2" t="n"/>
+      <c r="E88" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E88" s="2" t="n"/>
       <c r="F88" s="2" t="n"/>
       <c r="G88" s="2" t="n"/>
       <c r="H88" s="2" t="n"/>
@@ -5412,15 +5440,15 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
+          <t>having Medicare, Medicaid, Blue Cross, BUPA, being eligible for NHS treatment</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
           <t>policy holder role</t>
         </is>
       </c>
-      <c r="E89" s="2" t="n"/>
-      <c r="F89" s="2" t="inlineStr">
-        <is>
-          <t>having Medicare, Medicaid, Blue Cross, BUPA, being eligible for NHS treatment</t>
-        </is>
-      </c>
+      <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="n"/>
       <c r="H89" s="2" t="n"/>
       <c r="I89" s="2" t="n"/>
@@ -5471,15 +5499,15 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
+          <t>Having chicken pox, asthma, a heart attack</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E90" s="2" t="n"/>
-      <c r="F90" s="2" t="inlineStr">
-        <is>
-          <t>Having chicken pox, asthma, a heart attack</t>
-        </is>
-      </c>
+      <c r="F90" s="2" t="n"/>
       <c r="G90" s="2" t="inlineStr">
         <is>
           <t>NCIT_C16669</t>
@@ -5532,12 +5560,12 @@
           <t>A sexual orientation of an individual who experiences sexual attraction exclusively or primarily to members of a different sex.</t>
         </is>
       </c>
-      <c r="D91" s="2" t="inlineStr">
+      <c r="D91" s="2" t="n"/>
+      <c r="E91" s="2" t="inlineStr">
         <is>
           <t>sexual orientation</t>
         </is>
       </c>
-      <c r="E91" s="2" t="n"/>
       <c r="F91" s="2" t="n"/>
       <c r="G91" s="2" t="inlineStr">
         <is>
@@ -5591,12 +5619,12 @@
           <t>A frequency of past behaviour that is above a threshold.</t>
         </is>
       </c>
-      <c r="D92" s="2" t="inlineStr">
+      <c r="D92" s="2" t="n"/>
+      <c r="E92" s="2" t="inlineStr">
         <is>
           <t>frequency of past behaviour</t>
         </is>
       </c>
-      <c r="E92" s="2" t="n"/>
       <c r="F92" s="2" t="n"/>
       <c r="G92" s="2" t="n"/>
       <c r="H92" s="2" t="n"/>
@@ -5610,7 +5638,11 @@
       <c r="L92" s="2" t="n"/>
       <c r="M92" s="2" t="n"/>
       <c r="N92" s="2" t="n"/>
-      <c r="O92" s="2" t="n"/>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>percentage; proportion</t>
+        </is>
+      </c>
       <c r="P92" s="2" t="n"/>
       <c r="Q92" s="2" t="n"/>
       <c r="R92" s="2" t="inlineStr">
@@ -5638,12 +5670,12 @@
           <t xml:space="preserve">A student or trainee role realised by currently learning on an advanced educational programme in a university, college or professional school. For example, completing a university bachelor's or master's course of study, medical school or other professional school. </t>
         </is>
       </c>
-      <c r="D93" s="3" t="inlineStr">
+      <c r="D93" s="3" t="n"/>
+      <c r="E93" s="3" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E93" s="3" t="n"/>
       <c r="F93" s="3" t="n"/>
       <c r="G93" s="3" t="n"/>
       <c r="H93" s="3" t="n"/>
@@ -5695,15 +5727,15 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
+          <t>completing a university bachelor's or master's course of study, medical school or other professional school.</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E94" s="2" t="n"/>
-      <c r="F94" s="2" t="inlineStr">
-        <is>
-          <t>completing a university bachelor's or master's course of study, medical school or other professional school.</t>
-        </is>
-      </c>
+      <c r="F94" s="2" t="n"/>
       <c r="G94" s="2" t="n"/>
       <c r="H94" s="2" t="n"/>
       <c r="I94" s="2" t="n"/>
@@ -5752,12 +5784,12 @@
           <t>A personal attribute related to the highest level of education achieved.</t>
         </is>
       </c>
-      <c r="D95" s="2" t="inlineStr">
+      <c r="D95" s="2" t="n"/>
+      <c r="E95" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E95" s="2" t="n"/>
       <c r="F95" s="2" t="n"/>
       <c r="G95" s="2" t="inlineStr">
         <is>
@@ -5815,7 +5847,7 @@
           <t>A process that is the sum of the totality of processes taking place in the spatiotemporal region occupied by a material entity or site, including processes on the surface of the entity or within the cavities to which it serves as host.</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="E96" t="inlineStr">
         <is>
           <t>process</t>
         </is>
@@ -5849,15 +5881,15 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
+          <t>history of exposure to asbestos due to one's job</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E97" s="2" t="n"/>
-      <c r="F97" s="2" t="inlineStr">
-        <is>
-          <t>history of exposure to asbestos due to one's job</t>
-        </is>
-      </c>
+      <c r="F97" s="2" t="n"/>
       <c r="G97" s="2" t="n"/>
       <c r="H97" s="2" t="n"/>
       <c r="I97" s="2" t="n"/>
@@ -5908,15 +5940,15 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
+          <t>history of physical abuse by a parent</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E98" s="2" t="n"/>
-      <c r="F98" s="2" t="inlineStr">
-        <is>
-          <t>history of physical abuse by a parent</t>
-        </is>
-      </c>
+      <c r="F98" s="2" t="n"/>
       <c r="G98" s="2" t="n"/>
       <c r="H98" s="2" t="n"/>
       <c r="I98" s="2" t="n"/>
@@ -5965,12 +5997,12 @@
           <t>A person who does not own a residential facility and does not have an agreement with a residential facility owner that would enable them to live in a residential facility.</t>
         </is>
       </c>
-      <c r="D99" s="2" t="inlineStr">
+      <c r="D99" s="2" t="n"/>
+      <c r="E99" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E99" s="2" t="n"/>
       <c r="F99" s="2" t="n"/>
       <c r="G99" s="2" t="n"/>
       <c r="H99" s="2" t="inlineStr">
@@ -6024,12 +6056,12 @@
           <t>A personal attribute inhering in a person who does not bear a role realised in an employment process and who manages their home as their main daily activity.</t>
         </is>
       </c>
-      <c r="D100" s="2" t="inlineStr">
+      <c r="D100" s="2" t="n"/>
+      <c r="E100" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E100" s="2" t="n"/>
       <c r="F100" s="2" t="n"/>
       <c r="G100" s="2" t="inlineStr">
         <is>
@@ -6083,12 +6115,12 @@
           <t>A sexual orientation of an individual who experiences sexual attraction exclusively or primarily to members of the same sex.</t>
         </is>
       </c>
-      <c r="D101" s="2" t="inlineStr">
+      <c r="D101" s="2" t="n"/>
+      <c r="E101" s="2" t="inlineStr">
         <is>
           <t>sexual orientation</t>
         </is>
       </c>
-      <c r="E101" s="2" t="n"/>
       <c r="F101" s="2" t="n"/>
       <c r="G101" s="2" t="inlineStr">
         <is>
@@ -6142,7 +6174,7 @@
           <t>A human or collection of humans that occupies a housing unit by storing their possessions there and habitually sleeping there thereby participating in the realization of its residence function.</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr">
+      <c r="E102" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>
@@ -6179,12 +6211,12 @@
           <t>An aggregate of the individual incomes received by all the members of a household.</t>
         </is>
       </c>
-      <c r="D103" s="2" t="inlineStr">
+      <c r="D103" s="2" t="n"/>
+      <c r="E103" s="2" t="inlineStr">
         <is>
           <t>object aggregate</t>
         </is>
       </c>
-      <c r="E103" s="2" t="n"/>
       <c r="F103" s="2" t="n"/>
       <c r="G103" s="2" t="inlineStr">
         <is>
@@ -6215,7 +6247,7 @@
           <t>Mean;Minimum;Maximum;Median; percentage; proportion</t>
         </is>
       </c>
-      <c r="P103" s="2" t="inlineStr"/>
+      <c r="P103" s="2" t="n"/>
       <c r="Q103" s="2" t="n"/>
       <c r="R103" s="2" t="inlineStr">
         <is>
@@ -6242,12 +6274,12 @@
           <t>A personal attribute that is a time quality inhering in a person by virtue of how long since the person was born.</t>
         </is>
       </c>
-      <c r="D104" s="2" t="inlineStr">
+      <c r="D104" s="2" t="n"/>
+      <c r="E104" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E104" s="2" t="n"/>
       <c r="F104" s="2" t="n"/>
       <c r="G104" s="2" t="inlineStr">
         <is>
@@ -6301,12 +6333,12 @@
           <t>An object aggregate that consists of two or more people.</t>
         </is>
       </c>
-      <c r="D105" s="2" t="inlineStr">
+      <c r="D105" s="2" t="n"/>
+      <c r="E105" s="2" t="inlineStr">
         <is>
           <t>object aggregate</t>
         </is>
       </c>
-      <c r="E105" s="2" t="n"/>
       <c r="F105" s="2" t="n"/>
       <c r="G105" s="2" t="n"/>
       <c r="H105" s="2" t="n"/>
@@ -6348,7 +6380,7 @@
           <t>A cognitive representation of themselves by a person or group.</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr">
+      <c r="E106" t="inlineStr">
         <is>
           <t>cognitive representation</t>
         </is>
@@ -6380,12 +6412,12 @@
           <t>A person who has previously been a resident of a country and is now resident in another country.</t>
         </is>
       </c>
-      <c r="D107" s="2" t="inlineStr">
+      <c r="D107" s="2" t="n"/>
+      <c r="E107" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E107" s="2" t="n"/>
       <c r="F107" s="2" t="n"/>
       <c r="G107" s="2" t="n"/>
       <c r="H107" s="2" t="n"/>
@@ -6435,12 +6467,12 @@
           <t xml:space="preserve">A relationship status where the individual is in a legally formalised marriage or civil partnership. </t>
         </is>
       </c>
-      <c r="D108" s="2" t="inlineStr">
+      <c r="D108" s="2" t="n"/>
+      <c r="E108" s="2" t="inlineStr">
         <is>
           <t>relationship status</t>
         </is>
       </c>
-      <c r="E108" s="2" t="n"/>
       <c r="F108" s="2" t="n"/>
       <c r="G108" s="2" t="n"/>
       <c r="H108" s="2" t="n"/>
@@ -6491,12 +6523,12 @@
           <t>A relationship status where the individual has had the same partner for a significant length of time but is not in a legal union.</t>
         </is>
       </c>
-      <c r="D109" s="2" t="inlineStr">
+      <c r="D109" s="2" t="n"/>
+      <c r="E109" s="2" t="inlineStr">
         <is>
           <t>relationship status</t>
         </is>
       </c>
-      <c r="E109" s="2" t="n"/>
       <c r="F109" s="2" t="n"/>
       <c r="G109" s="2" t="n"/>
       <c r="H109" s="2" t="n"/>
@@ -6550,12 +6582,12 @@
           <t>An employment status realised by an individual working for a company or other organisation without a pre-determined end date, with security of employment and known working conditions.</t>
         </is>
       </c>
-      <c r="D110" s="2" t="inlineStr">
+      <c r="D110" s="2" t="n"/>
+      <c r="E110" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E110" s="2" t="n"/>
       <c r="F110" s="2" t="n"/>
       <c r="G110" s="2" t="n"/>
       <c r="H110" s="2" t="n"/>
@@ -6605,12 +6637,12 @@
           <t>An employment status realised by an individual working for a company or other organisation in a position that is of a known, fixed duration with security of employment for that duration and certain working conditions.</t>
         </is>
       </c>
-      <c r="D111" s="2" t="inlineStr">
+      <c r="D111" s="2" t="n"/>
+      <c r="E111" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E111" s="2" t="n"/>
       <c r="F111" s="2" t="n"/>
       <c r="G111" s="2" t="n"/>
       <c r="H111" s="2" t="n"/>
@@ -6660,12 +6692,12 @@
           <t>An employment status realised by an individual working for a company or other organisation in a position with uncertain duration or hours with unknown or low security of working conditions or pay.</t>
         </is>
       </c>
-      <c r="D112" s="2" t="inlineStr">
+      <c r="D112" s="2" t="n"/>
+      <c r="E112" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E112" s="2" t="n"/>
       <c r="F112" s="2" t="n"/>
       <c r="G112" s="2" t="n"/>
       <c r="H112" s="2" t="n"/>
@@ -6715,12 +6747,12 @@
           <t>Individual income that an individual otherwise of low-income receives as a payment made by the state or an insurance scheme in the form of housing vouchers,  credit or benefits.</t>
         </is>
       </c>
-      <c r="D113" s="2" t="inlineStr">
+      <c r="D113" s="2" t="n"/>
+      <c r="E113" s="2" t="inlineStr">
         <is>
           <t>individual income</t>
         </is>
       </c>
-      <c r="E113" s="2" t="n"/>
       <c r="F113" s="2" t="n"/>
       <c r="G113" s="2" t="n"/>
       <c r="H113" s="2" t="n"/>
@@ -6770,12 +6802,12 @@
           <t>A personal attribute inhering in a person who does not bear a role realised in an employment process due to possessing enough wealth to not need financial support from another person or require income from employment.</t>
         </is>
       </c>
-      <c r="D114" s="2" t="inlineStr">
+      <c r="D114" s="2" t="n"/>
+      <c r="E114" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E114" s="2" t="n"/>
       <c r="F114" s="2" t="n"/>
       <c r="G114" s="2" t="n"/>
       <c r="H114" s="2" t="n"/>
@@ -6827,15 +6859,15 @@
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
+          <t>walks for 15 mins/day, never eats meat, attends school daily</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
           <t>bodily process</t>
         </is>
       </c>
-      <c r="E115" s="2" t="n"/>
-      <c r="F115" s="2" t="inlineStr">
-        <is>
-          <t>walks for 15 mins/day, never eats meat, attends school daily</t>
-        </is>
-      </c>
+      <c r="F115" s="2" t="n"/>
       <c r="G115" s="2" t="n"/>
       <c r="H115" s="2" t="n"/>
       <c r="I115" s="2" t="n"/>
@@ -6884,12 +6916,12 @@
           <t>A personal attribute reflecting a benefit the person receives  derived from their capital or labour, usually measured in money.</t>
         </is>
       </c>
-      <c r="D116" s="2" t="inlineStr">
+      <c r="D116" s="2" t="n"/>
+      <c r="E116" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E116" s="2" t="n"/>
       <c r="F116" s="2" t="n"/>
       <c r="G116" s="2" t="inlineStr">
         <is>
@@ -6943,12 +6975,12 @@
           <t>A social role that involves influencing other people to adopt new ideas or behaviours.</t>
         </is>
       </c>
-      <c r="D117" s="2" t="inlineStr">
+      <c r="D117" s="2" t="n"/>
+      <c r="E117" s="2" t="inlineStr">
         <is>
           <t>social role</t>
         </is>
       </c>
-      <c r="E117" s="2" t="n"/>
       <c r="F117" s="2" t="n"/>
       <c r="G117" s="2" t="n"/>
       <c r="H117" s="2" t="n"/>
@@ -6998,12 +7030,12 @@
           <t>A student or trainee role realised by  currently learning in a non-institutional setting.</t>
         </is>
       </c>
-      <c r="D118" s="3" t="inlineStr">
+      <c r="D118" s="3" t="n"/>
+      <c r="E118" s="3" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E118" s="3" t="n"/>
       <c r="F118" s="3" t="n"/>
       <c r="G118" s="3" t="n"/>
       <c r="H118" s="3" t="n"/>
@@ -7053,12 +7085,12 @@
           <t>A student or trainee that is currently learning in a non-institutional setting.</t>
         </is>
       </c>
-      <c r="D119" s="2" t="inlineStr">
+      <c r="D119" s="2" t="n"/>
+      <c r="E119" s="2" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E119" s="2" t="n"/>
       <c r="F119" s="2" t="n"/>
       <c r="G119" s="2" t="n"/>
       <c r="H119" s="2" t="n"/>
@@ -7108,12 +7140,12 @@
           <t>A patient role which inheres in a person and is realized by being under the care of a physician or health care provider and being admitted to a hospital or equivalent facility.</t>
         </is>
       </c>
-      <c r="D120" s="2" t="inlineStr">
+      <c r="D120" s="2" t="n"/>
+      <c r="E120" s="2" t="inlineStr">
         <is>
           <t>patient role</t>
         </is>
       </c>
-      <c r="E120" s="2" t="n"/>
       <c r="F120" s="2" t="n"/>
       <c r="G120" s="2" t="n"/>
       <c r="H120" s="2" t="n"/>
@@ -7163,12 +7195,12 @@
           <t xml:space="preserve">A role that inheres in an organism that is able to receive benefits from an insurance policy. </t>
         </is>
       </c>
-      <c r="D121" s="3" t="inlineStr">
+      <c r="D121" s="3" t="n"/>
+      <c r="E121" s="3" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="E121" s="3" t="n"/>
       <c r="F121" s="3" t="n"/>
       <c r="G121" s="3" t="inlineStr">
         <is>
@@ -7226,7 +7258,7 @@
           <t xml:space="preserve">A role that inheres in an organism that is able to receive benefits from an insurance policy. </t>
         </is>
       </c>
-      <c r="D122" t="inlineStr">
+      <c r="E122" t="inlineStr">
         <is>
           <t>role</t>
         </is>
@@ -7278,12 +7310,12 @@
           <t>A role relating to personal relationships or association between an individual and other individuals, including kinship relations, romantic, business, and social interactions.</t>
         </is>
       </c>
-      <c r="D123" s="2" t="inlineStr">
+      <c r="D123" s="2" t="n"/>
+      <c r="E123" s="2" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="E123" s="2" t="n"/>
       <c r="F123" s="2" t="n"/>
       <c r="G123" s="2" t="inlineStr">
         <is>
@@ -7337,12 +7369,12 @@
           <t>A person who is exposed to an intervention.</t>
         </is>
       </c>
-      <c r="D124" s="2" t="inlineStr">
+      <c r="D124" s="2" t="n"/>
+      <c r="E124" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E124" s="2" t="n"/>
       <c r="F124" s="2" t="n"/>
       <c r="G124" s="2" t="n"/>
       <c r="H124" s="2" t="n"/>
@@ -7384,12 +7416,12 @@
           <t>A human population who are exposed to an intervention.</t>
         </is>
       </c>
-      <c r="D125" s="2" t="inlineStr">
+      <c r="D125" s="2" t="n"/>
+      <c r="E125" s="2" t="inlineStr">
         <is>
           <t>human population</t>
         </is>
       </c>
-      <c r="E125" s="2" t="n"/>
       <c r="F125" s="2" t="n"/>
       <c r="G125" s="2" t="n"/>
       <c r="H125" s="2" t="n"/>
@@ -7433,15 +7465,15 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Callers eligible for the study were adult cigarette smokers able to communicate in English </t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">linguistic capability </t>
         </is>
       </c>
-      <c r="E126" s="2" t="n"/>
-      <c r="F126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Callers eligible for the study were adult cigarette smokers able to communicate in English </t>
-        </is>
-      </c>
+      <c r="F126" s="2" t="n"/>
       <c r="G126" s="2" t="n"/>
       <c r="H126" s="2" t="n"/>
       <c r="I126" s="2" t="n"/>
@@ -7490,12 +7522,12 @@
           <t>A social role in which the holder is given or creates authority to exert influence on other members of a social group.</t>
         </is>
       </c>
-      <c r="D127" s="2" t="inlineStr">
+      <c r="D127" s="2" t="n"/>
+      <c r="E127" s="2" t="inlineStr">
         <is>
           <t>social role</t>
         </is>
       </c>
-      <c r="E127" s="2" t="n"/>
       <c r="F127" s="2" t="n"/>
       <c r="G127" s="2" t="n"/>
       <c r="H127" s="2" t="n"/>
@@ -7513,7 +7545,11 @@
       <c r="L127" s="2" t="n"/>
       <c r="M127" s="2" t="n"/>
       <c r="N127" s="2" t="n"/>
-      <c r="O127" s="2" t="n"/>
+      <c r="O127" s="2" t="inlineStr">
+        <is>
+          <t>percentage; proportion</t>
+        </is>
+      </c>
       <c r="P127" s="2" t="n"/>
       <c r="Q127" s="2" t="n"/>
       <c r="R127" s="2" t="inlineStr">
@@ -7541,7 +7577,7 @@
           <t>A mental capability that is realised in processes of communication involving language or in expressions of language.</t>
         </is>
       </c>
-      <c r="D128" t="inlineStr">
+      <c r="E128" t="inlineStr">
         <is>
           <t>mental capability</t>
         </is>
@@ -7583,12 +7619,12 @@
           <t>Disabled for at least 12 months.</t>
         </is>
       </c>
-      <c r="D129" s="2" t="inlineStr">
+      <c r="D129" s="2" t="n"/>
+      <c r="E129" s="2" t="inlineStr">
         <is>
           <t>disabled</t>
         </is>
       </c>
-      <c r="E129" s="2" t="n"/>
       <c r="F129" s="2" t="n"/>
       <c r="G129" s="2" t="n"/>
       <c r="H129" s="2" t="n"/>
@@ -7643,12 +7679,12 @@
           <t>A frequency of past behaviour that is below a threshold.</t>
         </is>
       </c>
-      <c r="D130" s="2" t="inlineStr">
+      <c r="D130" s="2" t="n"/>
+      <c r="E130" s="2" t="inlineStr">
         <is>
           <t>frequency of past behaviour</t>
         </is>
       </c>
-      <c r="E130" s="2" t="n"/>
       <c r="F130" s="2" t="n"/>
       <c r="G130" s="2" t="n"/>
       <c r="H130" s="2" t="n"/>
@@ -7662,7 +7698,11 @@
       <c r="L130" s="2" t="n"/>
       <c r="M130" s="2" t="n"/>
       <c r="N130" s="2" t="n"/>
-      <c r="O130" s="2" t="n"/>
+      <c r="O130" s="2" t="inlineStr">
+        <is>
+          <t>percentage; proportion</t>
+        </is>
+      </c>
       <c r="P130" s="2" t="n"/>
       <c r="Q130" s="2" t="n"/>
       <c r="R130" s="2" t="inlineStr">
@@ -7690,12 +7730,12 @@
           <t>A biological sex associated with the ability to produce male gametes.</t>
         </is>
       </c>
-      <c r="D131" s="2" t="inlineStr">
+      <c r="D131" s="2" t="n"/>
+      <c r="E131" s="2" t="inlineStr">
         <is>
           <t>biological sex</t>
         </is>
       </c>
-      <c r="E131" s="2" t="n"/>
       <c r="F131" s="2" t="n"/>
       <c r="G131" s="2" t="n"/>
       <c r="H131" s="2" t="n"/>
@@ -7745,12 +7785,12 @@
           <t>A gender identity as being male.</t>
         </is>
       </c>
-      <c r="D132" s="2" t="inlineStr">
+      <c r="D132" s="2" t="n"/>
+      <c r="E132" s="2" t="inlineStr">
         <is>
           <t>gender identity</t>
         </is>
       </c>
-      <c r="E132" s="2" t="n"/>
       <c r="F132" s="2" t="n"/>
       <c r="G132" s="2" t="inlineStr">
         <is>
@@ -7808,12 +7848,12 @@
           <t>A higher education student  role realised by currently studying for a masters degree.</t>
         </is>
       </c>
-      <c r="D133" s="3" t="inlineStr">
+      <c r="D133" s="3" t="n"/>
+      <c r="E133" s="3" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E133" s="3" t="n"/>
       <c r="F133" s="3" t="n"/>
       <c r="G133" s="3" t="n"/>
       <c r="H133" s="3" t="n"/>
@@ -7863,12 +7903,12 @@
           <t>A higher education student  role realised by currently studying for a masters degree.</t>
         </is>
       </c>
-      <c r="D134" s="2" t="inlineStr">
+      <c r="D134" s="2" t="n"/>
+      <c r="E134" s="2" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E134" s="2" t="n"/>
       <c r="F134" s="2" t="n"/>
       <c r="G134" s="2" t="n"/>
       <c r="H134" s="2" t="n"/>
@@ -7920,15 +7960,15 @@
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
+          <t>prescribed at least one antihypertensive medication, taking asthma preventer inhalers</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
           <t>health status attribute</t>
         </is>
       </c>
-      <c r="E135" s="2" t="n"/>
-      <c r="F135" s="2" t="inlineStr">
-        <is>
-          <t>prescribed at least one antihypertensive medication, taking asthma preventer inhalers</t>
-        </is>
-      </c>
+      <c r="F135" s="2" t="n"/>
       <c r="G135" s="2" t="n"/>
       <c r="H135" s="2" t="n"/>
       <c r="I135" s="2" t="n"/>
@@ -7981,12 +8021,12 @@
           <t>A person living in  a household with at least one other person.</t>
         </is>
       </c>
-      <c r="D136" s="2" t="inlineStr">
+      <c r="D136" s="2" t="n"/>
+      <c r="E136" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E136" s="2" t="n"/>
       <c r="F136" s="2" t="n"/>
       <c r="G136" s="2" t="n"/>
       <c r="H136" s="2" t="n"/>
@@ -8042,15 +8082,15 @@
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
+          <t>1) Co-habitating couple and their socially recognised children and elderly parents. 2) Co habitating couple with child and grandchild.</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
           <t>member of a multi-person household</t>
         </is>
       </c>
-      <c r="E137" s="2" t="n"/>
-      <c r="F137" s="2" t="inlineStr">
-        <is>
-          <t>1) Co-habitating couple and their socially recognised children and elderly parents. 2) Co habitating couple with child and grandchild.</t>
-        </is>
-      </c>
+      <c r="F137" s="2" t="n"/>
       <c r="G137" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">NCIT:C25173;PCO:0000020;STATO:0000257 </t>
@@ -8105,15 +8145,15 @@
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
+          <t>1) Two unrelated couples (unmarried couples). 2) Students sharing living accommodation. 3) Single professionals renting a room in a shared house.</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
           <t>member of a multi-person household</t>
         </is>
       </c>
-      <c r="E138" s="2" t="n"/>
-      <c r="F138" s="2" t="inlineStr">
-        <is>
-          <t>1) Two unrelated couples (unmarried couples). 2) Students sharing living accommodation. 3) Single professionals renting a room in a shared house.</t>
-        </is>
-      </c>
+      <c r="F138" s="2" t="n"/>
       <c r="G138" s="2" t="n"/>
       <c r="H138" s="2" t="n"/>
       <c r="I138" s="2" t="n"/>
@@ -8164,15 +8204,15 @@
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
+          <t>1) Cohabiting couple plus son and girlfriend. 2) Two brothers and their partners</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
           <t>member of a multi-person household</t>
         </is>
       </c>
-      <c r="E139" s="2" t="n"/>
-      <c r="F139" s="2" t="inlineStr">
-        <is>
-          <t>1) Cohabiting couple plus son and girlfriend. 2) Two brothers and their partners</t>
-        </is>
-      </c>
+      <c r="F139" s="2" t="n"/>
       <c r="G139" s="2" t="n"/>
       <c r="H139" s="2" t="n"/>
       <c r="I139" s="2" t="n"/>
@@ -8223,15 +8263,15 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
+          <t>1) A family unit of a pair of adults and their socially recognized children. 2) Co-habitating couples plus socially recognised children and elderly parents or grandchildren.</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
           <t>member of a multi-person household</t>
         </is>
       </c>
-      <c r="E140" s="2" t="n"/>
-      <c r="F140" s="2" t="inlineStr">
-        <is>
-          <t>1) A family unit of a pair of adults and their socially recognized children. 2) Co-habitating couples plus socially recognised children and elderly parents or grandchildren.</t>
-        </is>
-      </c>
+      <c r="F140" s="2" t="n"/>
       <c r="G140" s="2" t="n"/>
       <c r="H140" s="2" t="n"/>
       <c r="I140" s="2" t="n"/>
@@ -8284,12 +8324,12 @@
           <t>A person living alone in a household.</t>
         </is>
       </c>
-      <c r="D141" s="2" t="inlineStr">
+      <c r="D141" s="2" t="n"/>
+      <c r="E141" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E141" s="2" t="n"/>
       <c r="F141" s="2" t="n"/>
       <c r="G141" s="2" t="n"/>
       <c r="H141" s="2" t="n"/>
@@ -8339,7 +8379,7 @@
           <t>A personal capability that includes mental processes in its realisation.</t>
         </is>
       </c>
-      <c r="D142" t="inlineStr">
+      <c r="E142" t="inlineStr">
         <is>
           <t>personal capability</t>
         </is>
@@ -8381,12 +8421,12 @@
           <t>A parent who is female gender.</t>
         </is>
       </c>
-      <c r="D143" s="2" t="inlineStr">
+      <c r="D143" s="2" t="n"/>
+      <c r="E143" s="2" t="inlineStr">
         <is>
           <t>parent</t>
         </is>
       </c>
-      <c r="E143" s="2" t="n"/>
       <c r="F143" s="2" t="n"/>
       <c r="G143" s="2" t="n"/>
       <c r="H143" s="2" t="n"/>
@@ -8436,12 +8476,12 @@
           <t xml:space="preserve">A family member who is a child relation of one's sibling and is male gender. </t>
         </is>
       </c>
-      <c r="D144" s="2" t="inlineStr">
+      <c r="D144" s="2" t="n"/>
+      <c r="E144" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E144" s="2" t="n"/>
       <c r="F144" s="2" t="n"/>
       <c r="G144" s="2" t="n"/>
       <c r="H144" s="2" t="n"/>
@@ -8491,12 +8531,12 @@
           <t>A family member who is a child relation of one's sibling and is female gender.</t>
         </is>
       </c>
-      <c r="D145" s="2" t="inlineStr">
+      <c r="D145" s="2" t="n"/>
+      <c r="E145" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E145" s="2" t="n"/>
       <c r="F145" s="2" t="n"/>
       <c r="G145" s="2" t="n"/>
       <c r="H145" s="2" t="n"/>
@@ -8546,12 +8586,12 @@
           <t>A self-identity as not having a particular gender.</t>
         </is>
       </c>
-      <c r="D146" s="2" t="inlineStr">
+      <c r="D146" s="2" t="n"/>
+      <c r="E146" s="2" t="inlineStr">
         <is>
           <t>self-identity</t>
         </is>
       </c>
-      <c r="E146" s="2" t="n"/>
       <c r="F146" s="2" t="n"/>
       <c r="G146" s="2" t="inlineStr">
         <is>
@@ -8605,12 +8645,12 @@
           <t>A gender identity as having a gender that is not well-described by the binary categories of male or female.</t>
         </is>
       </c>
-      <c r="D147" s="2" t="inlineStr">
+      <c r="D147" s="2" t="n"/>
+      <c r="E147" s="2" t="inlineStr">
         <is>
           <t>gender identity</t>
         </is>
       </c>
-      <c r="E147" s="2" t="n"/>
       <c r="F147" s="2" t="n"/>
       <c r="G147" s="2" t="inlineStr">
         <is>
@@ -8664,12 +8704,12 @@
           <t>A personal attribute inhering in a person by virtue of that person not having a paid job and not currently seeking to begin participating in an employment process.</t>
         </is>
       </c>
-      <c r="D148" s="2" t="inlineStr">
+      <c r="D148" s="2" t="n"/>
+      <c r="E148" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E148" s="2" t="n"/>
       <c r="F148" s="2" t="n"/>
       <c r="G148" s="2" t="n"/>
       <c r="H148" s="2" t="n"/>
@@ -8719,12 +8759,12 @@
           <t>A personal attribute inhering in a person by virtue of that person not bearing a role realised in an employment process, due to being unable to work due to illness or disability.</t>
         </is>
       </c>
-      <c r="D149" s="2" t="inlineStr">
+      <c r="D149" s="2" t="n"/>
+      <c r="E149" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E149" s="2" t="n"/>
       <c r="F149" s="2" t="n"/>
       <c r="G149" s="2" t="n"/>
       <c r="H149" s="2" t="n"/>
@@ -8774,12 +8814,12 @@
           <t>A data item about the number of people in a population.</t>
         </is>
       </c>
-      <c r="D150" s="2" t="inlineStr">
+      <c r="D150" s="2" t="n"/>
+      <c r="E150" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E150" s="2" t="n"/>
       <c r="F150" s="2" t="n"/>
       <c r="G150" s="2" t="n"/>
       <c r="H150" s="2" t="n"/>
@@ -8821,12 +8861,12 @@
           <t>The number of years a person spent engaged in an education process.</t>
         </is>
       </c>
-      <c r="D151" s="2" t="inlineStr">
+      <c r="D151" s="2" t="n"/>
+      <c r="E151" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E151" s="2" t="n"/>
       <c r="F151" s="2" t="n"/>
       <c r="G151" s="2" t="n"/>
       <c r="H151" s="2" t="n"/>
@@ -8880,12 +8920,12 @@
           <t>A personal role that is realised in a person by doing a specified type of work or working in a specified way.</t>
         </is>
       </c>
-      <c r="D152" s="2" t="inlineStr">
+      <c r="D152" s="2" t="n"/>
+      <c r="E152" s="2" t="inlineStr">
         <is>
           <t>personal role</t>
         </is>
       </c>
-      <c r="E152" s="2" t="n"/>
       <c r="F152" s="2" t="n"/>
       <c r="G152" s="2" t="n"/>
       <c r="H152" s="2" t="n"/>
@@ -8935,12 +8975,12 @@
           <t>A person who lives in a residential facility they do not own  with the agreement of the residential facility owner, by virtue of the occupier bearing a role realised in an employment process.</t>
         </is>
       </c>
-      <c r="D153" s="2" t="inlineStr">
+      <c r="D153" s="2" t="n"/>
+      <c r="E153" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E153" s="2" t="n"/>
       <c r="F153" s="2" t="n"/>
       <c r="G153" s="2" t="n"/>
       <c r="H153" s="2" t="n"/>
@@ -8992,15 +9032,15 @@
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
+          <t>Scout leader, club chairperson</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
           <t>role</t>
         </is>
       </c>
-      <c r="E154" s="2" t="n"/>
-      <c r="F154" s="2" t="inlineStr">
-        <is>
-          <t>Scout leader, club chairperson</t>
-        </is>
-      </c>
+      <c r="F154" s="2" t="n"/>
       <c r="G154" s="2" t="n"/>
       <c r="H154" s="2" t="n"/>
       <c r="I154" s="2" t="n"/>
@@ -9049,12 +9089,12 @@
           <t>A sexual orientation of an individual who is sure of their sexual orientation and reports it as other than asexual, bisexual, heterosexual, homosexual, queer or questioning.</t>
         </is>
       </c>
-      <c r="D155" s="2" t="inlineStr">
+      <c r="D155" s="2" t="n"/>
+      <c r="E155" s="2" t="inlineStr">
         <is>
           <t>sexual orientation</t>
         </is>
       </c>
-      <c r="E155" s="2" t="n"/>
       <c r="F155" s="2" t="n"/>
       <c r="G155" s="2" t="n"/>
       <c r="H155" s="2" t="n"/>
@@ -9104,12 +9144,12 @@
           <t>A social group that is part of a person’s social environmental system and with which the person does not identify.</t>
         </is>
       </c>
-      <c r="D156" s="2" t="inlineStr">
+      <c r="D156" s="2" t="n"/>
+      <c r="E156" s="2" t="inlineStr">
         <is>
           <t>social group</t>
         </is>
       </c>
-      <c r="E156" s="2" t="n"/>
       <c r="F156" s="2" t="n"/>
       <c r="G156" s="2" t="n"/>
       <c r="H156" s="2" t="n"/>
@@ -9151,12 +9191,12 @@
           <t>A patient role which inheres in a person and is realized by coming to a healthcare facility for diagnosis or treatment but not being admitted for an overnight stay.</t>
         </is>
       </c>
-      <c r="D157" s="2" t="inlineStr">
+      <c r="D157" s="2" t="n"/>
+      <c r="E157" s="2" t="inlineStr">
         <is>
           <t>patient role</t>
         </is>
       </c>
-      <c r="E157" s="2" t="n"/>
       <c r="F157" s="2" t="n"/>
       <c r="G157" s="2" t="n"/>
       <c r="H157" s="2" t="n"/>
@@ -9206,12 +9246,12 @@
           <t>A person or organization that participates in an ownership process wherein they realize their role as owner by exercising their right to use, sell, rent, or gift an object.</t>
         </is>
       </c>
-      <c r="D158" s="2" t="inlineStr">
+      <c r="D158" s="2" t="n"/>
+      <c r="E158" s="2" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>
       </c>
-      <c r="E158" s="2" t="n"/>
       <c r="F158" s="2" t="n"/>
       <c r="G158" s="2" t="inlineStr">
         <is>
@@ -9269,12 +9309,12 @@
           <t>A person who lives in a residential facility of which they are the residential facility owner</t>
         </is>
       </c>
-      <c r="D159" s="2" t="inlineStr">
+      <c r="D159" s="2" t="n"/>
+      <c r="E159" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E159" s="2" t="n"/>
       <c r="F159" s="2" t="n"/>
       <c r="G159" s="2" t="n"/>
       <c r="H159" s="2" t="n"/>
@@ -9325,12 +9365,12 @@
           <t xml:space="preserve">A family member who is a key caretaker or immediate progenitor of a child. </t>
         </is>
       </c>
-      <c r="D160" s="2" t="inlineStr">
+      <c r="D160" s="2" t="n"/>
+      <c r="E160" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E160" s="2" t="n"/>
       <c r="F160" s="2" t="n"/>
       <c r="G160" s="2" t="inlineStr">
         <is>
@@ -9384,12 +9424,12 @@
           <t>An interpersonal role that is realised through a process of promoting and supporting the physical, emotional, social, and intellectual development of a child from infancy to adulthood.</t>
         </is>
       </c>
-      <c r="D161" s="2" t="inlineStr">
+      <c r="D161" s="2" t="n"/>
+      <c r="E161" s="2" t="inlineStr">
         <is>
           <t>interpersonal role</t>
         </is>
       </c>
-      <c r="E161" s="2" t="n"/>
       <c r="F161" s="2" t="n"/>
       <c r="G161" s="2" t="n"/>
       <c r="H161" s="2" t="n"/>
@@ -9443,12 +9483,12 @@
           <t>A personal history part that includes a behaviour.</t>
         </is>
       </c>
-      <c r="D162" s="2" t="inlineStr">
+      <c r="D162" s="2" t="n"/>
+      <c r="E162" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E162" s="2" t="n"/>
       <c r="F162" s="2" t="n"/>
       <c r="G162" s="2" t="n"/>
       <c r="H162" s="2" t="n"/>
@@ -9498,12 +9538,12 @@
           <t>A past behaviour that is the target of an intervention.</t>
         </is>
       </c>
-      <c r="D163" s="2" t="inlineStr">
+      <c r="D163" s="2" t="n"/>
+      <c r="E163" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">past behaviour </t>
         </is>
       </c>
-      <c r="E163" s="2" t="n"/>
       <c r="F163" s="2" t="n"/>
       <c r="G163" s="2" t="n"/>
       <c r="H163" s="2" t="n"/>
@@ -9517,7 +9557,11 @@
       <c r="L163" s="2" t="n"/>
       <c r="M163" s="2" t="n"/>
       <c r="N163" s="2" t="n"/>
-      <c r="O163" s="2" t="n"/>
+      <c r="O163" s="2" t="inlineStr">
+        <is>
+          <t>Mean;Minimum;Maximum;Median; percentage; proportion</t>
+        </is>
+      </c>
       <c r="P163" s="2" t="n"/>
       <c r="Q163" s="2" t="n"/>
       <c r="R163" s="2" t="inlineStr">
@@ -9545,7 +9589,7 @@
           <t>A role which inheres in a person and is realized by being under the care of a physician or health care provider.</t>
         </is>
       </c>
-      <c r="D164" t="inlineStr">
+      <c r="E164" t="inlineStr">
         <is>
           <t>role</t>
         </is>
@@ -9588,12 +9632,12 @@
           <t>A &lt;human population&gt; whose members are people with an intervention source role for a specified intervention.</t>
         </is>
       </c>
-      <c r="D165" s="2" t="inlineStr">
+      <c r="D165" s="2" t="n"/>
+      <c r="E165" s="2" t="inlineStr">
         <is>
           <t>human population</t>
         </is>
       </c>
-      <c r="E165" s="2" t="n"/>
       <c r="F165" s="2" t="n"/>
       <c r="G165" s="2" t="n"/>
       <c r="H165" s="2" t="n"/>
@@ -9635,7 +9679,7 @@
           <t>An extended organism that is a member of the species Homo sapiens.</t>
         </is>
       </c>
-      <c r="D166" t="inlineStr">
+      <c r="E166" t="inlineStr">
         <is>
           <t>extended organism</t>
         </is>
@@ -9667,12 +9711,12 @@
           <t>A &lt;person&gt; who is part of a social environmental system.</t>
         </is>
       </c>
-      <c r="D167" s="2" t="inlineStr">
+      <c r="D167" s="2" t="n"/>
+      <c r="E167" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E167" s="2" t="n"/>
       <c r="F167" s="2" t="n"/>
       <c r="G167" s="2" t="n"/>
       <c r="H167" s="2" t="n"/>
@@ -9714,12 +9758,12 @@
           <t>A specifically dependent continuant that inheres in a person.</t>
         </is>
       </c>
-      <c r="D168" s="2" t="inlineStr">
+      <c r="D168" s="2" t="n"/>
+      <c r="E168" s="2" t="inlineStr">
         <is>
           <t>specifically dependent continuant</t>
         </is>
       </c>
-      <c r="E168" s="2" t="n"/>
       <c r="F168" s="2" t="n"/>
       <c r="G168" s="2" t="n"/>
       <c r="H168" s="2" t="n"/>
@@ -9769,7 +9813,7 @@
           <t>A bodily disposition whose realization ordinarily brings benefits to an organism or group of organisms, where "ordinarily" means within a typical range or context.</t>
         </is>
       </c>
-      <c r="D169" t="inlineStr">
+      <c r="E169" t="inlineStr">
         <is>
           <t>bodily disposition</t>
         </is>
@@ -9812,12 +9856,12 @@
           <t>A history that is of a person.</t>
         </is>
       </c>
-      <c r="D170" s="2" t="inlineStr">
+      <c r="D170" s="2" t="n"/>
+      <c r="E170" s="2" t="inlineStr">
         <is>
           <t>history</t>
         </is>
       </c>
-      <c r="E170" s="2" t="n"/>
       <c r="F170" s="2" t="n"/>
       <c r="G170" s="2" t="n"/>
       <c r="H170" s="2" t="n"/>
@@ -9859,12 +9903,12 @@
           <t xml:space="preserve">A personal history part that includes a change from a less desired behaviour pattern to a more desired behaviour pattern followed by a temporary reversion to the previous behaviour pattern. </t>
         </is>
       </c>
-      <c r="D171" s="2" t="inlineStr">
+      <c r="D171" s="2" t="n"/>
+      <c r="E171" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E171" s="2" t="n"/>
       <c r="F171" s="2" t="n"/>
       <c r="G171" s="2" t="n"/>
       <c r="H171" s="2" t="n"/>
@@ -9914,12 +9958,12 @@
           <t xml:space="preserve">A personal history part that includes experience of events that influence behaviour. </t>
         </is>
       </c>
-      <c r="D172" s="2" t="inlineStr">
+      <c r="D172" s="2" t="n"/>
+      <c r="E172" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E172" s="2" t="n"/>
       <c r="F172" s="2" t="n"/>
       <c r="G172" s="2" t="n"/>
       <c r="H172" s="2" t="n"/>
@@ -9969,12 +10013,12 @@
           <t>A personal history part of exposure to an intervention targeting the same outcome as the current intervention.</t>
         </is>
       </c>
-      <c r="D173" s="2" t="inlineStr">
+      <c r="D173" s="2" t="n"/>
+      <c r="E173" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E173" s="2" t="n"/>
       <c r="F173" s="2" t="n"/>
       <c r="G173" s="2" t="n"/>
       <c r="H173" s="2" t="n"/>
@@ -10024,12 +10068,12 @@
           <t>A personal history part  that includes exposure to a prior intervention targeting the same outcome behaviour as the current intervention.</t>
         </is>
       </c>
-      <c r="D174" s="2" t="inlineStr">
+      <c r="D174" s="2" t="n"/>
+      <c r="E174" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E174" s="2" t="n"/>
       <c r="F174" s="2" t="n"/>
       <c r="G174" s="2" t="n"/>
       <c r="H174" s="2" t="n"/>
@@ -10079,12 +10123,12 @@
           <t>A personal history part that includes exposure to the same intervention as the current intervention.</t>
         </is>
       </c>
-      <c r="D175" s="2" t="inlineStr">
+      <c r="D175" s="2" t="n"/>
+      <c r="E175" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E175" s="2" t="n"/>
       <c r="F175" s="2" t="n"/>
       <c r="G175" s="2" t="n"/>
       <c r="H175" s="2" t="n"/>
@@ -10138,17 +10182,17 @@
           <t>A process that is part of a personal history.</t>
         </is>
       </c>
-      <c r="D176" s="2" t="inlineStr">
+      <c r="D176" s="2" t="n"/>
+      <c r="E176" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="E176" s="2" t="inlineStr">
+      <c r="F176" s="2" t="inlineStr">
         <is>
           <t>'process' and 'part of' some 'personal history'</t>
         </is>
       </c>
-      <c r="F176" s="2" t="n"/>
       <c r="G176" s="2" t="n"/>
       <c r="H176" s="2" t="n"/>
       <c r="I176" s="2" t="n"/>
@@ -10189,12 +10233,12 @@
           <t xml:space="preserve">A personal history part  that includes exposure to one or more interventions. </t>
         </is>
       </c>
-      <c r="D177" s="2" t="inlineStr">
+      <c r="D177" s="2" t="n"/>
+      <c r="E177" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E177" s="2" t="n"/>
       <c r="F177" s="2" t="n"/>
       <c r="G177" s="2" t="n"/>
       <c r="H177" s="2" t="n"/>
@@ -10246,15 +10290,15 @@
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
+          <t>low motivation to quit,  low self efficacy for physical activity, negative attitudes to healthy eating, contemplation stage of change, low numeracy</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E178" s="2" t="n"/>
-      <c r="F178" s="2" t="inlineStr">
-        <is>
-          <t>low motivation to quit,  low self efficacy for physical activity, negative attitudes to healthy eating, contemplation stage of change, low numeracy</t>
-        </is>
-      </c>
+      <c r="F178" s="2" t="n"/>
       <c r="G178" s="2" t="n"/>
       <c r="H178" s="2" t="n"/>
       <c r="I178" s="2" t="n"/>
@@ -10303,12 +10347,12 @@
           <t>A role that inheres in a human being by virtue of their social and institutional circumstances.</t>
         </is>
       </c>
-      <c r="D179" s="2" t="inlineStr">
+      <c r="D179" s="2" t="n"/>
+      <c r="E179" s="2" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="E179" s="2" t="n"/>
       <c r="F179" s="2" t="n"/>
       <c r="G179" s="2" t="n"/>
       <c r="H179" s="2" t="n"/>
@@ -10360,15 +10404,15 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
+          <t>susceptibility to addiction, vulnerability to depression</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
           <t>disposition</t>
         </is>
       </c>
-      <c r="E180" s="2" t="n"/>
-      <c r="F180" s="2" t="inlineStr">
-        <is>
-          <t>susceptibility to addiction, vulnerability to depression</t>
-        </is>
-      </c>
+      <c r="F180" s="2" t="n"/>
       <c r="G180" s="2" t="n"/>
       <c r="H180" s="2" t="n"/>
       <c r="I180" s="2" t="n"/>
@@ -10417,12 +10461,12 @@
           <t>A personal vulnerability towards performing a behaviour that causes net harm.</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D181" s="2" t="n"/>
+      <c r="E181" s="2" t="inlineStr">
         <is>
           <t>personal vulnerability</t>
         </is>
       </c>
-      <c r="E181" s="2" t="n"/>
       <c r="F181" s="2" t="n"/>
       <c r="G181" s="2" t="n"/>
       <c r="H181" s="2" t="inlineStr">
@@ -10476,12 +10520,12 @@
           <t>A geographic location in which a person resides.</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D182" s="2" t="n"/>
+      <c r="E182" s="2" t="inlineStr">
         <is>
           <t>geographic location</t>
         </is>
       </c>
-      <c r="E182" s="2" t="n"/>
       <c r="F182" s="2" t="n"/>
       <c r="G182" s="2" t="n"/>
       <c r="H182" s="2" t="n"/>
@@ -10531,7 +10575,7 @@
           <t>An insured party role that inheres in a person who participates in the creation of the insurance contract and is eligible to receive benefits as specified by the insurance contract.</t>
         </is>
       </c>
-      <c r="D183" t="inlineStr">
+      <c r="E183" t="inlineStr">
         <is>
           <t>insured party role</t>
         </is>
@@ -10575,16 +10619,16 @@
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="E184" s="2" t="n"/>
-      <c r="F184" s="2" t="inlineStr">
-        <is>
           <t>Percentage of highly educated individuals in a population. 
 Mean age in a population.</t>
         </is>
       </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="n"/>
       <c r="G184" s="2" t="n"/>
       <c r="H184" s="2" t="n"/>
       <c r="I184" s="2" t="n"/>
@@ -10621,12 +10665,12 @@
           <t>A student or trainee role realised by  currently learning at an initial level of organised instruction, primarily to familiarise the bearer to the school-type environment.</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
+      <c r="D185" s="2" t="n"/>
+      <c r="E185" s="2" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E185" s="2" t="n"/>
       <c r="F185" s="2" t="n"/>
       <c r="G185" s="2" t="n"/>
       <c r="H185" s="2" t="n"/>
@@ -10676,12 +10720,12 @@
           <t>A &lt;disposition&gt; that decreases the likelihood of engaging with harmful behaviour.</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
+      <c r="D186" s="2" t="n"/>
+      <c r="E186" s="2" t="inlineStr">
         <is>
           <t>disposition</t>
         </is>
       </c>
-      <c r="E186" s="2" t="n"/>
       <c r="F186" s="2" t="n"/>
       <c r="G186" s="2" t="n"/>
       <c r="H186" s="2" t="n"/>
@@ -10731,7 +10775,7 @@
           <t>A specifically dependent continuant that, in contrast to roles and dispositions, does not require any further process in order to be realized.</t>
         </is>
       </c>
-      <c r="D187" t="inlineStr">
+      <c r="E187" t="inlineStr">
         <is>
           <t>specifically dependent continuant</t>
         </is>
@@ -10765,15 +10809,15 @@
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
+          <t>12 acres, a flock of 20 goats</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E188" s="2" t="n"/>
-      <c r="F188" s="2" t="inlineStr">
-        <is>
-          <t>12 acres, a flock of 20 goats</t>
-        </is>
-      </c>
+      <c r="F188" s="2" t="n"/>
       <c r="G188" s="2" t="n"/>
       <c r="H188" s="2" t="n"/>
       <c r="I188" s="2" t="n"/>
@@ -10826,12 +10870,12 @@
           <t>A sexual orientation that is not exclusively homosexual or heterosexual, or of a person who does not identify with heterosexual, homosexual or bisexual labels.</t>
         </is>
       </c>
-      <c r="D189" s="2" t="inlineStr">
+      <c r="D189" s="2" t="n"/>
+      <c r="E189" s="2" t="inlineStr">
         <is>
           <t>sexual orientation</t>
         </is>
       </c>
-      <c r="E189" s="2" t="n"/>
       <c r="F189" s="2" t="n"/>
       <c r="G189" s="2" t="inlineStr">
         <is>
@@ -10885,12 +10929,12 @@
           <t xml:space="preserve">A self-identity as being in the process of exploring one's sexual orientation. </t>
         </is>
       </c>
-      <c r="D190" s="2" t="inlineStr">
+      <c r="D190" s="2" t="n"/>
+      <c r="E190" s="2" t="inlineStr">
         <is>
           <t>self-identity</t>
         </is>
       </c>
-      <c r="E190" s="2" t="n"/>
       <c r="F190" s="2" t="n"/>
       <c r="G190" s="2" t="inlineStr">
         <is>
@@ -10944,12 +10988,12 @@
           <t>A personal attribute that is whether an individual is connected or associated with another through romantic attraction or marriage.</t>
         </is>
       </c>
-      <c r="D191" s="2" t="inlineStr">
+      <c r="D191" s="2" t="n"/>
+      <c r="E191" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E191" s="2" t="n"/>
       <c r="F191" s="2" t="n"/>
       <c r="G191" s="2" t="n"/>
       <c r="H191" s="2" t="n"/>
@@ -11001,15 +11045,15 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve"> Religion Baptist 157 (37.0%) 163 (40.3%) Catholic 54 (12.7%) 60 (14.9%) Muslim 39 (9.2%) </t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E192" s="2" t="n"/>
-      <c r="F192" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Religion Baptist 157 (37.0%) 163 (40.3%) Catholic 54 (12.7%) 60 (14.9%) Muslim 39 (9.2%) </t>
-        </is>
-      </c>
+      <c r="F192" s="2" t="n"/>
       <c r="G192" s="2" t="inlineStr">
         <is>
           <t>NCIT_C103282</t>
@@ -11066,12 +11110,12 @@
           <t>A person who lives in a residential facility they do not own without paying an agreed sum of money to the residential facility owner.</t>
         </is>
       </c>
-      <c r="D193" s="2" t="inlineStr">
+      <c r="D193" s="2" t="n"/>
+      <c r="E193" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E193" s="2" t="n"/>
       <c r="F193" s="2" t="n"/>
       <c r="G193" s="2" t="n"/>
       <c r="H193" s="2" t="n"/>
@@ -11123,15 +11167,15 @@
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
+          <t>squatters</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
           <t>rent-free occupier</t>
         </is>
       </c>
-      <c r="E194" s="2" t="n"/>
-      <c r="F194" s="2" t="inlineStr">
-        <is>
-          <t>squatters</t>
-        </is>
-      </c>
+      <c r="F194" s="2" t="n"/>
       <c r="G194" s="2" t="n"/>
       <c r="H194" s="2" t="n"/>
       <c r="I194" s="2" t="n"/>
@@ -11180,12 +11224,12 @@
           <t>A person who lives in a residential facility they do not own in return for paying an agreed sum of money to the residential facility owner</t>
         </is>
       </c>
-      <c r="D195" s="2" t="inlineStr">
+      <c r="D195" s="2" t="n"/>
+      <c r="E195" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E195" s="2" t="n"/>
       <c r="F195" s="2" t="n"/>
       <c r="G195" s="2" t="n"/>
       <c r="H195" s="2" t="n"/>
@@ -11237,15 +11281,15 @@
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
+          <t>renters living in "public housing"[US], council housing [UK], housing association properties, non-profit organisation, alms house occupier</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
           <t>renter</t>
         </is>
       </c>
-      <c r="E196" s="2" t="n"/>
-      <c r="F196" s="2" t="inlineStr">
-        <is>
-          <t>renters living in "public housing"[US], council housing [UK], housing association properties, non-profit organisation, alms house occupier</t>
-        </is>
-      </c>
+      <c r="F196" s="2" t="n"/>
       <c r="G196" s="2" t="n"/>
       <c r="H196" s="2" t="n"/>
       <c r="I196" s="2" t="n"/>
@@ -11294,12 +11338,12 @@
           <t>An owner of a residential facility.</t>
         </is>
       </c>
-      <c r="D197" s="2" t="inlineStr">
+      <c r="D197" s="2" t="n"/>
+      <c r="E197" s="2" t="inlineStr">
         <is>
           <t>owner</t>
         </is>
       </c>
-      <c r="E197" s="2" t="n"/>
       <c r="F197" s="2" t="n"/>
       <c r="G197" s="2" t="n"/>
       <c r="H197" s="2" t="n"/>
@@ -11349,12 +11393,12 @@
           <t>A personal attribute inhering in a person who previously bore a role realised in an employment process but has withdrawn from that employment process, having concluded their working or professional career.</t>
         </is>
       </c>
-      <c r="D198" s="2" t="inlineStr">
+      <c r="D198" s="2" t="n"/>
+      <c r="E198" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E198" s="2" t="n"/>
       <c r="F198" s="2" t="n"/>
       <c r="G198" s="2" t="n"/>
       <c r="H198" s="2" t="n"/>
@@ -11404,7 +11448,7 @@
           <t>b is a role means: b is a realizable entity and b exists because there is some single bearer that is in some special physical, social, or institutional set of circumstances in which this bearer does not have to beand b is not such that, if it ceases to exist, then the physical make-up of the bearer is thereby changed.</t>
         </is>
       </c>
-      <c r="D199" t="inlineStr">
+      <c r="E199" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
@@ -11436,12 +11480,12 @@
           <t xml:space="preserve">A student or trainee role realised by currently learning at a primary or secondary education level in an institutional, organised setting. </t>
         </is>
       </c>
-      <c r="D200" s="3" t="inlineStr">
+      <c r="D200" s="3" t="n"/>
+      <c r="E200" s="3" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E200" s="3" t="n"/>
       <c r="F200" s="3" t="n"/>
       <c r="G200" s="3" t="n"/>
       <c r="H200" s="3" t="n"/>
@@ -11491,12 +11535,12 @@
           <t xml:space="preserve">A student or trainee role realised by currently learning at a primary or secondary education level in an institutional, organised setting. </t>
         </is>
       </c>
-      <c r="D201" s="2" t="inlineStr">
+      <c r="D201" s="2" t="n"/>
+      <c r="E201" s="2" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E201" s="2" t="n"/>
       <c r="F201" s="2" t="n"/>
       <c r="G201" s="2" t="n"/>
       <c r="H201" s="2" t="n"/>
@@ -11546,12 +11590,12 @@
           <t>A person who has at least one parent who is an immigrant.</t>
         </is>
       </c>
-      <c r="D202" s="2" t="inlineStr">
+      <c r="D202" s="2" t="n"/>
+      <c r="E202" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E202" s="2" t="n"/>
       <c r="F202" s="2" t="n"/>
       <c r="G202" s="2" t="n"/>
       <c r="H202" s="2" t="n"/>
@@ -11601,12 +11645,12 @@
           <t>An employment status realised by a person earning income directly from customers, clients, or other organisations rather than as a specified salary or wages from an employer.</t>
         </is>
       </c>
-      <c r="D203" s="2" t="inlineStr">
+      <c r="D203" s="2" t="n"/>
+      <c r="E203" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E203" s="2" t="n"/>
       <c r="F203" s="2" t="n"/>
       <c r="G203" s="2" t="inlineStr">
         <is>
@@ -11664,7 +11708,7 @@
           <t>An identity that a person has about themselves.</t>
         </is>
       </c>
-      <c r="D204" t="inlineStr">
+      <c r="E204" t="inlineStr">
         <is>
           <t>identity</t>
         </is>
@@ -11696,12 +11740,12 @@
           <t xml:space="preserve">A personal attribute that is the pattern of a person's emotional, romantic and/or sexual attractions. </t>
         </is>
       </c>
-      <c r="D205" s="2" t="inlineStr">
+      <c r="D205" s="2" t="n"/>
+      <c r="E205" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E205" s="2" t="n"/>
       <c r="F205" s="2" t="n"/>
       <c r="G205" s="2" t="inlineStr">
         <is>
@@ -11755,12 +11799,12 @@
           <t>A family member with whom the subject shares a parent.</t>
         </is>
       </c>
-      <c r="D206" s="2" t="inlineStr">
+      <c r="D206" s="2" t="n"/>
+      <c r="E206" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E206" s="2" t="n"/>
       <c r="F206" s="2" t="n"/>
       <c r="G206" s="2" t="n"/>
       <c r="H206" s="2" t="n"/>
@@ -11811,12 +11855,12 @@
           <t>A relationship status where the individual is not in a relationship with another person.</t>
         </is>
       </c>
-      <c r="D207" s="2" t="inlineStr">
+      <c r="D207" s="2" t="n"/>
+      <c r="E207" s="2" t="inlineStr">
         <is>
           <t>relationship status</t>
         </is>
       </c>
-      <c r="E207" s="2" t="n"/>
       <c r="F207" s="2" t="n"/>
       <c r="G207" s="2" t="n"/>
       <c r="H207" s="2" t="n"/>
@@ -11866,12 +11910,12 @@
           <t>A personal attribute that holds within a given situation.</t>
         </is>
       </c>
-      <c r="D208" s="2" t="inlineStr">
+      <c r="D208" s="2" t="n"/>
+      <c r="E208" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E208" s="2" t="n"/>
       <c r="F208" s="2" t="n"/>
       <c r="G208" s="2" t="n"/>
       <c r="H208" s="2" t="n"/>
@@ -11913,12 +11957,12 @@
           <t>A social grouping that identifies as such and sometimes acts collectively.</t>
         </is>
       </c>
-      <c r="D209" s="2" t="inlineStr">
+      <c r="D209" s="2" t="n"/>
+      <c r="E209" s="2" t="inlineStr">
         <is>
           <t>social grouping</t>
         </is>
       </c>
-      <c r="E209" s="2" t="n"/>
       <c r="F209" s="2" t="n"/>
       <c r="G209" s="2" t="n"/>
       <c r="H209" s="2" t="n"/>
@@ -11960,12 +12004,12 @@
           <t>A human population who share some common attribute that involves some form of social interaction.</t>
         </is>
       </c>
-      <c r="D210" s="2" t="inlineStr">
+      <c r="D210" s="2" t="n"/>
+      <c r="E210" s="2" t="inlineStr">
         <is>
           <t>human population</t>
         </is>
       </c>
-      <c r="E210" s="2" t="n"/>
       <c r="F210" s="2" t="n"/>
       <c r="G210" s="2" t="n"/>
       <c r="H210" s="2" t="n"/>
@@ -12011,12 +12055,12 @@
           <t>A personal role that is realised in human social processes.</t>
         </is>
       </c>
-      <c r="D211" s="2" t="inlineStr">
+      <c r="D211" s="2" t="n"/>
+      <c r="E211" s="2" t="inlineStr">
         <is>
           <t>personal role</t>
         </is>
       </c>
-      <c r="E211" s="2" t="n"/>
       <c r="F211" s="2" t="n"/>
       <c r="G211" s="2" t="n"/>
       <c r="H211" s="2" t="n"/>
@@ -12058,12 +12102,12 @@
           <t>A &lt;personal attribute&gt; that, together with other attributes, characterises a person’s position in society.</t>
         </is>
       </c>
-      <c r="D212" s="2" t="inlineStr">
+      <c r="D212" s="2" t="n"/>
+      <c r="E212" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E212" s="2" t="n"/>
       <c r="F212" s="2" t="n"/>
       <c r="G212" s="2" t="n"/>
       <c r="H212" s="2" t="n"/>
@@ -12109,7 +12153,7 @@
           <t xml:space="preserve">A personal attribute reflecting a person's economic and social position in relation to others, based on their income, education, or occupation.  </t>
         </is>
       </c>
-      <c r="D213" t="inlineStr">
+      <c r="E213" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
@@ -12143,15 +12187,15 @@
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
+          <t>Semi-routine and routine occupations, blue collar occupations</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E214" s="2" t="n"/>
-      <c r="F214" s="2" t="inlineStr">
-        <is>
-          <t>Semi-routine and routine occupations, blue collar occupations</t>
-        </is>
-      </c>
+      <c r="F214" s="2" t="n"/>
       <c r="G214" s="2" t="n"/>
       <c r="H214" s="2" t="n"/>
       <c r="I214" s="2" t="n"/>
@@ -12204,12 +12248,12 @@
           <t xml:space="preserve">A data item about a score on a measure of a person's socioeconomic status, calculated by combining information about the number of years of education completed, their individual or household income, their current occupation or the industry in which they work or family size or household. </t>
         </is>
       </c>
-      <c r="D215" s="2" t="inlineStr">
+      <c r="D215" s="2" t="n"/>
+      <c r="E215" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E215" s="2" t="n"/>
       <c r="F215" s="2" t="n"/>
       <c r="G215" s="2" t="n"/>
       <c r="H215" s="2" t="n"/>
@@ -12263,12 +12307,12 @@
           <t>A personal attribute inhering in a person by virtue of that person not bearing a role realised in an employment process, due to being a homemaker whose work includes caring for children.</t>
         </is>
       </c>
-      <c r="D216" s="2" t="inlineStr">
+      <c r="D216" s="2" t="n"/>
+      <c r="E216" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E216" s="2" t="n"/>
       <c r="F216" s="2" t="n"/>
       <c r="G216" s="2" t="inlineStr">
         <is>
@@ -12322,12 +12366,12 @@
           <t>A parent in a parent-child relationship established by the parent's subsequent marriage to one of the child's original biological or legal parents.</t>
         </is>
       </c>
-      <c r="D217" s="2" t="inlineStr">
+      <c r="D217" s="2" t="n"/>
+      <c r="E217" s="2" t="inlineStr">
         <is>
           <t>parent</t>
         </is>
       </c>
-      <c r="E217" s="2" t="n"/>
       <c r="F217" s="2" t="n"/>
       <c r="G217" s="2" t="inlineStr">
         <is>
@@ -12381,12 +12425,12 @@
           <t>A sibling who is the child of one's step-parent.</t>
         </is>
       </c>
-      <c r="D218" s="2" t="inlineStr">
+      <c r="D218" s="2" t="n"/>
+      <c r="E218" s="2" t="inlineStr">
         <is>
           <t>sibling</t>
         </is>
       </c>
-      <c r="E218" s="2" t="n"/>
       <c r="F218" s="2" t="n"/>
       <c r="G218" s="2" t="n"/>
       <c r="H218" s="2" t="n"/>
@@ -12436,12 +12480,12 @@
           <t>A step-sibling who is male gender.</t>
         </is>
       </c>
-      <c r="D219" s="2" t="inlineStr">
+      <c r="D219" s="2" t="n"/>
+      <c r="E219" s="2" t="inlineStr">
         <is>
           <t>step-sibling</t>
         </is>
       </c>
-      <c r="E219" s="2" t="n"/>
       <c r="F219" s="2" t="n"/>
       <c r="G219" s="2" t="n"/>
       <c r="H219" s="2" t="n"/>
@@ -12491,12 +12535,12 @@
           <t>A child relation in a parent-child relationship established by the parent's subsequent marriage to one of the child's original biological or legal parents.</t>
         </is>
       </c>
-      <c r="D220" s="2" t="inlineStr">
+      <c r="D220" s="2" t="n"/>
+      <c r="E220" s="2" t="inlineStr">
         <is>
           <t>child relation</t>
         </is>
       </c>
-      <c r="E220" s="2" t="n"/>
       <c r="F220" s="2" t="n"/>
       <c r="G220" s="2" t="n"/>
       <c r="H220" s="2" t="n"/>
@@ -12546,12 +12590,12 @@
           <t>A stepchild who is female gender.</t>
         </is>
       </c>
-      <c r="D221" s="2" t="inlineStr">
+      <c r="D221" s="2" t="n"/>
+      <c r="E221" s="2" t="inlineStr">
         <is>
           <t>stepchild</t>
         </is>
       </c>
-      <c r="E221" s="2" t="n"/>
       <c r="F221" s="2" t="n"/>
       <c r="G221" s="2" t="n"/>
       <c r="H221" s="2" t="n"/>
@@ -12601,12 +12645,12 @@
           <t>A step-parent who is male gender.</t>
         </is>
       </c>
-      <c r="D222" s="2" t="inlineStr">
+      <c r="D222" s="2" t="n"/>
+      <c r="E222" s="2" t="inlineStr">
         <is>
           <t>step-parent</t>
         </is>
       </c>
-      <c r="E222" s="2" t="n"/>
       <c r="F222" s="2" t="n"/>
       <c r="G222" s="2" t="n"/>
       <c r="H222" s="2" t="n"/>
@@ -12656,12 +12700,12 @@
           <t>A step-parent who is female gender.</t>
         </is>
       </c>
-      <c r="D223" s="2" t="inlineStr">
+      <c r="D223" s="2" t="n"/>
+      <c r="E223" s="2" t="inlineStr">
         <is>
           <t>step-parent</t>
         </is>
       </c>
-      <c r="E223" s="2" t="n"/>
       <c r="F223" s="2" t="n"/>
       <c r="G223" s="2" t="n"/>
       <c r="H223" s="2" t="n"/>
@@ -12711,12 +12755,12 @@
           <t>A step-sibling who is female gender.</t>
         </is>
       </c>
-      <c r="D224" s="2" t="inlineStr">
+      <c r="D224" s="2" t="n"/>
+      <c r="E224" s="2" t="inlineStr">
         <is>
           <t>step-sibling</t>
         </is>
       </c>
-      <c r="E224" s="2" t="n"/>
       <c r="F224" s="2" t="n"/>
       <c r="G224" s="2" t="n"/>
       <c r="H224" s="2" t="n"/>
@@ -12766,12 +12810,12 @@
           <t>A stepchild who is male gender.</t>
         </is>
       </c>
-      <c r="D225" s="2" t="inlineStr">
+      <c r="D225" s="2" t="n"/>
+      <c r="E225" s="2" t="inlineStr">
         <is>
           <t>stepchild</t>
         </is>
       </c>
-      <c r="E225" s="2" t="n"/>
       <c r="F225" s="2" t="n"/>
       <c r="G225" s="2" t="n"/>
       <c r="H225" s="2" t="n"/>
@@ -12821,12 +12865,12 @@
           <t>A role which inheres in a person and is realised by being enrolled in an educational institution or a formal programme of professional training.</t>
         </is>
       </c>
-      <c r="D226" s="2" t="inlineStr">
+      <c r="D226" s="2" t="n"/>
+      <c r="E226" s="2" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="E226" s="2" t="n"/>
       <c r="F226" s="2" t="n"/>
       <c r="G226" s="2" t="n"/>
       <c r="H226" s="2" t="n"/>
@@ -12876,7 +12920,7 @@
           <t>A person between 13 and 19 years of age.</t>
         </is>
       </c>
-      <c r="D227" t="inlineStr">
+      <c r="E227" t="inlineStr">
         <is>
           <t>person</t>
         </is>
@@ -12918,12 +12962,12 @@
           <t>A gender identity that differs from the person's assigned sex at birth.</t>
         </is>
       </c>
-      <c r="D228" s="2" t="inlineStr">
+      <c r="D228" s="2" t="n"/>
+      <c r="E228" s="2" t="inlineStr">
         <is>
           <t>gender identity</t>
         </is>
       </c>
-      <c r="E228" s="2" t="n"/>
       <c r="F228" s="2" t="n"/>
       <c r="G228" s="2" t="inlineStr">
         <is>
@@ -12977,12 +13021,12 @@
           <t xml:space="preserve">One of two siblings who resulted from the same pregnancy. </t>
         </is>
       </c>
-      <c r="D229" s="2" t="inlineStr">
+      <c r="D229" s="2" t="n"/>
+      <c r="E229" s="2" t="inlineStr">
         <is>
           <t>sibling</t>
         </is>
       </c>
-      <c r="E229" s="2" t="n"/>
       <c r="F229" s="2" t="n"/>
       <c r="G229" s="2" t="n"/>
       <c r="H229" s="2" t="n"/>
@@ -13032,12 +13076,12 @@
           <t>A situational personal attribute in which a person has not thought about enacting a behaviour.</t>
         </is>
       </c>
-      <c r="D230" s="2" t="inlineStr">
+      <c r="D230" s="2" t="n"/>
+      <c r="E230" s="2" t="inlineStr">
         <is>
           <t>situational personal attribute</t>
         </is>
       </c>
-      <c r="E230" s="2" t="n"/>
       <c r="F230" s="2" t="n"/>
       <c r="G230" s="2" t="n"/>
       <c r="H230" s="2" t="n"/>
@@ -13087,12 +13131,12 @@
           <t>A family member who is the brother of one's parent.</t>
         </is>
       </c>
-      <c r="D231" s="2" t="inlineStr">
+      <c r="D231" s="2" t="n"/>
+      <c r="E231" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E231" s="2" t="n"/>
       <c r="F231" s="2" t="n"/>
       <c r="G231" s="2" t="n"/>
       <c r="H231" s="2" t="n"/>
@@ -13142,12 +13186,12 @@
           <t>A situational personal attribute in which the person has thought about a behaviour but not formed an intention regarding whether to enact it.</t>
         </is>
       </c>
-      <c r="D232" s="2" t="inlineStr">
+      <c r="D232" s="2" t="n"/>
+      <c r="E232" s="2" t="inlineStr">
         <is>
           <t>situational personal attribute</t>
         </is>
       </c>
-      <c r="E232" s="2" t="n"/>
       <c r="F232" s="2" t="n"/>
       <c r="G232" s="2" t="n"/>
       <c r="H232" s="2" t="n"/>
@@ -13197,12 +13241,12 @@
           <t>A higher education student role realised by currently studying for an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D233" s="3" t="inlineStr">
+      <c r="D233" s="3" t="n"/>
+      <c r="E233" s="3" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E233" s="3" t="n"/>
       <c r="F233" s="3" t="n"/>
       <c r="G233" s="3" t="n"/>
       <c r="H233" s="3" t="n"/>
@@ -13252,12 +13296,12 @@
           <t>A higher education student role realised by currently studying for an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D234" s="2" t="inlineStr">
+      <c r="D234" s="2" t="n"/>
+      <c r="E234" s="2" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E234" s="2" t="n"/>
       <c r="F234" s="2" t="n"/>
       <c r="G234" s="2" t="n"/>
       <c r="H234" s="2" t="n"/>
@@ -13307,12 +13351,12 @@
           <t>An employment status in which the person is not employed or self-employed, is looking for work and able to start in paid employment.</t>
         </is>
       </c>
-      <c r="D235" s="2" t="inlineStr">
+      <c r="D235" s="2" t="n"/>
+      <c r="E235" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E235" s="2" t="n"/>
       <c r="F235" s="2" t="n"/>
       <c r="G235" s="2" t="inlineStr">
         <is>
@@ -13366,12 +13410,12 @@
           <t>A personal attribute inhering in a person by virtue of that person not bearing a role realised in an employment process, due to their primary occupation being caring, without receiving a wage for it, for an adult friend or family member who, due to illness or disability, requires support in their daily life activities.</t>
         </is>
       </c>
-      <c r="D236" s="2" t="inlineStr">
+      <c r="D236" s="2" t="n"/>
+      <c r="E236" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E236" s="2" t="n"/>
       <c r="F236" s="2" t="n"/>
       <c r="G236" s="2" t="n"/>
       <c r="H236" s="2" t="n"/>
@@ -13423,15 +13467,15 @@
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
+          <t>farmland, jewellery, livestock</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="inlineStr">
+        <is>
           <t>object aggregate</t>
         </is>
       </c>
-      <c r="E237" s="2" t="n"/>
-      <c r="F237" s="2" t="inlineStr">
-        <is>
-          <t>farmland, jewellery, livestock</t>
-        </is>
-      </c>
+      <c r="F237" s="2" t="n"/>
       <c r="G237" s="2" t="inlineStr">
         <is>
           <t>SDGIO:00010048</t>
@@ -13478,15 +13522,15 @@
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
+          <t>$400, 3000 euros</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E238" s="2" t="n"/>
-      <c r="F238" s="2" t="inlineStr">
-        <is>
-          <t>$400, 3000 euros</t>
-        </is>
-      </c>
+      <c r="F238" s="2" t="n"/>
       <c r="G238" s="2" t="n"/>
       <c r="H238" s="2" t="n"/>
       <c r="I238" s="2" t="n"/>
@@ -13539,12 +13583,12 @@
           <t>A student or trainee role realised by currently learning the curriculum material of vocational programme, normally in preparation for employment in a trade, job or profession.</t>
         </is>
       </c>
-      <c r="D239" s="3" t="inlineStr">
+      <c r="D239" s="3" t="n"/>
+      <c r="E239" s="3" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E239" s="3" t="n"/>
       <c r="F239" s="3" t="n"/>
       <c r="G239" s="3" t="n"/>
       <c r="H239" s="3" t="n"/>
@@ -13594,12 +13638,12 @@
           <t>A student or trainee role that is currently learning the curriculum material of vocational programme, normally in preparation for employment in a trade, job or profession.</t>
         </is>
       </c>
-      <c r="D240" s="2" t="inlineStr">
+      <c r="D240" s="2" t="n"/>
+      <c r="E240" s="2" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E240" s="2" t="n"/>
       <c r="F240" s="2" t="n"/>
       <c r="G240" s="2" t="n"/>
       <c r="H240" s="2" t="n"/>
@@ -13649,12 +13693,12 @@
           <t>A personal attribute inhering in a person by virtue of that person working or assisting at a workplace without receiving remuneration.</t>
         </is>
       </c>
-      <c r="D241" s="2" t="inlineStr">
+      <c r="D241" s="2" t="n"/>
+      <c r="E241" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E241" s="2" t="n"/>
       <c r="F241" s="2" t="n"/>
       <c r="G241" s="2" t="n"/>
       <c r="H241" s="2" t="n"/>
@@ -13708,12 +13752,12 @@
           <t xml:space="preserve">A relationship status where the individual is no longer in a legally formalised marriage or civil partnership due to the death of their spouse or partner. </t>
         </is>
       </c>
-      <c r="D242" s="2" t="inlineStr">
+      <c r="D242" s="2" t="n"/>
+      <c r="E242" s="2" t="inlineStr">
         <is>
           <t>relationship status</t>
         </is>
       </c>
-      <c r="E242" s="2" t="n"/>
       <c r="F242" s="2" t="n"/>
       <c r="G242" s="2" t="n"/>
       <c r="H242" s="2" t="n"/>

</xml_diff>

<commit_message>
Update Curation status of socioeconomic position in BCIO_Population.xlsx
</commit_message>
<xml_diff>
--- a/Population/BCIO_Population.xlsx
+++ b/Population/BCIO_Population.xlsx
@@ -49,7 +49,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ffffff"/>
+        <fgColor rgb="00ffe4b5"/>
       </patternFill>
     </fill>
   </fills>
@@ -12191,7 +12191,7 @@
       </c>
       <c r="R213" s="4" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Discussed</t>
         </is>
       </c>
       <c r="S213" s="4" t="n"/>

</xml_diff>

<commit_message>
Update Kind of socioeconomic position in BCIO_Population.xlsx
</commit_message>
<xml_diff>
--- a/Population/BCIO_Population.xlsx
+++ b/Population/BCIO_Population.xlsx
@@ -451,32 +451,32 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Informal definition</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Logical definition</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Parent</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Logical definition</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Cross-reference</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Synonyms</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Examples</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Cross-reference</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Synonyms</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Informal definition</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -556,20 +556,20 @@
           <t>A linguistic capability that is realised by following and understanding speech in the intervention language.</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">linguistic capability </t>
-        </is>
-      </c>
+      <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Comprehend the German language</t>
+          <t xml:space="preserve">linguistic capability </t>
         </is>
       </c>
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Comprehend the German language</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -615,20 +615,20 @@
           <t>A linguistic capability that is realised by reading and understanding text in the intervention language.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">linguistic capability </t>
-        </is>
-      </c>
+      <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>The exclusion criteria were an inability to read English</t>
+          <t xml:space="preserve">linguistic capability </t>
         </is>
       </c>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>The exclusion criteria were an inability to read English</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -674,20 +674,20 @@
           <t xml:space="preserve">A linguistic capability that is realised by producing speech  in the intervention language. </t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">linguistic capability </t>
-        </is>
-      </c>
+      <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Able to speak Chinese.</t>
+          <t xml:space="preserve">linguistic capability </t>
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Able to speak Chinese.</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -733,20 +733,20 @@
           <t>A linguistic capability that is realised by generating written text in the intervention language.</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">linguistic capability </t>
-        </is>
-      </c>
+      <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Fluency in written English.</t>
+          <t xml:space="preserve">linguistic capability </t>
         </is>
       </c>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="n"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Fluency in written English.</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="inlineStr">
         <is>
@@ -792,13 +792,13 @@
           <t>A highest level of formal education qualification achieved after participating in an education process intended to result in the acquisition and development of skills and knowledge in a specialised discipline that culminated in the award of an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>highest level of formal educational qualification achieved</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>OMRSE_00002048</t>
@@ -855,13 +855,13 @@
           <t xml:space="preserve">A highest level of formal educational qualification achieved after participating in an education process devoted to advanced study and original research that led to the award of a PhD or equivalent level qualification. </t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>highest level of formal educational qualification achieved</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="n"/>
@@ -914,13 +914,13 @@
           <t xml:space="preserve">A highest level of formal educational qualification achieved after participating in an education process intended to introduce very young children to a school-type environment. </t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>highest level of formal educational qualification achieved</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
@@ -973,13 +973,13 @@
           <t>A highest level of formal educational qualification achieved after participating in an education process intended to result in the acquisition and development of skills and knowledge in subject areas more specialised than basic reading, writing and mathematics, with the overall goal of laying the foundation for lifelong learning and human development on which education systems may systematically expand further educational opportunities.</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>highest level of formal educational qualification achieved</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
           <t>OMRSE_00002036</t>
@@ -1036,13 +1036,13 @@
           <t>A highest level of formal educational qualification achieved after participating in an education process which has as a prerequisite an undergraduate degree and which is intended to result in the acquisition and development of advanced academic or professional skills and knowledge in a specialised discipline, that culminated in the award of a Master's or equivalent degree.</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>highest level of formal educational qualification achieved</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
@@ -1095,13 +1095,13 @@
           <t>A highest level of formal educational qualification achieved after participating in an education process intended to result in the acquisition of fundamental skills in reading, writing and mathematics.</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>highest level of formal educational qualification achieved</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">OMRSE_00002035  </t>
@@ -1158,24 +1158,24 @@
           <t>A highest level of formal educational qualification achieved after participating in an education process intended to result in the acquisition and development of skills and knowledge that prepare participants for tertiary education or employment.</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>highest level of formal educational qualification achieved</t>
-        </is>
-      </c>
+      <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
+          <t>highest level of formal educational qualification achieved</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>OMRSE_00002040</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
           <t>graduated high school, International Baccaulaureate, A Levels</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>OMRSE_00002040</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
           <t>A highest level of formal educational qualification achieved that corresponds to the final stage of secondary education in most OECD countries. Instruction is often more organised along subject-matter lines than at ISCED 2 level and teachers typically need to have a higher level, or more subject-specific, qualifications than at ISCED 2. The entrance age to this level is typically 15 or 16 years. There are substantial differences in the typical duration of ISCED 3 programmes both between and within countries, typically ranging from 2 to 5 years of schooling. ISCED 3 may either be “terminal” (i.e. preparing students for direct entry into working life) and/or “preparatory” (i.e. preparing students for tertiary education).</t>
@@ -1225,13 +1225,13 @@
           <t>An adoptive sibling who is male gender.</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>adoptive sibling</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="n"/>
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="n"/>
@@ -1280,13 +1280,13 @@
           <t xml:space="preserve">A child relation in a parent-child relationship established by a legal adoption process. </t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>child relation</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>NCIT:C166130</t>
@@ -1339,13 +1339,13 @@
           <t>An adoptive child who is female gender.</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>adoptive child</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="n"/>
@@ -1394,13 +1394,13 @@
           <t>An adoptive parent who is male gender.</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>adoptive parent</t>
         </is>
       </c>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
@@ -1449,13 +1449,13 @@
           <t>An adoptive parent who is female gender.</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>adoptive parent</t>
         </is>
       </c>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="n"/>
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="n"/>
@@ -1504,13 +1504,13 @@
           <t>A parent in a parent-child relationship established by a legal adoption process.</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>parent</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>NCIT:C166129</t>
@@ -1563,13 +1563,13 @@
           <t>A sibling with whom the subject shares a parent through a parent-child relationship established by a legal adoption process.</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>sibling</t>
         </is>
       </c>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="n"/>
@@ -1618,13 +1618,13 @@
           <t>An adoptive sibling who is female gender.</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>adoptive sibling</t>
         </is>
       </c>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
       <c r="I20" s="2" t="n"/>
@@ -1673,13 +1673,13 @@
           <t>An adoptive child who is male gender.</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>adoptive child</t>
         </is>
       </c>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="n"/>
       <c r="I21" s="2" t="n"/>
@@ -1728,7 +1728,7 @@
           <t>A person who has reached maturity.</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>person</t>
         </is>
@@ -1775,13 +1775,13 @@
           <t>A rent-free occupier who lives in the residential facility with the agreement of the residential facility owner.</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>rent-free occupier</t>
         </is>
       </c>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
       <c r="H23" s="2" t="n"/>
       <c r="I23" s="2" t="n"/>
@@ -1830,13 +1830,13 @@
           <t xml:space="preserve">A sexual orientation of an individual who does not experience sexual attraction. </t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>sexual orientation</t>
         </is>
       </c>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
           <t>NCIT_C155696</t>
@@ -1889,13 +1889,13 @@
           <t>A family member who is the sister of one's parent.</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="2" t="n"/>
@@ -1944,13 +1944,13 @@
           <t>An intervention participant who is exposed to a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>intervention participant</t>
         </is>
       </c>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="n"/>
@@ -1995,13 +1995,13 @@
           <t>An intervention population who are exposed to a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>intervention population</t>
         </is>
       </c>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="2" t="n"/>
@@ -2042,13 +2042,13 @@
           <t>A data item that is about the rate of individual human behaviour change.</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="n"/>
@@ -2093,13 +2093,13 @@
           <t>A person who has formed an intention to enact a specified behaviour, and has enacted that behaviour.</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -2149,13 +2149,13 @@
           <t>A person who has formed an intention to enact a specified behaviour, but has not acted on this intention.</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="2" t="n"/>
@@ -2201,13 +2201,13 @@
           <t>A person who has not formed an intention to enact a specified behaviour.</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">person </t>
         </is>
       </c>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="n"/>
@@ -2255,18 +2255,18 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
+          <t>The number of times a person performs a behaviour within a specific period.</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="n"/>
       <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>The number of times a person performs a behaviour within a specific period.</t>
-        </is>
-      </c>
+      <c r="I32" s="2" t="n"/>
       <c r="J32" s="2" t="n"/>
       <c r="K32" s="2" t="inlineStr">
         <is>
@@ -2312,13 +2312,13 @@
           <t>A biological sibling who is male gender.</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>biological sibling</t>
         </is>
       </c>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="n"/>
       <c r="H33" s="2" t="n"/>
       <c r="I33" s="2" t="n"/>
@@ -2367,13 +2367,13 @@
           <t>A child relation who is genetically related to their parent.</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>child relation</t>
         </is>
       </c>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="n"/>
       <c r="H34" s="2" t="n"/>
       <c r="I34" s="2" t="n"/>
@@ -2422,13 +2422,13 @@
           <t>A biological child who is female gender.</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>biological child</t>
         </is>
       </c>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="n"/>
       <c r="H35" s="2" t="n"/>
       <c r="I35" s="2" t="n"/>
@@ -2477,13 +2477,13 @@
           <t>A biological parent who provided the sperm.</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>biological parent</t>
         </is>
       </c>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="n"/>
       <c r="H36" s="2" t="n"/>
       <c r="I36" s="2" t="n"/>
@@ -2532,13 +2532,13 @@
           <t>A biological parent who provided an egg.</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>biological parent</t>
         </is>
       </c>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="n"/>
       <c r="H37" s="2" t="n"/>
       <c r="I37" s="2" t="n"/>
@@ -2587,13 +2587,13 @@
           <t>A parent who provided one of the gametes that resulted in one's conception.</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>parent</t>
         </is>
       </c>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
           <t>NCIT:C166114, GSSO:001986</t>
@@ -2646,13 +2646,13 @@
           <t>A bodily quality based on reproductive function or organs.</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>bodily quality</t>
         </is>
       </c>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="n"/>
       <c r="H39" s="2" t="n"/>
       <c r="I39" s="2" t="n"/>
@@ -2701,13 +2701,13 @@
           <t>A sibling with whom the subject shares a biological parent.</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>sibling</t>
         </is>
       </c>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="n"/>
       <c r="H40" s="2" t="n"/>
       <c r="I40" s="2" t="n"/>
@@ -2756,13 +2756,13 @@
           <t>A biological sibling who is female gender.</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>biological sibling</t>
         </is>
       </c>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="n"/>
       <c r="H41" s="2" t="n"/>
       <c r="I41" s="2" t="n"/>
@@ -2811,13 +2811,13 @@
           <t>A biological child who is male gender.</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>biological child</t>
         </is>
       </c>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="n"/>
       <c r="H42" s="2" t="n"/>
       <c r="I42" s="2" t="n"/>
@@ -2866,13 +2866,13 @@
           <t>A sexual orientation of an individual who experiences sexual attraction to members of more than one sex.</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>sexual orientation</t>
         </is>
       </c>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
           <t>NCIT_C84364</t>
@@ -2925,7 +2925,7 @@
           <t>A quality that inheres in some extended organism.</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>quality</t>
         </is>
@@ -2957,13 +2957,13 @@
           <t>A role which inheres in a person and is realised by the person assuming responsibility for the physical and emotional needs of another who has difficulties with self care.</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="n"/>
       <c r="H45" s="2" t="n"/>
       <c r="I45" s="2" t="n"/>
@@ -3012,13 +3012,13 @@
           <t>A personal attribute as belonging to a group within a stratified system of categorisation based on a status conferred at birth based on descent, in which individuals have limited or no mobility due to custom or law.</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="n"/>
       <c r="H46" s="2" t="n"/>
       <c r="I46" s="2" t="n"/>
@@ -3071,13 +3071,13 @@
           <t xml:space="preserve">A person who has not yet reached maturity. </t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="n"/>
       <c r="H47" s="2" t="n"/>
       <c r="I47" s="2" t="n"/>
@@ -3130,13 +3130,13 @@
           <t>A family member who is a person's first generation offspring.</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="n"/>
       <c r="H48" s="2" t="n"/>
       <c r="I48" s="2" t="n"/>
@@ -3185,13 +3185,13 @@
           <t>A gender identity that matches the person's assigned sex at birth.</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>gender identity</t>
         </is>
       </c>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
           <t>GSSO:004240</t>
@@ -3244,13 +3244,13 @@
           <t xml:space="preserve">A geographic location that is the country in which a person was born. </t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>geographic location</t>
         </is>
       </c>
-      <c r="E50" s="2" t="n"/>
-      <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
           <t>GENEPIO_0001094</t>
@@ -3303,13 +3303,13 @@
           <t>A family member who is a child relation of one's aunt or uncle.</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E51" s="2" t="n"/>
-      <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="n"/>
       <c r="H51" s="2" t="n"/>
       <c r="I51" s="2" t="n"/>
@@ -3358,13 +3358,13 @@
           <t>A personal attribute in which the person has impaired physical or mental functioning that has a notable effect on their ability to do typical daily activities.</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D52" s="2" t="n"/>
+      <c r="E52" s="2" t="n"/>
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E52" s="2" t="n"/>
-      <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="n"/>
       <c r="H52" s="2" t="n"/>
       <c r="I52" s="2" t="n"/>
@@ -3413,20 +3413,20 @@
           <t>An expertise discipline of the programme of study currently undertaken by the bearer of a student or trainee role.</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>expertise discipline</t>
-        </is>
-      </c>
+      <c r="D53" s="2" t="n"/>
       <c r="E53" s="2" t="n"/>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>psychology, counselling, public health</t>
+          <t>expertise discipline</t>
         </is>
       </c>
       <c r="G53" s="2" t="n"/>
       <c r="H53" s="2" t="n"/>
-      <c r="I53" s="2" t="n"/>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>psychology, counselling, public health</t>
+        </is>
+      </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
           <t>The division of knowledge and practice into different disciplines or fields is complex and depends on historical, social and structural factors</t>
@@ -3476,20 +3476,20 @@
           <t>An expertise discipline of the highest level of formal educational qualification a person has achieved.</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>expertise discipline</t>
-        </is>
-      </c>
+      <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="n"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Mathematics, English, hairdressing skills, vehicle engineering, nursing, astrophysics, accountancy</t>
+          <t>expertise discipline</t>
         </is>
       </c>
       <c r="G54" s="2" t="n"/>
       <c r="H54" s="2" t="n"/>
-      <c r="I54" s="2" t="n"/>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Mathematics, English, hairdressing skills, vehicle engineering, nursing, astrophysics, accountancy</t>
+        </is>
+      </c>
       <c r="J54" s="2" t="n"/>
       <c r="K54" s="2" t="inlineStr">
         <is>
@@ -3535,13 +3535,13 @@
           <t>A relationship status where the individual was previously in a legally formalised relationship and this relationship has now ended or dissolved.</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D55" s="2" t="n"/>
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>relationship status</t>
         </is>
       </c>
-      <c r="E55" s="2" t="n"/>
-      <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="n"/>
       <c r="H55" s="2" t="n"/>
       <c r="I55" s="2" t="n"/>
@@ -3590,13 +3590,13 @@
           <t>A higher education student  role realised by currently studying for a doctoral degree.</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="D56" s="3" t="n"/>
+      <c r="E56" s="3" t="n"/>
+      <c r="F56" s="3" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E56" s="3" t="n"/>
-      <c r="F56" s="3" t="n"/>
       <c r="G56" s="3" t="n"/>
       <c r="H56" s="3" t="n"/>
       <c r="I56" s="3" t="n"/>
@@ -3645,13 +3645,13 @@
           <t>A higher education student  role realised by currently studying for a doctoral degree.</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E57" s="2" t="n"/>
-      <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="n"/>
       <c r="H57" s="2" t="n"/>
       <c r="I57" s="2" t="n"/>
@@ -3700,13 +3700,13 @@
           <t>A &lt;social group&gt; of two people who interact and influence each other.</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D58" s="2" t="n"/>
+      <c r="E58" s="2" t="n"/>
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>social group</t>
         </is>
       </c>
-      <c r="E58" s="2" t="n"/>
-      <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="n"/>
       <c r="H58" s="2" t="n"/>
       <c r="I58" s="2" t="n"/>
@@ -3747,13 +3747,13 @@
           <t>A planned process wherein knowledge and skills is imparted.</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D59" s="2" t="n"/>
+      <c r="E59" s="2" t="n"/>
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="E59" s="2" t="n"/>
-      <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
           <t>education process in the Sustainable Development Goals Interface Ontology (SDGIO:00010001)</t>
@@ -3798,13 +3798,13 @@
           <t>An employment status realised by an individual being engaged in an activity or service for wages or salary.</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D60" s="2" t="n"/>
+      <c r="E60" s="2" t="n"/>
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E60" s="2" t="n"/>
-      <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
           <t>NCIT_C25172</t>
@@ -3857,13 +3857,13 @@
           <t>An employment status realised by an individual working a standard number of hours defined as full-time by their employer.</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D61" s="2" t="n"/>
+      <c r="E61" s="2" t="n"/>
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E61" s="2" t="n"/>
-      <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
           <t>OPMI:0000123</t>
@@ -3916,13 +3916,13 @@
           <t>An employment status realised by an individual working for recurring periods in which different groups of workers do the same jobs in relay.</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D62" s="2" t="n"/>
+      <c r="E62" s="2" t="n"/>
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E62" s="2" t="n"/>
-      <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="n"/>
       <c r="H62" s="2" t="n"/>
       <c r="I62" s="2" t="n"/>
@@ -3971,13 +3971,13 @@
           <t>An employment status realised by an individual whose working hours involving less than the standard or customary working time.</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D63" s="2" t="n"/>
+      <c r="E63" s="2" t="n"/>
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E63" s="2" t="n"/>
-      <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
           <t>NCIT_C75562</t>
@@ -4030,13 +4030,13 @@
           <t>A quality inhering in a person by virtue of that person bearing a role realised in an employment process.</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="D64" s="2" t="n"/>
+      <c r="E64" s="2" t="n"/>
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>quality</t>
         </is>
       </c>
-      <c r="E64" s="2" t="n"/>
-      <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
           <t>Sustainable Development Goals Interface Ontology (SDGIO:00010029)</t>
@@ -4094,13 +4094,13 @@
           <t>A self-identity as belonging to a social group or groups whose members have a common cultural or ancestral heritage.</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="D65" s="2" t="n"/>
+      <c r="E65" s="2" t="n"/>
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>self-identity</t>
         </is>
       </c>
-      <c r="E65" s="2" t="n"/>
-      <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
           <t>EFO:0001799</t>
@@ -4157,13 +4157,13 @@
           <t>An attribute that is a field of knowledge or practice.</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D66" s="2" t="n"/>
+      <c r="E66" s="2" t="n"/>
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>specifically dependent continuant</t>
         </is>
       </c>
-      <c r="E66" s="2" t="n"/>
-      <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="n"/>
       <c r="H66" s="2" t="n"/>
       <c r="I66" s="2" t="n"/>
@@ -4212,13 +4212,13 @@
           <t>A data item that is the extent to which the person’s past behaviour has reached or exceeded a standard.</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="D67" s="2" t="n"/>
+      <c r="E67" s="2" t="n"/>
+      <c r="F67" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E67" s="2" t="n"/>
-      <c r="F67" s="2" t="n"/>
       <c r="G67" s="2" t="n"/>
       <c r="H67" s="2" t="n"/>
       <c r="I67" s="2" t="n"/>
@@ -4267,13 +4267,13 @@
           <t>A person who is a member of a group of persons united by blood, or by marriage or other legal arrangement, or by self-identity as belonging to the same family.</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="D68" s="2" t="n"/>
+      <c r="E68" s="2" t="n"/>
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E68" s="2" t="n"/>
-      <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
           <t>NCIT:C41256</t>
@@ -4326,13 +4326,13 @@
           <t>A parent who is male gender.</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="D69" s="2" t="n"/>
+      <c r="E69" s="2" t="n"/>
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>parent</t>
         </is>
       </c>
-      <c r="E69" s="2" t="n"/>
-      <c r="F69" s="2" t="n"/>
       <c r="G69" s="2" t="n"/>
       <c r="H69" s="2" t="n"/>
       <c r="I69" s="2" t="n"/>
@@ -4381,13 +4381,13 @@
           <t>A biological sex associated with the ability to produce female gametes.</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="D70" s="2" t="n"/>
+      <c r="E70" s="2" t="n"/>
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>biological sex</t>
         </is>
       </c>
-      <c r="E70" s="2" t="n"/>
-      <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="n"/>
       <c r="H70" s="2" t="n"/>
       <c r="I70" s="2" t="n"/>
@@ -4436,13 +4436,13 @@
           <t>A gender identity as being female.</t>
         </is>
       </c>
-      <c r="D71" s="2" t="inlineStr">
+      <c r="D71" s="2" t="n"/>
+      <c r="E71" s="2" t="n"/>
+      <c r="F71" s="2" t="inlineStr">
         <is>
           <t>gender identity</t>
         </is>
       </c>
-      <c r="E71" s="2" t="n"/>
-      <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
           <t>GSSO:000089</t>
@@ -4499,13 +4499,13 @@
           <t>A foster sibling who is male gender.</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="D72" s="2" t="n"/>
+      <c r="E72" s="2" t="n"/>
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>foster sibling</t>
         </is>
       </c>
-      <c r="E72" s="2" t="n"/>
-      <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="n"/>
       <c r="H72" s="2" t="n"/>
       <c r="I72" s="2" t="n"/>
@@ -4554,13 +4554,13 @@
           <t xml:space="preserve">A child relation in a parent-child relationship created by a foster care arrangement. </t>
         </is>
       </c>
-      <c r="D73" s="2" t="inlineStr">
+      <c r="D73" s="2" t="n"/>
+      <c r="E73" s="2" t="n"/>
+      <c r="F73" s="2" t="inlineStr">
         <is>
           <t>child relation</t>
         </is>
       </c>
-      <c r="E73" s="2" t="n"/>
-      <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="n"/>
       <c r="H73" s="2" t="n"/>
       <c r="I73" s="2" t="n"/>
@@ -4609,13 +4609,13 @@
           <t>A foster child who is female gender.</t>
         </is>
       </c>
-      <c r="D74" s="2" t="inlineStr">
+      <c r="D74" s="2" t="n"/>
+      <c r="E74" s="2" t="n"/>
+      <c r="F74" s="2" t="inlineStr">
         <is>
           <t>foster child</t>
         </is>
       </c>
-      <c r="E74" s="2" t="n"/>
-      <c r="F74" s="2" t="n"/>
       <c r="G74" s="2" t="n"/>
       <c r="H74" s="2" t="n"/>
       <c r="I74" s="2" t="n"/>
@@ -4664,13 +4664,13 @@
           <t>A foster parent who is male gender.</t>
         </is>
       </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="D75" s="2" t="n"/>
+      <c r="E75" s="2" t="n"/>
+      <c r="F75" s="2" t="inlineStr">
         <is>
           <t>foster parent</t>
         </is>
       </c>
-      <c r="E75" s="2" t="n"/>
-      <c r="F75" s="2" t="n"/>
       <c r="G75" s="2" t="n"/>
       <c r="H75" s="2" t="n"/>
       <c r="I75" s="2" t="n"/>
@@ -4719,13 +4719,13 @@
           <t>A foster parent who is female gender.</t>
         </is>
       </c>
-      <c r="D76" s="2" t="inlineStr">
+      <c r="D76" s="2" t="n"/>
+      <c r="E76" s="2" t="n"/>
+      <c r="F76" s="2" t="inlineStr">
         <is>
           <t>foster parent</t>
         </is>
       </c>
-      <c r="E76" s="2" t="n"/>
-      <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="n"/>
       <c r="H76" s="2" t="n"/>
       <c r="I76" s="2" t="n"/>
@@ -4774,13 +4774,13 @@
           <t>A parent who cares for a child who has been placed with them in a foster care arrangement.</t>
         </is>
       </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="D77" s="2" t="n"/>
+      <c r="E77" s="2" t="n"/>
+      <c r="F77" s="2" t="inlineStr">
         <is>
           <t>parent</t>
         </is>
       </c>
-      <c r="E77" s="2" t="n"/>
-      <c r="F77" s="2" t="n"/>
       <c r="G77" s="2" t="inlineStr">
         <is>
           <t>GSSO:001987</t>
@@ -4833,13 +4833,13 @@
           <t>A sibling who shares a parent through a parent-child relationship created by a foster care agreement.</t>
         </is>
       </c>
-      <c r="D78" s="2" t="inlineStr">
+      <c r="D78" s="2" t="n"/>
+      <c r="E78" s="2" t="n"/>
+      <c r="F78" s="2" t="inlineStr">
         <is>
           <t>sibling</t>
         </is>
       </c>
-      <c r="E78" s="2" t="n"/>
-      <c r="F78" s="2" t="n"/>
       <c r="G78" s="2" t="n"/>
       <c r="H78" s="2" t="n"/>
       <c r="I78" s="2" t="n"/>
@@ -4888,13 +4888,13 @@
           <t>A foster sibling who is female gender.</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
+      <c r="D79" s="2" t="n"/>
+      <c r="E79" s="2" t="n"/>
+      <c r="F79" s="2" t="inlineStr">
         <is>
           <t>foster sibling</t>
         </is>
       </c>
-      <c r="E79" s="2" t="n"/>
-      <c r="F79" s="2" t="n"/>
       <c r="G79" s="2" t="n"/>
       <c r="H79" s="2" t="n"/>
       <c r="I79" s="2" t="n"/>
@@ -4943,13 +4943,13 @@
           <t>A foster child who is male gender.</t>
         </is>
       </c>
-      <c r="D80" s="2" t="inlineStr">
+      <c r="D80" s="2" t="n"/>
+      <c r="E80" s="2" t="n"/>
+      <c r="F80" s="2" t="inlineStr">
         <is>
           <t>foster child</t>
         </is>
       </c>
-      <c r="E80" s="2" t="n"/>
-      <c r="F80" s="2" t="n"/>
       <c r="G80" s="2" t="n"/>
       <c r="H80" s="2" t="n"/>
       <c r="I80" s="2" t="n"/>
@@ -4998,13 +4998,13 @@
           <t>A behavioural frequency about the number of times a person has enacted a behaviour per unit of time.</t>
         </is>
       </c>
-      <c r="D81" s="2" t="inlineStr">
+      <c r="D81" s="2" t="n"/>
+      <c r="E81" s="2" t="n"/>
+      <c r="F81" s="2" t="inlineStr">
         <is>
           <t>behavioural frequency</t>
         </is>
       </c>
-      <c r="E81" s="2" t="n"/>
-      <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="n"/>
       <c r="H81" s="2" t="n"/>
       <c r="I81" s="2" t="n"/>
@@ -5053,13 +5053,13 @@
           <t>A self-identity as having a particular gender, which may or may not correspond with sex assigned at birth.</t>
         </is>
       </c>
-      <c r="D82" s="2" t="inlineStr">
+      <c r="D82" s="2" t="n"/>
+      <c r="E82" s="2" t="n"/>
+      <c r="F82" s="2" t="inlineStr">
         <is>
           <t>self-identity</t>
         </is>
       </c>
-      <c r="E82" s="2" t="n"/>
-      <c r="F82" s="2" t="n"/>
       <c r="G82" s="2" t="n"/>
       <c r="H82" s="2" t="n"/>
       <c r="I82" s="2" t="n"/>
@@ -5108,13 +5108,13 @@
           <t>A higher education student role realised by currently studying for a more advanced degree after completing an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D83" s="3" t="inlineStr">
+      <c r="D83" s="3" t="n"/>
+      <c r="E83" s="3" t="n"/>
+      <c r="F83" s="3" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E83" s="3" t="n"/>
-      <c r="F83" s="3" t="n"/>
       <c r="G83" s="3" t="n"/>
       <c r="H83" s="3" t="n"/>
       <c r="I83" s="3" t="n"/>
@@ -5163,13 +5163,13 @@
           <t>A higher education student role realised by currently studying for a more advanced degree after completing an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D84" s="2" t="inlineStr">
+      <c r="D84" s="2" t="n"/>
+      <c r="E84" s="2" t="n"/>
+      <c r="F84" s="2" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E84" s="2" t="n"/>
-      <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="n"/>
       <c r="H84" s="2" t="n"/>
       <c r="I84" s="2" t="n"/>
@@ -5218,13 +5218,13 @@
           <t>A grandparent who is male gender.</t>
         </is>
       </c>
-      <c r="D85" s="2" t="inlineStr">
+      <c r="D85" s="2" t="n"/>
+      <c r="E85" s="2" t="n"/>
+      <c r="F85" s="2" t="inlineStr">
         <is>
           <t>grandparent</t>
         </is>
       </c>
-      <c r="E85" s="2" t="n"/>
-      <c r="F85" s="2" t="n"/>
       <c r="G85" s="2" t="n"/>
       <c r="H85" s="2" t="n"/>
       <c r="I85" s="2" t="n"/>
@@ -5273,13 +5273,13 @@
           <t>A grandparent who is female gender.</t>
         </is>
       </c>
-      <c r="D86" s="2" t="inlineStr">
+      <c r="D86" s="2" t="n"/>
+      <c r="E86" s="2" t="n"/>
+      <c r="F86" s="2" t="inlineStr">
         <is>
           <t>grandparent</t>
         </is>
       </c>
-      <c r="E86" s="2" t="n"/>
-      <c r="F86" s="2" t="n"/>
       <c r="G86" s="2" t="n"/>
       <c r="H86" s="2" t="n"/>
       <c r="I86" s="2" t="n"/>
@@ -5328,13 +5328,13 @@
           <t>A family member who is the parent of one's parent.</t>
         </is>
       </c>
-      <c r="D87" s="2" t="inlineStr">
+      <c r="D87" s="2" t="n"/>
+      <c r="E87" s="2" t="n"/>
+      <c r="F87" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E87" s="2" t="n"/>
-      <c r="F87" s="2" t="n"/>
       <c r="G87" s="2" t="n"/>
       <c r="H87" s="2" t="n"/>
       <c r="I87" s="2" t="n"/>
@@ -5383,13 +5383,13 @@
           <t xml:space="preserve">A personal history part that includes previously performing a behaviour. </t>
         </is>
       </c>
-      <c r="D88" s="2" t="inlineStr">
+      <c r="D88" s="2" t="n"/>
+      <c r="E88" s="2" t="n"/>
+      <c r="F88" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E88" s="2" t="n"/>
-      <c r="F88" s="2" t="n"/>
       <c r="G88" s="2" t="n"/>
       <c r="H88" s="2" t="n"/>
       <c r="I88" s="2" t="n"/>
@@ -5438,20 +5438,20 @@
           <t>A policy holder role that inheres in a person who participates in the creation of an insurance contract designed to cover some or all of the cost of treating the insured person's illnesses or injuries as well as possibly providing preventive health care.</t>
         </is>
       </c>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t>policy holder role</t>
-        </is>
-      </c>
+      <c r="D89" s="2" t="n"/>
       <c r="E89" s="2" t="n"/>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>having Medicare, Medicaid, Blue Cross, BUPA, being eligible for NHS treatment</t>
+          <t>policy holder role</t>
         </is>
       </c>
       <c r="G89" s="2" t="n"/>
       <c r="H89" s="2" t="n"/>
-      <c r="I89" s="2" t="n"/>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>having Medicare, Medicaid, Blue Cross, BUPA, being eligible for NHS treatment</t>
+        </is>
+      </c>
       <c r="J89" s="2" t="n"/>
       <c r="K89" s="2" t="inlineStr">
         <is>
@@ -5497,24 +5497,24 @@
           <t>A personal attribute that is the state of an individual's mental or physical condition.</t>
         </is>
       </c>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="D90" s="2" t="n"/>
       <c r="E90" s="2" t="n"/>
       <c r="F90" s="2" t="inlineStr">
         <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>NCIT_C16669</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="n"/>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
           <t>Having chicken pox, asthma, a heart attack</t>
         </is>
       </c>
-      <c r="G90" s="2" t="inlineStr">
-        <is>
-          <t>NCIT_C16669</t>
-        </is>
-      </c>
-      <c r="H90" s="2" t="n"/>
-      <c r="I90" s="2" t="n"/>
       <c r="J90" s="2" t="n"/>
       <c r="K90" s="2" t="inlineStr">
         <is>
@@ -5560,13 +5560,13 @@
           <t>A sexual orientation of an individual who experiences sexual attraction exclusively or primarily to members of a different sex.</t>
         </is>
       </c>
-      <c r="D91" s="2" t="inlineStr">
+      <c r="D91" s="2" t="n"/>
+      <c r="E91" s="2" t="n"/>
+      <c r="F91" s="2" t="inlineStr">
         <is>
           <t>sexual orientation</t>
         </is>
       </c>
-      <c r="E91" s="2" t="n"/>
-      <c r="F91" s="2" t="n"/>
       <c r="G91" s="2" t="inlineStr">
         <is>
           <t>NCIT_C84362</t>
@@ -5619,13 +5619,13 @@
           <t>A frequency of past behaviour that is above a threshold.</t>
         </is>
       </c>
-      <c r="D92" s="2" t="inlineStr">
+      <c r="D92" s="2" t="n"/>
+      <c r="E92" s="2" t="n"/>
+      <c r="F92" s="2" t="inlineStr">
         <is>
           <t>frequency of past behaviour</t>
         </is>
       </c>
-      <c r="E92" s="2" t="n"/>
-      <c r="F92" s="2" t="n"/>
       <c r="G92" s="2" t="n"/>
       <c r="H92" s="2" t="n"/>
       <c r="I92" s="2" t="n"/>
@@ -5670,13 +5670,13 @@
           <t xml:space="preserve">A student or trainee role realised by currently learning on an advanced educational programme in a university, college or professional school. For example, completing a university bachelor's or master's course of study, medical school or other professional school. </t>
         </is>
       </c>
-      <c r="D93" s="3" t="inlineStr">
+      <c r="D93" s="3" t="n"/>
+      <c r="E93" s="3" t="n"/>
+      <c r="F93" s="3" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E93" s="3" t="n"/>
-      <c r="F93" s="3" t="n"/>
       <c r="G93" s="3" t="n"/>
       <c r="H93" s="3" t="n"/>
       <c r="I93" s="3" t="n"/>
@@ -5725,20 +5725,20 @@
           <t>A student or trainee role realised by currently learning on an advanced educational programme in a university, college or professional school.</t>
         </is>
       </c>
-      <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>student or trainee role</t>
-        </is>
-      </c>
+      <c r="D94" s="2" t="n"/>
       <c r="E94" s="2" t="n"/>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>completing a university bachelor's or master's course of study, medical school or other professional school.</t>
+          <t>student or trainee role</t>
         </is>
       </c>
       <c r="G94" s="2" t="n"/>
       <c r="H94" s="2" t="n"/>
-      <c r="I94" s="2" t="n"/>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>completing a university bachelor's or master's course of study, medical school or other professional school.</t>
+        </is>
+      </c>
       <c r="J94" s="2" t="n"/>
       <c r="K94" s="2" t="inlineStr">
         <is>
@@ -5784,13 +5784,13 @@
           <t>A personal attribute related to the highest level of education achieved.</t>
         </is>
       </c>
-      <c r="D95" s="2" t="inlineStr">
+      <c r="D95" s="2" t="n"/>
+      <c r="E95" s="2" t="n"/>
+      <c r="F95" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E95" s="2" t="n"/>
-      <c r="F95" s="2" t="n"/>
       <c r="G95" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">NCIT_C17953 </t>
@@ -5847,7 +5847,7 @@
           <t>A process that is the sum of the totality of processes taking place in the spatiotemporal region occupied by a material entity or site, including processes on the surface of the entity or within the cavities to which it serves as host.</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="F96" t="inlineStr">
         <is>
           <t>process</t>
         </is>
@@ -5879,20 +5879,20 @@
           <t>A personal history part that includes exposure to a potentially harmful agent as a result of one's occupation.</t>
         </is>
       </c>
-      <c r="D97" s="2" t="inlineStr">
-        <is>
-          <t>personal history part</t>
-        </is>
-      </c>
+      <c r="D97" s="2" t="n"/>
       <c r="E97" s="2" t="n"/>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>history of exposure to asbestos due to one's job</t>
+          <t>personal history part</t>
         </is>
       </c>
       <c r="G97" s="2" t="n"/>
       <c r="H97" s="2" t="n"/>
-      <c r="I97" s="2" t="n"/>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>history of exposure to asbestos due to one's job</t>
+        </is>
+      </c>
       <c r="J97" s="2" t="n"/>
       <c r="K97" s="2" t="inlineStr">
         <is>
@@ -5938,20 +5938,20 @@
           <t>A personal history part that includes experience of physical, sexual, or psychological maltreatment during the first 18 years of life.</t>
         </is>
       </c>
-      <c r="D98" s="2" t="inlineStr">
-        <is>
-          <t>personal history part</t>
-        </is>
-      </c>
+      <c r="D98" s="2" t="n"/>
       <c r="E98" s="2" t="n"/>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>history of physical abuse by a parent</t>
+          <t>personal history part</t>
         </is>
       </c>
       <c r="G98" s="2" t="n"/>
       <c r="H98" s="2" t="n"/>
-      <c r="I98" s="2" t="n"/>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>history of physical abuse by a parent</t>
+        </is>
+      </c>
       <c r="J98" s="2" t="n"/>
       <c r="K98" s="2" t="inlineStr">
         <is>
@@ -5997,13 +5997,13 @@
           <t>A person who does not own a residential facility and does not have an agreement with a residential facility owner that would enable them to live in a residential facility.</t>
         </is>
       </c>
-      <c r="D99" s="2" t="inlineStr">
+      <c r="D99" s="2" t="n"/>
+      <c r="E99" s="2" t="n"/>
+      <c r="F99" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E99" s="2" t="n"/>
-      <c r="F99" s="2" t="n"/>
       <c r="G99" s="2" t="n"/>
       <c r="H99" s="2" t="inlineStr">
         <is>
@@ -6056,13 +6056,13 @@
           <t>A personal attribute inhering in a person who does not bear a role realised in an employment process and who manages their home as their main daily activity.</t>
         </is>
       </c>
-      <c r="D100" s="2" t="inlineStr">
+      <c r="D100" s="2" t="n"/>
+      <c r="E100" s="2" t="n"/>
+      <c r="F100" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E100" s="2" t="n"/>
-      <c r="F100" s="2" t="n"/>
       <c r="G100" s="2" t="inlineStr">
         <is>
           <t>NCIT_C75560</t>
@@ -6115,13 +6115,13 @@
           <t>A sexual orientation of an individual who experiences sexual attraction exclusively or primarily to members of the same sex.</t>
         </is>
       </c>
-      <c r="D101" s="2" t="inlineStr">
+      <c r="D101" s="2" t="n"/>
+      <c r="E101" s="2" t="n"/>
+      <c r="F101" s="2" t="inlineStr">
         <is>
           <t>sexual orientation</t>
         </is>
       </c>
-      <c r="E101" s="2" t="n"/>
-      <c r="F101" s="2" t="n"/>
       <c r="G101" s="2" t="inlineStr">
         <is>
           <t>NCIT_C84363</t>
@@ -6174,7 +6174,7 @@
           <t>A human or collection of humans that occupies a housing unit by storing their possessions there and habitually sleeping there thereby participating in the realization of its residence function.</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr">
+      <c r="F102" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>
@@ -6211,13 +6211,13 @@
           <t>An aggregate of the individual incomes received by all the members of a household.</t>
         </is>
       </c>
-      <c r="D103" s="2" t="inlineStr">
+      <c r="D103" s="2" t="n"/>
+      <c r="E103" s="2" t="n"/>
+      <c r="F103" s="2" t="inlineStr">
         <is>
           <t>object aggregate</t>
         </is>
       </c>
-      <c r="E103" s="2" t="n"/>
-      <c r="F103" s="2" t="n"/>
       <c r="G103" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">EFO_0009695 </t>
@@ -6274,13 +6274,13 @@
           <t>A personal attribute that is a time quality inhering in a person by virtue of how long since the person was born.</t>
         </is>
       </c>
-      <c r="D104" s="2" t="inlineStr">
+      <c r="D104" s="2" t="n"/>
+      <c r="E104" s="2" t="n"/>
+      <c r="F104" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E104" s="2" t="n"/>
-      <c r="F104" s="2" t="n"/>
       <c r="G104" s="2" t="inlineStr">
         <is>
           <t>PATO:0000011</t>
@@ -6333,13 +6333,13 @@
           <t>An object aggregate that consists of two or more people.</t>
         </is>
       </c>
-      <c r="D105" s="2" t="inlineStr">
+      <c r="D105" s="2" t="n"/>
+      <c r="E105" s="2" t="n"/>
+      <c r="F105" s="2" t="inlineStr">
         <is>
           <t>object aggregate</t>
         </is>
       </c>
-      <c r="E105" s="2" t="n"/>
-      <c r="F105" s="2" t="n"/>
       <c r="G105" s="2" t="n"/>
       <c r="H105" s="2" t="n"/>
       <c r="I105" s="2" t="n"/>
@@ -6380,7 +6380,7 @@
           <t>A cognitive representation of themselves by a person or group.</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr">
+      <c r="F106" t="inlineStr">
         <is>
           <t>cognitive representation</t>
         </is>
@@ -6412,13 +6412,13 @@
           <t>A person who has previously been a resident of a country and is now resident in another country.</t>
         </is>
       </c>
-      <c r="D107" s="2" t="inlineStr">
+      <c r="D107" s="2" t="n"/>
+      <c r="E107" s="2" t="n"/>
+      <c r="F107" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E107" s="2" t="n"/>
-      <c r="F107" s="2" t="n"/>
       <c r="G107" s="2" t="n"/>
       <c r="H107" s="2" t="n"/>
       <c r="I107" s="2" t="n"/>
@@ -6467,13 +6467,13 @@
           <t xml:space="preserve">A relationship status where the individual is in a legally formalised marriage or civil partnership. </t>
         </is>
       </c>
-      <c r="D108" s="2" t="inlineStr">
+      <c r="D108" s="2" t="n"/>
+      <c r="E108" s="2" t="n"/>
+      <c r="F108" s="2" t="inlineStr">
         <is>
           <t>relationship status</t>
         </is>
       </c>
-      <c r="E108" s="2" t="n"/>
-      <c r="F108" s="2" t="n"/>
       <c r="G108" s="2" t="n"/>
       <c r="H108" s="2" t="n"/>
       <c r="I108" s="2" t="n"/>
@@ -6523,13 +6523,13 @@
           <t>A relationship status where the individual has had the same partner for a significant length of time but is not in a legal union.</t>
         </is>
       </c>
-      <c r="D109" s="2" t="inlineStr">
+      <c r="D109" s="2" t="n"/>
+      <c r="E109" s="2" t="n"/>
+      <c r="F109" s="2" t="inlineStr">
         <is>
           <t>relationship status</t>
         </is>
       </c>
-      <c r="E109" s="2" t="n"/>
-      <c r="F109" s="2" t="n"/>
       <c r="G109" s="2" t="n"/>
       <c r="H109" s="2" t="n"/>
       <c r="I109" s="2" t="n"/>
@@ -6582,13 +6582,13 @@
           <t>An employment status realised by an individual working for a company or other organisation without a pre-determined end date, with security of employment and known working conditions.</t>
         </is>
       </c>
-      <c r="D110" s="2" t="inlineStr">
+      <c r="D110" s="2" t="n"/>
+      <c r="E110" s="2" t="n"/>
+      <c r="F110" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E110" s="2" t="n"/>
-      <c r="F110" s="2" t="n"/>
       <c r="G110" s="2" t="n"/>
       <c r="H110" s="2" t="n"/>
       <c r="I110" s="2" t="n"/>
@@ -6637,13 +6637,13 @@
           <t>An employment status realised by an individual working for a company or other organisation in a position that is of a known, fixed duration with security of employment for that duration and certain working conditions.</t>
         </is>
       </c>
-      <c r="D111" s="2" t="inlineStr">
+      <c r="D111" s="2" t="n"/>
+      <c r="E111" s="2" t="n"/>
+      <c r="F111" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E111" s="2" t="n"/>
-      <c r="F111" s="2" t="n"/>
       <c r="G111" s="2" t="n"/>
       <c r="H111" s="2" t="n"/>
       <c r="I111" s="2" t="n"/>
@@ -6692,13 +6692,13 @@
           <t>An employment status realised by an individual working for a company or other organisation in a position with uncertain duration or hours with unknown or low security of working conditions or pay.</t>
         </is>
       </c>
-      <c r="D112" s="2" t="inlineStr">
+      <c r="D112" s="2" t="n"/>
+      <c r="E112" s="2" t="n"/>
+      <c r="F112" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E112" s="2" t="n"/>
-      <c r="F112" s="2" t="n"/>
       <c r="G112" s="2" t="n"/>
       <c r="H112" s="2" t="n"/>
       <c r="I112" s="2" t="n"/>
@@ -6747,13 +6747,13 @@
           <t>Individual income that an individual otherwise of low-income receives as a payment made by the state or an insurance scheme in the form of housing vouchers,  credit or benefits.</t>
         </is>
       </c>
-      <c r="D113" s="2" t="inlineStr">
+      <c r="D113" s="2" t="n"/>
+      <c r="E113" s="2" t="n"/>
+      <c r="F113" s="2" t="inlineStr">
         <is>
           <t>individual income</t>
         </is>
       </c>
-      <c r="E113" s="2" t="n"/>
-      <c r="F113" s="2" t="n"/>
       <c r="G113" s="2" t="n"/>
       <c r="H113" s="2" t="n"/>
       <c r="I113" s="2" t="n"/>
@@ -6802,13 +6802,13 @@
           <t>A personal attribute inhering in a person who does not bear a role realised in an employment process due to possessing enough wealth to not need financial support from another person or require income from employment.</t>
         </is>
       </c>
-      <c r="D114" s="2" t="inlineStr">
+      <c r="D114" s="2" t="n"/>
+      <c r="E114" s="2" t="n"/>
+      <c r="F114" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E114" s="2" t="n"/>
-      <c r="F114" s="2" t="n"/>
       <c r="G114" s="2" t="n"/>
       <c r="H114" s="2" t="n"/>
       <c r="I114" s="2" t="n"/>
@@ -6857,20 +6857,20 @@
           <t>A bodily process of a human that involves co-ordinated contraction of striated muscles controlled by the brain.</t>
         </is>
       </c>
-      <c r="D115" s="2" t="inlineStr">
-        <is>
-          <t>bodily process</t>
-        </is>
-      </c>
+      <c r="D115" s="2" t="n"/>
       <c r="E115" s="2" t="n"/>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>walks for 15 mins/day, never eats meat, attends school daily</t>
+          <t>bodily process</t>
         </is>
       </c>
       <c r="G115" s="2" t="n"/>
       <c r="H115" s="2" t="n"/>
-      <c r="I115" s="2" t="n"/>
+      <c r="I115" s="2" t="inlineStr">
+        <is>
+          <t>walks for 15 mins/day, never eats meat, attends school daily</t>
+        </is>
+      </c>
       <c r="J115" s="2" t="n"/>
       <c r="K115" s="2" t="inlineStr">
         <is>
@@ -6916,13 +6916,13 @@
           <t>A personal attribute reflecting a benefit the person receives  derived from their capital or labour, usually measured in money.</t>
         </is>
       </c>
-      <c r="D116" s="2" t="inlineStr">
+      <c r="D116" s="2" t="n"/>
+      <c r="E116" s="2" t="n"/>
+      <c r="F116" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E116" s="2" t="n"/>
-      <c r="F116" s="2" t="n"/>
       <c r="G116" s="2" t="inlineStr">
         <is>
           <t>OMRSE_00002061</t>
@@ -6975,13 +6975,13 @@
           <t>A social role that involves influencing other people to adopt new ideas or behaviours.</t>
         </is>
       </c>
-      <c r="D117" s="2" t="inlineStr">
+      <c r="D117" s="2" t="n"/>
+      <c r="E117" s="2" t="n"/>
+      <c r="F117" s="2" t="inlineStr">
         <is>
           <t>social role</t>
         </is>
       </c>
-      <c r="E117" s="2" t="n"/>
-      <c r="F117" s="2" t="n"/>
       <c r="G117" s="2" t="n"/>
       <c r="H117" s="2" t="n"/>
       <c r="I117" s="2" t="n"/>
@@ -7030,13 +7030,13 @@
           <t>A student or trainee role realised by  currently learning in a non-institutional setting.</t>
         </is>
       </c>
-      <c r="D118" s="3" t="inlineStr">
+      <c r="D118" s="3" t="n"/>
+      <c r="E118" s="3" t="n"/>
+      <c r="F118" s="3" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E118" s="3" t="n"/>
-      <c r="F118" s="3" t="n"/>
       <c r="G118" s="3" t="n"/>
       <c r="H118" s="3" t="n"/>
       <c r="I118" s="3" t="n"/>
@@ -7085,13 +7085,13 @@
           <t>A student or trainee that is currently learning in a non-institutional setting.</t>
         </is>
       </c>
-      <c r="D119" s="2" t="inlineStr">
+      <c r="D119" s="2" t="n"/>
+      <c r="E119" s="2" t="n"/>
+      <c r="F119" s="2" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E119" s="2" t="n"/>
-      <c r="F119" s="2" t="n"/>
       <c r="G119" s="2" t="n"/>
       <c r="H119" s="2" t="n"/>
       <c r="I119" s="2" t="n"/>
@@ -7140,13 +7140,13 @@
           <t>A patient role which inheres in a person and is realized by being under the care of a physician or health care provider and being admitted to a hospital or equivalent facility.</t>
         </is>
       </c>
-      <c r="D120" s="2" t="inlineStr">
+      <c r="D120" s="2" t="n"/>
+      <c r="E120" s="2" t="n"/>
+      <c r="F120" s="2" t="inlineStr">
         <is>
           <t>patient role</t>
         </is>
       </c>
-      <c r="E120" s="2" t="n"/>
-      <c r="F120" s="2" t="n"/>
       <c r="G120" s="2" t="n"/>
       <c r="H120" s="2" t="n"/>
       <c r="I120" s="2" t="n"/>
@@ -7195,13 +7195,13 @@
           <t xml:space="preserve">A role that inheres in an organism that is able to receive benefits from an insurance policy. </t>
         </is>
       </c>
-      <c r="D121" s="3" t="inlineStr">
+      <c r="D121" s="3" t="n"/>
+      <c r="E121" s="3" t="n"/>
+      <c r="F121" s="3" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="E121" s="3" t="n"/>
-      <c r="F121" s="3" t="n"/>
       <c r="G121" s="3" t="inlineStr">
         <is>
           <t>OMRSE:00000092</t>
@@ -7258,7 +7258,7 @@
           <t xml:space="preserve">A role that inheres in an organism that is able to receive benefits from an insurance policy. </t>
         </is>
       </c>
-      <c r="D122" t="inlineStr">
+      <c r="F122" t="inlineStr">
         <is>
           <t>role</t>
         </is>
@@ -7310,13 +7310,13 @@
           <t>A role relating to personal relationships or association between an individual and other individuals, including kinship relations, romantic, business, and social interactions.</t>
         </is>
       </c>
-      <c r="D123" s="2" t="inlineStr">
+      <c r="D123" s="2" t="n"/>
+      <c r="E123" s="2" t="n"/>
+      <c r="F123" s="2" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="E123" s="2" t="n"/>
-      <c r="F123" s="2" t="n"/>
       <c r="G123" s="2" t="inlineStr">
         <is>
           <t>NCIT_C92454</t>
@@ -7369,13 +7369,13 @@
           <t>A person who is exposed to an intervention.</t>
         </is>
       </c>
-      <c r="D124" s="2" t="inlineStr">
+      <c r="D124" s="2" t="n"/>
+      <c r="E124" s="2" t="n"/>
+      <c r="F124" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E124" s="2" t="n"/>
-      <c r="F124" s="2" t="n"/>
       <c r="G124" s="2" t="n"/>
       <c r="H124" s="2" t="n"/>
       <c r="I124" s="2" t="n"/>
@@ -7416,13 +7416,13 @@
           <t>A human population who are exposed to an intervention.</t>
         </is>
       </c>
-      <c r="D125" s="2" t="inlineStr">
+      <c r="D125" s="2" t="n"/>
+      <c r="E125" s="2" t="n"/>
+      <c r="F125" s="2" t="inlineStr">
         <is>
           <t>human population</t>
         </is>
       </c>
-      <c r="E125" s="2" t="n"/>
-      <c r="F125" s="2" t="n"/>
       <c r="G125" s="2" t="n"/>
       <c r="H125" s="2" t="n"/>
       <c r="I125" s="2" t="n"/>
@@ -7463,20 +7463,20 @@
           <t>A linguistic capability that is realised by using a language accurately and appropriately in more than one setting.</t>
         </is>
       </c>
-      <c r="D126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">linguistic capability </t>
-        </is>
-      </c>
+      <c r="D126" s="2" t="n"/>
       <c r="E126" s="2" t="n"/>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Callers eligible for the study were adult cigarette smokers able to communicate in English </t>
+          <t xml:space="preserve">linguistic capability </t>
         </is>
       </c>
       <c r="G126" s="2" t="n"/>
       <c r="H126" s="2" t="n"/>
-      <c r="I126" s="2" t="n"/>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Callers eligible for the study were adult cigarette smokers able to communicate in English </t>
+        </is>
+      </c>
       <c r="J126" s="2" t="n"/>
       <c r="K126" s="2" t="inlineStr">
         <is>
@@ -7522,13 +7522,13 @@
           <t>A social role in which the holder is given or creates authority to exert influence on other members of a social group.</t>
         </is>
       </c>
-      <c r="D127" s="2" t="inlineStr">
+      <c r="D127" s="2" t="n"/>
+      <c r="E127" s="2" t="n"/>
+      <c r="F127" s="2" t="inlineStr">
         <is>
           <t>social role</t>
         </is>
       </c>
-      <c r="E127" s="2" t="n"/>
-      <c r="F127" s="2" t="n"/>
       <c r="G127" s="2" t="n"/>
       <c r="H127" s="2" t="n"/>
       <c r="I127" s="2" t="n"/>
@@ -7577,7 +7577,7 @@
           <t>A mental capability that is realised in processes of communication involving language or in expressions of language.</t>
         </is>
       </c>
-      <c r="D128" t="inlineStr">
+      <c r="F128" t="inlineStr">
         <is>
           <t>mental capability</t>
         </is>
@@ -7619,13 +7619,13 @@
           <t>Disabled for at least 12 months.</t>
         </is>
       </c>
-      <c r="D129" s="2" t="inlineStr">
+      <c r="D129" s="2" t="n"/>
+      <c r="E129" s="2" t="n"/>
+      <c r="F129" s="2" t="inlineStr">
         <is>
           <t>disabled</t>
         </is>
       </c>
-      <c r="E129" s="2" t="n"/>
-      <c r="F129" s="2" t="n"/>
       <c r="G129" s="2" t="n"/>
       <c r="H129" s="2" t="n"/>
       <c r="I129" s="2" t="n"/>
@@ -7679,13 +7679,13 @@
           <t>A frequency of past behaviour that is below a threshold.</t>
         </is>
       </c>
-      <c r="D130" s="2" t="inlineStr">
+      <c r="D130" s="2" t="n"/>
+      <c r="E130" s="2" t="n"/>
+      <c r="F130" s="2" t="inlineStr">
         <is>
           <t>frequency of past behaviour</t>
         </is>
       </c>
-      <c r="E130" s="2" t="n"/>
-      <c r="F130" s="2" t="n"/>
       <c r="G130" s="2" t="n"/>
       <c r="H130" s="2" t="n"/>
       <c r="I130" s="2" t="n"/>
@@ -7730,13 +7730,13 @@
           <t>A biological sex associated with the ability to produce male gametes.</t>
         </is>
       </c>
-      <c r="D131" s="2" t="inlineStr">
+      <c r="D131" s="2" t="n"/>
+      <c r="E131" s="2" t="n"/>
+      <c r="F131" s="2" t="inlineStr">
         <is>
           <t>biological sex</t>
         </is>
       </c>
-      <c r="E131" s="2" t="n"/>
-      <c r="F131" s="2" t="n"/>
       <c r="G131" s="2" t="n"/>
       <c r="H131" s="2" t="n"/>
       <c r="I131" s="2" t="n"/>
@@ -7785,13 +7785,13 @@
           <t>A gender identity as being male.</t>
         </is>
       </c>
-      <c r="D132" s="2" t="inlineStr">
+      <c r="D132" s="2" t="n"/>
+      <c r="E132" s="2" t="n"/>
+      <c r="F132" s="2" t="inlineStr">
         <is>
           <t>gender identity</t>
         </is>
       </c>
-      <c r="E132" s="2" t="n"/>
-      <c r="F132" s="2" t="n"/>
       <c r="G132" s="2" t="inlineStr">
         <is>
           <t>GSSO:000090</t>
@@ -7848,13 +7848,13 @@
           <t>A higher education student  role realised by currently studying for a masters degree.</t>
         </is>
       </c>
-      <c r="D133" s="3" t="inlineStr">
+      <c r="D133" s="3" t="n"/>
+      <c r="E133" s="3" t="n"/>
+      <c r="F133" s="3" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E133" s="3" t="n"/>
-      <c r="F133" s="3" t="n"/>
       <c r="G133" s="3" t="n"/>
       <c r="H133" s="3" t="n"/>
       <c r="I133" s="3" t="n"/>
@@ -7903,13 +7903,13 @@
           <t>A higher education student  role realised by currently studying for a masters degree.</t>
         </is>
       </c>
-      <c r="D134" s="2" t="inlineStr">
+      <c r="D134" s="2" t="n"/>
+      <c r="E134" s="2" t="n"/>
+      <c r="F134" s="2" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E134" s="2" t="n"/>
-      <c r="F134" s="2" t="n"/>
       <c r="G134" s="2" t="n"/>
       <c r="H134" s="2" t="n"/>
       <c r="I134" s="2" t="n"/>
@@ -7958,20 +7958,20 @@
           <t>A health status attribute that is having been prescribed the use of one or more drugs to improve, maintain or protect one's health.</t>
         </is>
       </c>
-      <c r="D135" s="2" t="inlineStr">
-        <is>
-          <t>health status attribute</t>
-        </is>
-      </c>
+      <c r="D135" s="2" t="n"/>
       <c r="E135" s="2" t="n"/>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>prescribed at least one antihypertensive medication, taking asthma preventer inhalers</t>
+          <t>health status attribute</t>
         </is>
       </c>
       <c r="G135" s="2" t="n"/>
       <c r="H135" s="2" t="n"/>
-      <c r="I135" s="2" t="n"/>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
+          <t>prescribed at least one antihypertensive medication, taking asthma preventer inhalers</t>
+        </is>
+      </c>
       <c r="J135" s="2" t="inlineStr">
         <is>
           <t>This entity reflects having been prescribed a medication.  Actual use of the medicine would be captured as a behaviour</t>
@@ -8021,13 +8021,13 @@
           <t>A person living in  a household with at least one other person.</t>
         </is>
       </c>
-      <c r="D136" s="2" t="inlineStr">
+      <c r="D136" s="2" t="n"/>
+      <c r="E136" s="2" t="n"/>
+      <c r="F136" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E136" s="2" t="n"/>
-      <c r="F136" s="2" t="n"/>
       <c r="G136" s="2" t="n"/>
       <c r="H136" s="2" t="n"/>
       <c r="I136" s="2" t="n"/>
@@ -8080,24 +8080,24 @@
           <t>A member of a multi-person household where all of the household members are related.</t>
         </is>
       </c>
-      <c r="D137" s="2" t="inlineStr">
-        <is>
-          <t>member of a multi-person household</t>
-        </is>
-      </c>
+      <c r="D137" s="2" t="n"/>
       <c r="E137" s="2" t="n"/>
       <c r="F137" s="2" t="inlineStr">
         <is>
+          <t>member of a multi-person household</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NCIT:C25173;PCO:0000020;STATO:0000257 </t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="n"/>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
           <t>1) Co-habitating couple and their socially recognised children and elderly parents. 2) Co habitating couple with child and grandchild.</t>
         </is>
       </c>
-      <c r="G137" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NCIT:C25173;PCO:0000020;STATO:0000257 </t>
-        </is>
-      </c>
-      <c r="H137" s="2" t="n"/>
-      <c r="I137" s="2" t="n"/>
       <c r="J137" s="2" t="n"/>
       <c r="K137" s="2" t="inlineStr">
         <is>
@@ -8143,20 +8143,20 @@
           <t>A member of a multi-person household where none of the household members are related.</t>
         </is>
       </c>
-      <c r="D138" s="2" t="inlineStr">
-        <is>
-          <t>member of a multi-person household</t>
-        </is>
-      </c>
+      <c r="D138" s="2" t="n"/>
       <c r="E138" s="2" t="n"/>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>1) Two unrelated couples (unmarried couples). 2) Students sharing living accommodation. 3) Single professionals renting a room in a shared house.</t>
+          <t>member of a multi-person household</t>
         </is>
       </c>
       <c r="G138" s="2" t="n"/>
       <c r="H138" s="2" t="n"/>
-      <c r="I138" s="2" t="n"/>
+      <c r="I138" s="2" t="inlineStr">
+        <is>
+          <t>1) Two unrelated couples (unmarried couples). 2) Students sharing living accommodation. 3) Single professionals renting a room in a shared house.</t>
+        </is>
+      </c>
       <c r="J138" s="2" t="n"/>
       <c r="K138" s="2" t="inlineStr">
         <is>
@@ -8202,20 +8202,20 @@
           <t>A member of a multi-person household where some household members are related.</t>
         </is>
       </c>
-      <c r="D139" s="2" t="inlineStr">
-        <is>
-          <t>member of a multi-person household</t>
-        </is>
-      </c>
+      <c r="D139" s="2" t="n"/>
       <c r="E139" s="2" t="n"/>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>1) Cohabiting couple plus son and girlfriend. 2) Two brothers and their partners</t>
+          <t>member of a multi-person household</t>
         </is>
       </c>
       <c r="G139" s="2" t="n"/>
       <c r="H139" s="2" t="n"/>
-      <c r="I139" s="2" t="n"/>
+      <c r="I139" s="2" t="inlineStr">
+        <is>
+          <t>1) Cohabiting couple plus son and girlfriend. 2) Two brothers and their partners</t>
+        </is>
+      </c>
       <c r="J139" s="2" t="n"/>
       <c r="K139" s="2" t="inlineStr">
         <is>
@@ -8261,20 +8261,20 @@
           <t>A member of a multi-person household where some household members belong to different generations.</t>
         </is>
       </c>
-      <c r="D140" s="2" t="inlineStr">
-        <is>
-          <t>member of a multi-person household</t>
-        </is>
-      </c>
+      <c r="D140" s="2" t="n"/>
       <c r="E140" s="2" t="n"/>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>1) A family unit of a pair of adults and their socially recognized children. 2) Co-habitating couples plus socially recognised children and elderly parents or grandchildren.</t>
+          <t>member of a multi-person household</t>
         </is>
       </c>
       <c r="G140" s="2" t="n"/>
       <c r="H140" s="2" t="n"/>
-      <c r="I140" s="2" t="n"/>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>1) A family unit of a pair of adults and their socially recognized children. 2) Co-habitating couples plus socially recognised children and elderly parents or grandchildren.</t>
+        </is>
+      </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
           <t>A member of a multi-generational household lives with other people that are from more than one generation. A generation is all the people of about the same age within a society or within a particular family</t>
@@ -8324,13 +8324,13 @@
           <t>A person living alone in a household.</t>
         </is>
       </c>
-      <c r="D141" s="2" t="inlineStr">
+      <c r="D141" s="2" t="n"/>
+      <c r="E141" s="2" t="n"/>
+      <c r="F141" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E141" s="2" t="n"/>
-      <c r="F141" s="2" t="n"/>
       <c r="G141" s="2" t="n"/>
       <c r="H141" s="2" t="n"/>
       <c r="I141" s="2" t="n"/>
@@ -8379,7 +8379,7 @@
           <t>A personal capability that includes mental processes in its realisation.</t>
         </is>
       </c>
-      <c r="D142" t="inlineStr">
+      <c r="F142" t="inlineStr">
         <is>
           <t>personal capability</t>
         </is>
@@ -8421,13 +8421,13 @@
           <t>A parent who is female gender.</t>
         </is>
       </c>
-      <c r="D143" s="2" t="inlineStr">
+      <c r="D143" s="2" t="n"/>
+      <c r="E143" s="2" t="n"/>
+      <c r="F143" s="2" t="inlineStr">
         <is>
           <t>parent</t>
         </is>
       </c>
-      <c r="E143" s="2" t="n"/>
-      <c r="F143" s="2" t="n"/>
       <c r="G143" s="2" t="n"/>
       <c r="H143" s="2" t="n"/>
       <c r="I143" s="2" t="n"/>
@@ -8476,13 +8476,13 @@
           <t xml:space="preserve">A family member who is a child relation of one's sibling and is male gender. </t>
         </is>
       </c>
-      <c r="D144" s="2" t="inlineStr">
+      <c r="D144" s="2" t="n"/>
+      <c r="E144" s="2" t="n"/>
+      <c r="F144" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E144" s="2" t="n"/>
-      <c r="F144" s="2" t="n"/>
       <c r="G144" s="2" t="n"/>
       <c r="H144" s="2" t="n"/>
       <c r="I144" s="2" t="n"/>
@@ -8531,13 +8531,13 @@
           <t>A family member who is a child relation of one's sibling and is female gender.</t>
         </is>
       </c>
-      <c r="D145" s="2" t="inlineStr">
+      <c r="D145" s="2" t="n"/>
+      <c r="E145" s="2" t="n"/>
+      <c r="F145" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E145" s="2" t="n"/>
-      <c r="F145" s="2" t="n"/>
       <c r="G145" s="2" t="n"/>
       <c r="H145" s="2" t="n"/>
       <c r="I145" s="2" t="n"/>
@@ -8586,13 +8586,13 @@
           <t>A self-identity as not having a particular gender.</t>
         </is>
       </c>
-      <c r="D146" s="2" t="inlineStr">
+      <c r="D146" s="2" t="n"/>
+      <c r="E146" s="2" t="n"/>
+      <c r="F146" s="2" t="inlineStr">
         <is>
           <t>self-identity</t>
         </is>
       </c>
-      <c r="E146" s="2" t="n"/>
-      <c r="F146" s="2" t="n"/>
       <c r="G146" s="2" t="inlineStr">
         <is>
           <t>GSSO:002331</t>
@@ -8645,13 +8645,13 @@
           <t>A gender identity as having a gender that is not well-described by the binary categories of male or female.</t>
         </is>
       </c>
-      <c r="D147" s="2" t="inlineStr">
+      <c r="D147" s="2" t="n"/>
+      <c r="E147" s="2" t="n"/>
+      <c r="F147" s="2" t="inlineStr">
         <is>
           <t>gender identity</t>
         </is>
       </c>
-      <c r="E147" s="2" t="n"/>
-      <c r="F147" s="2" t="n"/>
       <c r="G147" s="2" t="inlineStr">
         <is>
           <t>GSSO:002328</t>
@@ -8704,13 +8704,13 @@
           <t>A personal attribute inhering in a person by virtue of that person not having a paid job and not currently seeking to begin participating in an employment process.</t>
         </is>
       </c>
-      <c r="D148" s="2" t="inlineStr">
+      <c r="D148" s="2" t="n"/>
+      <c r="E148" s="2" t="n"/>
+      <c r="F148" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E148" s="2" t="n"/>
-      <c r="F148" s="2" t="n"/>
       <c r="G148" s="2" t="n"/>
       <c r="H148" s="2" t="n"/>
       <c r="I148" s="2" t="n"/>
@@ -8759,13 +8759,13 @@
           <t>A personal attribute inhering in a person by virtue of that person not bearing a role realised in an employment process, due to being unable to work due to illness or disability.</t>
         </is>
       </c>
-      <c r="D149" s="2" t="inlineStr">
+      <c r="D149" s="2" t="n"/>
+      <c r="E149" s="2" t="n"/>
+      <c r="F149" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E149" s="2" t="n"/>
-      <c r="F149" s="2" t="n"/>
       <c r="G149" s="2" t="n"/>
       <c r="H149" s="2" t="n"/>
       <c r="I149" s="2" t="n"/>
@@ -8814,13 +8814,13 @@
           <t>A data item about the number of people in a population.</t>
         </is>
       </c>
-      <c r="D150" s="2" t="inlineStr">
+      <c r="D150" s="2" t="n"/>
+      <c r="E150" s="2" t="n"/>
+      <c r="F150" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E150" s="2" t="n"/>
-      <c r="F150" s="2" t="n"/>
       <c r="G150" s="2" t="n"/>
       <c r="H150" s="2" t="n"/>
       <c r="I150" s="2" t="n"/>
@@ -8861,13 +8861,13 @@
           <t>The number of years a person spent engaged in an education process.</t>
         </is>
       </c>
-      <c r="D151" s="2" t="inlineStr">
+      <c r="D151" s="2" t="n"/>
+      <c r="E151" s="2" t="n"/>
+      <c r="F151" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E151" s="2" t="n"/>
-      <c r="F151" s="2" t="n"/>
       <c r="G151" s="2" t="n"/>
       <c r="H151" s="2" t="n"/>
       <c r="I151" s="2" t="n"/>
@@ -8920,13 +8920,13 @@
           <t>A personal role that is realised in a person by doing a specified type of work or working in a specified way.</t>
         </is>
       </c>
-      <c r="D152" s="2" t="inlineStr">
+      <c r="D152" s="2" t="n"/>
+      <c r="E152" s="2" t="n"/>
+      <c r="F152" s="2" t="inlineStr">
         <is>
           <t>personal role</t>
         </is>
       </c>
-      <c r="E152" s="2" t="n"/>
-      <c r="F152" s="2" t="n"/>
       <c r="G152" s="2" t="n"/>
       <c r="H152" s="2" t="n"/>
       <c r="I152" s="2" t="n"/>
@@ -8975,13 +8975,13 @@
           <t>A person who lives in a residential facility they do not own  with the agreement of the residential facility owner, by virtue of the occupier bearing a role realised in an employment process.</t>
         </is>
       </c>
-      <c r="D153" s="2" t="inlineStr">
+      <c r="D153" s="2" t="n"/>
+      <c r="E153" s="2" t="n"/>
+      <c r="F153" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E153" s="2" t="n"/>
-      <c r="F153" s="2" t="n"/>
       <c r="G153" s="2" t="n"/>
       <c r="H153" s="2" t="n"/>
       <c r="I153" s="2" t="n"/>
@@ -9030,20 +9030,20 @@
           <t>A role which inheres in a person and is realised by performing the activities deemed appropriate for that particular role as specified in the organisation rules.</t>
         </is>
       </c>
-      <c r="D154" s="2" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
+      <c r="D154" s="2" t="n"/>
       <c r="E154" s="2" t="n"/>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>Scout leader, club chairperson</t>
+          <t>role</t>
         </is>
       </c>
       <c r="G154" s="2" t="n"/>
       <c r="H154" s="2" t="n"/>
-      <c r="I154" s="2" t="n"/>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>Scout leader, club chairperson</t>
+        </is>
+      </c>
       <c r="J154" s="2" t="n"/>
       <c r="K154" s="2" t="inlineStr">
         <is>
@@ -9089,13 +9089,13 @@
           <t>A sexual orientation of an individual who is sure of their sexual orientation and reports it as other than asexual, bisexual, heterosexual, homosexual, queer or questioning.</t>
         </is>
       </c>
-      <c r="D155" s="2" t="inlineStr">
+      <c r="D155" s="2" t="n"/>
+      <c r="E155" s="2" t="n"/>
+      <c r="F155" s="2" t="inlineStr">
         <is>
           <t>sexual orientation</t>
         </is>
       </c>
-      <c r="E155" s="2" t="n"/>
-      <c r="F155" s="2" t="n"/>
       <c r="G155" s="2" t="n"/>
       <c r="H155" s="2" t="n"/>
       <c r="I155" s="2" t="n"/>
@@ -9144,13 +9144,13 @@
           <t>A social group that is part of a person’s social environmental system and with which the person does not identify.</t>
         </is>
       </c>
-      <c r="D156" s="2" t="inlineStr">
+      <c r="D156" s="2" t="n"/>
+      <c r="E156" s="2" t="n"/>
+      <c r="F156" s="2" t="inlineStr">
         <is>
           <t>social group</t>
         </is>
       </c>
-      <c r="E156" s="2" t="n"/>
-      <c r="F156" s="2" t="n"/>
       <c r="G156" s="2" t="n"/>
       <c r="H156" s="2" t="n"/>
       <c r="I156" s="2" t="n"/>
@@ -9191,13 +9191,13 @@
           <t>A patient role which inheres in a person and is realized by coming to a healthcare facility for diagnosis or treatment but not being admitted for an overnight stay.</t>
         </is>
       </c>
-      <c r="D157" s="2" t="inlineStr">
+      <c r="D157" s="2" t="n"/>
+      <c r="E157" s="2" t="n"/>
+      <c r="F157" s="2" t="inlineStr">
         <is>
           <t>patient role</t>
         </is>
       </c>
-      <c r="E157" s="2" t="n"/>
-      <c r="F157" s="2" t="n"/>
       <c r="G157" s="2" t="n"/>
       <c r="H157" s="2" t="n"/>
       <c r="I157" s="2" t="n"/>
@@ -9246,13 +9246,13 @@
           <t>A person or organization that participates in an ownership process wherein they realize their role as owner by exercising their right to use, sell, rent, or gift an object.</t>
         </is>
       </c>
-      <c r="D158" s="2" t="inlineStr">
+      <c r="D158" s="2" t="n"/>
+      <c r="E158" s="2" t="n"/>
+      <c r="F158" s="2" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>
       </c>
-      <c r="E158" s="2" t="n"/>
-      <c r="F158" s="2" t="n"/>
       <c r="G158" s="2" t="inlineStr">
         <is>
           <t>owner in the Sustainable Development Goals Interface Ontology (SDGIO:00010028)</t>
@@ -9309,13 +9309,13 @@
           <t>A person who lives in a residential facility of which they are the residential facility owner</t>
         </is>
       </c>
-      <c r="D159" s="2" t="inlineStr">
+      <c r="D159" s="2" t="n"/>
+      <c r="E159" s="2" t="n"/>
+      <c r="F159" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E159" s="2" t="n"/>
-      <c r="F159" s="2" t="n"/>
       <c r="G159" s="2" t="n"/>
       <c r="H159" s="2" t="n"/>
       <c r="I159" s="2" t="n"/>
@@ -9365,13 +9365,13 @@
           <t xml:space="preserve">A family member who is a key caretaker or immediate progenitor of a child. </t>
         </is>
       </c>
-      <c r="D160" s="2" t="inlineStr">
+      <c r="D160" s="2" t="n"/>
+      <c r="E160" s="2" t="n"/>
+      <c r="F160" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E160" s="2" t="n"/>
-      <c r="F160" s="2" t="n"/>
       <c r="G160" s="2" t="inlineStr">
         <is>
           <t>GSSO:001953</t>
@@ -9424,13 +9424,13 @@
           <t>An interpersonal role that is realised through a process of promoting and supporting the physical, emotional, social, and intellectual development of a child from infancy to adulthood.</t>
         </is>
       </c>
-      <c r="D161" s="2" t="inlineStr">
+      <c r="D161" s="2" t="n"/>
+      <c r="E161" s="2" t="n"/>
+      <c r="F161" s="2" t="inlineStr">
         <is>
           <t>interpersonal role</t>
         </is>
       </c>
-      <c r="E161" s="2" t="n"/>
-      <c r="F161" s="2" t="n"/>
       <c r="G161" s="2" t="n"/>
       <c r="H161" s="2" t="n"/>
       <c r="I161" s="2" t="n"/>
@@ -9483,13 +9483,13 @@
           <t>A personal history part that includes a behaviour.</t>
         </is>
       </c>
-      <c r="D162" s="2" t="inlineStr">
+      <c r="D162" s="2" t="n"/>
+      <c r="E162" s="2" t="n"/>
+      <c r="F162" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E162" s="2" t="n"/>
-      <c r="F162" s="2" t="n"/>
       <c r="G162" s="2" t="n"/>
       <c r="H162" s="2" t="n"/>
       <c r="I162" s="2" t="n"/>
@@ -9534,13 +9534,13 @@
           <t>A past behaviour that is the target of an intervention.</t>
         </is>
       </c>
-      <c r="D163" s="2" t="inlineStr">
+      <c r="D163" s="2" t="n"/>
+      <c r="E163" s="2" t="n"/>
+      <c r="F163" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">past behaviour </t>
         </is>
       </c>
-      <c r="E163" s="2" t="n"/>
-      <c r="F163" s="2" t="n"/>
       <c r="G163" s="2" t="n"/>
       <c r="H163" s="2" t="n"/>
       <c r="I163" s="2" t="n"/>
@@ -9585,7 +9585,7 @@
           <t>A role which inheres in a person and is realized by being under the care of a physician or health care provider.</t>
         </is>
       </c>
-      <c r="D164" t="inlineStr">
+      <c r="F164" t="inlineStr">
         <is>
           <t>role</t>
         </is>
@@ -9628,13 +9628,13 @@
           <t>A &lt;human population&gt; whose members are people with an intervention source role for a specified intervention.</t>
         </is>
       </c>
-      <c r="D165" s="2" t="inlineStr">
+      <c r="D165" s="2" t="n"/>
+      <c r="E165" s="2" t="n"/>
+      <c r="F165" s="2" t="inlineStr">
         <is>
           <t>human population</t>
         </is>
       </c>
-      <c r="E165" s="2" t="n"/>
-      <c r="F165" s="2" t="n"/>
       <c r="G165" s="2" t="n"/>
       <c r="H165" s="2" t="n"/>
       <c r="I165" s="2" t="n"/>
@@ -9675,7 +9675,7 @@
           <t>An extended organism that is a member of the species Homo sapiens.</t>
         </is>
       </c>
-      <c r="D166" t="inlineStr">
+      <c r="F166" t="inlineStr">
         <is>
           <t>extended organism</t>
         </is>
@@ -9707,13 +9707,13 @@
           <t>A &lt;person&gt; who is part of a social environmental system.</t>
         </is>
       </c>
-      <c r="D167" s="2" t="inlineStr">
+      <c r="D167" s="2" t="n"/>
+      <c r="E167" s="2" t="n"/>
+      <c r="F167" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E167" s="2" t="n"/>
-      <c r="F167" s="2" t="n"/>
       <c r="G167" s="2" t="n"/>
       <c r="H167" s="2" t="n"/>
       <c r="I167" s="2" t="n"/>
@@ -9754,13 +9754,13 @@
           <t>A specifically dependent continuant that inheres in a person.</t>
         </is>
       </c>
-      <c r="D168" s="2" t="inlineStr">
+      <c r="D168" s="2" t="n"/>
+      <c r="E168" s="2" t="n"/>
+      <c r="F168" s="2" t="inlineStr">
         <is>
           <t>specifically dependent continuant</t>
         </is>
       </c>
-      <c r="E168" s="2" t="n"/>
-      <c r="F168" s="2" t="n"/>
       <c r="G168" s="2" t="n"/>
       <c r="H168" s="2" t="n"/>
       <c r="I168" s="2" t="n"/>
@@ -9811,12 +9811,12 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
+          <t>The ability of someone to perform some useful and/or beneficial activity.</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
           <t>bodily disposition</t>
-        </is>
-      </c>
-      <c r="I169" t="inlineStr">
-        <is>
-          <t>The ability of someone to perform some useful and/or beneficial activity.</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
@@ -9852,13 +9852,13 @@
           <t>A history that is of a person.</t>
         </is>
       </c>
-      <c r="D170" s="2" t="inlineStr">
+      <c r="D170" s="2" t="n"/>
+      <c r="E170" s="2" t="n"/>
+      <c r="F170" s="2" t="inlineStr">
         <is>
           <t>history</t>
         </is>
       </c>
-      <c r="E170" s="2" t="n"/>
-      <c r="F170" s="2" t="n"/>
       <c r="G170" s="2" t="n"/>
       <c r="H170" s="2" t="n"/>
       <c r="I170" s="2" t="n"/>
@@ -9899,13 +9899,13 @@
           <t xml:space="preserve">A personal history part that includes a change from a less desired behaviour pattern to a more desired behaviour pattern followed by a temporary reversion to the previous behaviour pattern. </t>
         </is>
       </c>
-      <c r="D171" s="2" t="inlineStr">
+      <c r="D171" s="2" t="n"/>
+      <c r="E171" s="2" t="n"/>
+      <c r="F171" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E171" s="2" t="n"/>
-      <c r="F171" s="2" t="n"/>
       <c r="G171" s="2" t="n"/>
       <c r="H171" s="2" t="n"/>
       <c r="I171" s="2" t="n"/>
@@ -9954,13 +9954,13 @@
           <t xml:space="preserve">A personal history part that includes experience of events that influence behaviour. </t>
         </is>
       </c>
-      <c r="D172" s="2" t="inlineStr">
+      <c r="D172" s="2" t="n"/>
+      <c r="E172" s="2" t="n"/>
+      <c r="F172" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E172" s="2" t="n"/>
-      <c r="F172" s="2" t="n"/>
       <c r="G172" s="2" t="n"/>
       <c r="H172" s="2" t="n"/>
       <c r="I172" s="2" t="n"/>
@@ -10009,13 +10009,13 @@
           <t>A personal history part of exposure to an intervention targeting the same outcome as the current intervention.</t>
         </is>
       </c>
-      <c r="D173" s="2" t="inlineStr">
+      <c r="D173" s="2" t="n"/>
+      <c r="E173" s="2" t="n"/>
+      <c r="F173" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E173" s="2" t="n"/>
-      <c r="F173" s="2" t="n"/>
       <c r="G173" s="2" t="n"/>
       <c r="H173" s="2" t="n"/>
       <c r="I173" s="2" t="n"/>
@@ -10064,13 +10064,13 @@
           <t>A personal history part  that includes exposure to a prior intervention targeting the same outcome behaviour as the current intervention.</t>
         </is>
       </c>
-      <c r="D174" s="2" t="inlineStr">
+      <c r="D174" s="2" t="n"/>
+      <c r="E174" s="2" t="n"/>
+      <c r="F174" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E174" s="2" t="n"/>
-      <c r="F174" s="2" t="n"/>
       <c r="G174" s="2" t="n"/>
       <c r="H174" s="2" t="n"/>
       <c r="I174" s="2" t="n"/>
@@ -10119,13 +10119,13 @@
           <t>A personal history part that includes exposure to the same intervention as the current intervention.</t>
         </is>
       </c>
-      <c r="D175" s="2" t="inlineStr">
+      <c r="D175" s="2" t="n"/>
+      <c r="E175" s="2" t="n"/>
+      <c r="F175" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E175" s="2" t="n"/>
-      <c r="F175" s="2" t="n"/>
       <c r="G175" s="2" t="n"/>
       <c r="H175" s="2" t="n"/>
       <c r="I175" s="2" t="n"/>
@@ -10178,17 +10178,17 @@
           <t>A process that is part of a personal history.</t>
         </is>
       </c>
-      <c r="D176" s="2" t="inlineStr">
+      <c r="D176" s="2" t="n"/>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>'process' and 'part of' some 'personal history'</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="E176" s="2" t="inlineStr">
-        <is>
-          <t>'process' and 'part of' some 'personal history'</t>
-        </is>
-      </c>
-      <c r="F176" s="2" t="n"/>
       <c r="G176" s="2" t="n"/>
       <c r="H176" s="2" t="n"/>
       <c r="I176" s="2" t="n"/>
@@ -10229,13 +10229,13 @@
           <t xml:space="preserve">A personal history part  that includes exposure to one or more interventions. </t>
         </is>
       </c>
-      <c r="D177" s="2" t="inlineStr">
+      <c r="D177" s="2" t="n"/>
+      <c r="E177" s="2" t="n"/>
+      <c r="F177" s="2" t="inlineStr">
         <is>
           <t>personal history part</t>
         </is>
       </c>
-      <c r="E177" s="2" t="n"/>
-      <c r="F177" s="2" t="n"/>
       <c r="G177" s="2" t="n"/>
       <c r="H177" s="2" t="n"/>
       <c r="I177" s="2" t="n"/>
@@ -10284,20 +10284,20 @@
           <t>An attribute reflecting a person's mental dispositions, mental processes or capabilities.</t>
         </is>
       </c>
-      <c r="D178" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="D178" s="2" t="n"/>
       <c r="E178" s="2" t="n"/>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>low motivation to quit,  low self efficacy for physical activity, negative attitudes to healthy eating, contemplation stage of change, low numeracy</t>
+          <t>personal attribute</t>
         </is>
       </c>
       <c r="G178" s="2" t="n"/>
       <c r="H178" s="2" t="n"/>
-      <c r="I178" s="2" t="n"/>
+      <c r="I178" s="2" t="inlineStr">
+        <is>
+          <t>low motivation to quit,  low self efficacy for physical activity, negative attitudes to healthy eating, contemplation stage of change, low numeracy</t>
+        </is>
+      </c>
       <c r="J178" s="2" t="n"/>
       <c r="K178" s="2" t="inlineStr">
         <is>
@@ -10345,18 +10345,18 @@
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
+          <t>A role can be assigned without being realised. A person realises a role by doing something.</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="n"/>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
           <t>role</t>
         </is>
       </c>
-      <c r="E179" s="2" t="n"/>
-      <c r="F179" s="2" t="n"/>
       <c r="G179" s="2" t="n"/>
       <c r="H179" s="2" t="n"/>
-      <c r="I179" s="2" t="inlineStr">
-        <is>
-          <t>A role can be assigned without being realised. A person realises a role by doing something.</t>
-        </is>
-      </c>
+      <c r="I179" s="2" t="n"/>
       <c r="J179" s="2" t="inlineStr">
         <is>
           <t>A role can be assigned without being realised. A person realises a role by doing something.</t>
@@ -10398,20 +10398,20 @@
           <t>A disposition to undergo undesirable change in response to exposure to another entity.</t>
         </is>
       </c>
-      <c r="D180" s="2" t="inlineStr">
-        <is>
-          <t>disposition</t>
-        </is>
-      </c>
+      <c r="D180" s="2" t="n"/>
       <c r="E180" s="2" t="n"/>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>susceptibility to addiction, vulnerability to depression</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="G180" s="2" t="n"/>
       <c r="H180" s="2" t="n"/>
-      <c r="I180" s="2" t="n"/>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>susceptibility to addiction, vulnerability to depression</t>
+        </is>
+      </c>
       <c r="J180" s="2" t="n"/>
       <c r="K180" s="2" t="inlineStr">
         <is>
@@ -10457,13 +10457,13 @@
           <t>A personal vulnerability towards performing a behaviour that causes net harm.</t>
         </is>
       </c>
-      <c r="D181" s="2" t="inlineStr">
+      <c r="D181" s="2" t="n"/>
+      <c r="E181" s="2" t="n"/>
+      <c r="F181" s="2" t="inlineStr">
         <is>
           <t>personal vulnerability</t>
         </is>
       </c>
-      <c r="E181" s="2" t="n"/>
-      <c r="F181" s="2" t="n"/>
       <c r="G181" s="2" t="n"/>
       <c r="H181" s="2" t="inlineStr">
         <is>
@@ -10516,13 +10516,13 @@
           <t>A geographic location in which a person resides.</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
+      <c r="D182" s="2" t="n"/>
+      <c r="E182" s="2" t="n"/>
+      <c r="F182" s="2" t="inlineStr">
         <is>
           <t>geographic location</t>
         </is>
       </c>
-      <c r="E182" s="2" t="n"/>
-      <c r="F182" s="2" t="n"/>
       <c r="G182" s="2" t="n"/>
       <c r="H182" s="2" t="n"/>
       <c r="I182" s="2" t="n"/>
@@ -10571,7 +10571,7 @@
           <t>An insured party role that inheres in a person who participates in the creation of the insurance contract and is eligible to receive benefits as specified by the insurance contract.</t>
         </is>
       </c>
-      <c r="D183" t="inlineStr">
+      <c r="F183" t="inlineStr">
         <is>
           <t>insured party role</t>
         </is>
@@ -10613,21 +10613,21 @@
           <t xml:space="preserve">A data item that is about the number or extent of something in a population. </t>
         </is>
       </c>
-      <c r="D184" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
+      <c r="D184" s="2" t="n"/>
       <c r="E184" s="2" t="n"/>
       <c r="F184" s="2" t="inlineStr">
         <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="n"/>
+      <c r="H184" s="2" t="n"/>
+      <c r="I184" s="2" t="inlineStr">
+        <is>
           <t>Percentage of highly educated individuals in a population. 
 Mean age in a population.</t>
         </is>
       </c>
-      <c r="G184" s="2" t="n"/>
-      <c r="H184" s="2" t="n"/>
-      <c r="I184" s="2" t="n"/>
       <c r="J184" s="2" t="n"/>
       <c r="K184" s="2" t="n"/>
       <c r="L184" s="2" t="n"/>
@@ -10661,13 +10661,13 @@
           <t>A student or trainee role realised by  currently learning at an initial level of organised instruction, primarily to familiarise the bearer to the school-type environment.</t>
         </is>
       </c>
-      <c r="D185" s="2" t="inlineStr">
+      <c r="D185" s="2" t="n"/>
+      <c r="E185" s="2" t="n"/>
+      <c r="F185" s="2" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E185" s="2" t="n"/>
-      <c r="F185" s="2" t="n"/>
       <c r="G185" s="2" t="n"/>
       <c r="H185" s="2" t="n"/>
       <c r="I185" s="2" t="n"/>
@@ -10716,13 +10716,13 @@
           <t>A &lt;disposition&gt; that decreases the likelihood of engaging with harmful behaviour.</t>
         </is>
       </c>
-      <c r="D186" s="2" t="inlineStr">
+      <c r="D186" s="2" t="n"/>
+      <c r="E186" s="2" t="n"/>
+      <c r="F186" s="2" t="inlineStr">
         <is>
           <t>disposition</t>
         </is>
       </c>
-      <c r="E186" s="2" t="n"/>
-      <c r="F186" s="2" t="n"/>
       <c r="G186" s="2" t="n"/>
       <c r="H186" s="2" t="n"/>
       <c r="I186" s="2" t="n"/>
@@ -10771,7 +10771,7 @@
           <t>A specifically dependent continuant that, in contrast to roles and dispositions, does not require any further process in order to be realized.</t>
         </is>
       </c>
-      <c r="D187" t="inlineStr">
+      <c r="F187" t="inlineStr">
         <is>
           <t>specifically dependent continuant</t>
         </is>
@@ -10803,20 +10803,20 @@
           <t>A data item about the number of units of a valuable material resource possessed by a person.</t>
         </is>
       </c>
-      <c r="D188" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
+      <c r="D188" s="2" t="n"/>
       <c r="E188" s="2" t="n"/>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>12 acres, a flock of 20 goats</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="G188" s="2" t="n"/>
       <c r="H188" s="2" t="n"/>
-      <c r="I188" s="2" t="n"/>
+      <c r="I188" s="2" t="inlineStr">
+        <is>
+          <t>12 acres, a flock of 20 goats</t>
+        </is>
+      </c>
       <c r="J188" s="2" t="n"/>
       <c r="K188" s="2" t="inlineStr">
         <is>
@@ -10866,13 +10866,13 @@
           <t>A sexual orientation that is not exclusively homosexual or heterosexual, or of a person who does not identify with heterosexual, homosexual or bisexual labels.</t>
         </is>
       </c>
-      <c r="D189" s="2" t="inlineStr">
+      <c r="D189" s="2" t="n"/>
+      <c r="E189" s="2" t="n"/>
+      <c r="F189" s="2" t="inlineStr">
         <is>
           <t>sexual orientation</t>
         </is>
       </c>
-      <c r="E189" s="2" t="n"/>
-      <c r="F189" s="2" t="n"/>
       <c r="G189" s="2" t="inlineStr">
         <is>
           <t>NCIT_C155691</t>
@@ -10925,13 +10925,13 @@
           <t xml:space="preserve">A self-identity as being in the process of exploring one's sexual orientation. </t>
         </is>
       </c>
-      <c r="D190" s="2" t="inlineStr">
+      <c r="D190" s="2" t="n"/>
+      <c r="E190" s="2" t="n"/>
+      <c r="F190" s="2" t="inlineStr">
         <is>
           <t>self-identity</t>
         </is>
       </c>
-      <c r="E190" s="2" t="n"/>
-      <c r="F190" s="2" t="n"/>
       <c r="G190" s="2" t="inlineStr">
         <is>
           <t>NCIT_C155692</t>
@@ -10984,13 +10984,13 @@
           <t>A personal attribute that is whether an individual is connected or associated with another through romantic attraction or marriage.</t>
         </is>
       </c>
-      <c r="D191" s="2" t="inlineStr">
+      <c r="D191" s="2" t="n"/>
+      <c r="E191" s="2" t="n"/>
+      <c r="F191" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E191" s="2" t="n"/>
-      <c r="F191" s="2" t="n"/>
       <c r="G191" s="2" t="n"/>
       <c r="H191" s="2" t="n"/>
       <c r="I191" s="2" t="n"/>
@@ -11039,24 +11039,24 @@
           <t xml:space="preserve">A personal attribute that is belonging to a group that is characterised by the practice of a common religion by the group members. </t>
         </is>
       </c>
-      <c r="D192" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="D192" s="2" t="n"/>
       <c r="E192" s="2" t="n"/>
       <c r="F192" s="2" t="inlineStr">
         <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>NCIT_C103282</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="n"/>
+      <c r="I192" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve"> Religion Baptist 157 (37.0%) 163 (40.3%) Catholic 54 (12.7%) 60 (14.9%) Muslim 39 (9.2%) </t>
         </is>
       </c>
-      <c r="G192" s="2" t="inlineStr">
-        <is>
-          <t>NCIT_C103282</t>
-        </is>
-      </c>
-      <c r="H192" s="2" t="n"/>
-      <c r="I192" s="2" t="n"/>
       <c r="J192" s="2" t="inlineStr">
         <is>
           <t>presented in aggregated form as proportion/percentage belonging to a specified religious group</t>
@@ -11106,13 +11106,13 @@
           <t>A person who lives in a residential facility they do not own without paying an agreed sum of money to the residential facility owner.</t>
         </is>
       </c>
-      <c r="D193" s="2" t="inlineStr">
+      <c r="D193" s="2" t="n"/>
+      <c r="E193" s="2" t="n"/>
+      <c r="F193" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E193" s="2" t="n"/>
-      <c r="F193" s="2" t="n"/>
       <c r="G193" s="2" t="n"/>
       <c r="H193" s="2" t="n"/>
       <c r="I193" s="2" t="n"/>
@@ -11161,20 +11161,20 @@
           <t>A rent-free occupier who lives in the residential facility without the agreement of the residential facility owner.</t>
         </is>
       </c>
-      <c r="D194" s="2" t="inlineStr">
-        <is>
-          <t>rent-free occupier</t>
-        </is>
-      </c>
+      <c r="D194" s="2" t="n"/>
       <c r="E194" s="2" t="n"/>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>squatters</t>
+          <t>rent-free occupier</t>
         </is>
       </c>
       <c r="G194" s="2" t="n"/>
       <c r="H194" s="2" t="n"/>
-      <c r="I194" s="2" t="n"/>
+      <c r="I194" s="2" t="inlineStr">
+        <is>
+          <t>squatters</t>
+        </is>
+      </c>
       <c r="J194" s="2" t="n"/>
       <c r="K194" s="2" t="inlineStr">
         <is>
@@ -11220,13 +11220,13 @@
           <t>A person who lives in a residential facility they do not own in return for paying an agreed sum of money to the residential facility owner</t>
         </is>
       </c>
-      <c r="D195" s="2" t="inlineStr">
+      <c r="D195" s="2" t="n"/>
+      <c r="E195" s="2" t="n"/>
+      <c r="F195" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E195" s="2" t="n"/>
-      <c r="F195" s="2" t="n"/>
       <c r="G195" s="2" t="n"/>
       <c r="H195" s="2" t="n"/>
       <c r="I195" s="2" t="n"/>
@@ -11275,20 +11275,20 @@
           <t>A renter who lives in a residential facility where the residential facility owner decides who can live in the residential facility based on their perceived social or economic needs.</t>
         </is>
       </c>
-      <c r="D196" s="2" t="inlineStr">
-        <is>
-          <t>renter</t>
-        </is>
-      </c>
+      <c r="D196" s="2" t="n"/>
       <c r="E196" s="2" t="n"/>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>renters living in "public housing"[US], council housing [UK], housing association properties, non-profit organisation, alms house occupier</t>
+          <t>renter</t>
         </is>
       </c>
       <c r="G196" s="2" t="n"/>
       <c r="H196" s="2" t="n"/>
-      <c r="I196" s="2" t="n"/>
+      <c r="I196" s="2" t="inlineStr">
+        <is>
+          <t>renters living in "public housing"[US], council housing [UK], housing association properties, non-profit organisation, alms house occupier</t>
+        </is>
+      </c>
       <c r="J196" s="2" t="n"/>
       <c r="K196" s="2" t="inlineStr">
         <is>
@@ -11334,13 +11334,13 @@
           <t>An owner of a residential facility.</t>
         </is>
       </c>
-      <c r="D197" s="2" t="inlineStr">
+      <c r="D197" s="2" t="n"/>
+      <c r="E197" s="2" t="n"/>
+      <c r="F197" s="2" t="inlineStr">
         <is>
           <t>owner</t>
         </is>
       </c>
-      <c r="E197" s="2" t="n"/>
-      <c r="F197" s="2" t="n"/>
       <c r="G197" s="2" t="n"/>
       <c r="H197" s="2" t="n"/>
       <c r="I197" s="2" t="n"/>
@@ -11389,13 +11389,13 @@
           <t>A personal attribute inhering in a person who previously bore a role realised in an employment process but has withdrawn from that employment process, having concluded their working or professional career.</t>
         </is>
       </c>
-      <c r="D198" s="2" t="inlineStr">
+      <c r="D198" s="2" t="n"/>
+      <c r="E198" s="2" t="n"/>
+      <c r="F198" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E198" s="2" t="n"/>
-      <c r="F198" s="2" t="n"/>
       <c r="G198" s="2" t="n"/>
       <c r="H198" s="2" t="n"/>
       <c r="I198" s="2" t="n"/>
@@ -11444,7 +11444,7 @@
           <t>b is a role means: b is a realizable entity and b exists because there is some single bearer that is in some special physical, social, or institutional set of circumstances in which this bearer does not have to beand b is not such that, if it ceases to exist, then the physical make-up of the bearer is thereby changed.</t>
         </is>
       </c>
-      <c r="D199" t="inlineStr">
+      <c r="F199" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
@@ -11476,13 +11476,13 @@
           <t xml:space="preserve">A student or trainee role realised by currently learning at a primary or secondary education level in an institutional, organised setting. </t>
         </is>
       </c>
-      <c r="D200" s="3" t="inlineStr">
+      <c r="D200" s="3" t="n"/>
+      <c r="E200" s="3" t="n"/>
+      <c r="F200" s="3" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E200" s="3" t="n"/>
-      <c r="F200" s="3" t="n"/>
       <c r="G200" s="3" t="n"/>
       <c r="H200" s="3" t="n"/>
       <c r="I200" s="3" t="n"/>
@@ -11531,13 +11531,13 @@
           <t xml:space="preserve">A student or trainee role realised by currently learning at a primary or secondary education level in an institutional, organised setting. </t>
         </is>
       </c>
-      <c r="D201" s="2" t="inlineStr">
+      <c r="D201" s="2" t="n"/>
+      <c r="E201" s="2" t="n"/>
+      <c r="F201" s="2" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E201" s="2" t="n"/>
-      <c r="F201" s="2" t="n"/>
       <c r="G201" s="2" t="n"/>
       <c r="H201" s="2" t="n"/>
       <c r="I201" s="2" t="n"/>
@@ -11586,13 +11586,13 @@
           <t>A person who has at least one parent who is an immigrant.</t>
         </is>
       </c>
-      <c r="D202" s="2" t="inlineStr">
+      <c r="D202" s="2" t="n"/>
+      <c r="E202" s="2" t="n"/>
+      <c r="F202" s="2" t="inlineStr">
         <is>
           <t>person</t>
         </is>
       </c>
-      <c r="E202" s="2" t="n"/>
-      <c r="F202" s="2" t="n"/>
       <c r="G202" s="2" t="n"/>
       <c r="H202" s="2" t="n"/>
       <c r="I202" s="2" t="n"/>
@@ -11641,13 +11641,13 @@
           <t>An employment status realised by a person earning income directly from customers, clients, or other organisations rather than as a specified salary or wages from an employer.</t>
         </is>
       </c>
-      <c r="D203" s="2" t="inlineStr">
+      <c r="D203" s="2" t="n"/>
+      <c r="E203" s="2" t="n"/>
+      <c r="F203" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E203" s="2" t="n"/>
-      <c r="F203" s="2" t="n"/>
       <c r="G203" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">NCIT_C116000 </t>
@@ -11704,7 +11704,7 @@
           <t>An identity that a person has about themselves.</t>
         </is>
       </c>
-      <c r="D204" t="inlineStr">
+      <c r="F204" t="inlineStr">
         <is>
           <t>identity</t>
         </is>
@@ -11736,13 +11736,13 @@
           <t xml:space="preserve">A personal attribute that is the pattern of a person's emotional, romantic and/or sexual attractions. </t>
         </is>
       </c>
-      <c r="D205" s="2" t="inlineStr">
+      <c r="D205" s="2" t="n"/>
+      <c r="E205" s="2" t="n"/>
+      <c r="F205" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E205" s="2" t="n"/>
-      <c r="F205" s="2" t="n"/>
       <c r="G205" s="2" t="inlineStr">
         <is>
           <t>NCIT_C84361</t>
@@ -11795,13 +11795,13 @@
           <t>A family member with whom the subject shares a parent.</t>
         </is>
       </c>
-      <c r="D206" s="2" t="inlineStr">
+      <c r="D206" s="2" t="n"/>
+      <c r="E206" s="2" t="n"/>
+      <c r="F206" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E206" s="2" t="n"/>
-      <c r="F206" s="2" t="n"/>
       <c r="G206" s="2" t="n"/>
       <c r="H206" s="2" t="n"/>
       <c r="I206" s="2" t="n"/>
@@ -11851,13 +11851,13 @@
           <t>A relationship status where the individual is not in a relationship with another person.</t>
         </is>
       </c>
-      <c r="D207" s="2" t="inlineStr">
+      <c r="D207" s="2" t="n"/>
+      <c r="E207" s="2" t="n"/>
+      <c r="F207" s="2" t="inlineStr">
         <is>
           <t>relationship status</t>
         </is>
       </c>
-      <c r="E207" s="2" t="n"/>
-      <c r="F207" s="2" t="n"/>
       <c r="G207" s="2" t="n"/>
       <c r="H207" s="2" t="n"/>
       <c r="I207" s="2" t="n"/>
@@ -11906,13 +11906,13 @@
           <t>A personal attribute that holds within a given situation.</t>
         </is>
       </c>
-      <c r="D208" s="2" t="inlineStr">
+      <c r="D208" s="2" t="n"/>
+      <c r="E208" s="2" t="n"/>
+      <c r="F208" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E208" s="2" t="n"/>
-      <c r="F208" s="2" t="n"/>
       <c r="G208" s="2" t="n"/>
       <c r="H208" s="2" t="n"/>
       <c r="I208" s="2" t="n"/>
@@ -11953,13 +11953,13 @@
           <t>A social grouping that identifies as such and sometimes acts collectively.</t>
         </is>
       </c>
-      <c r="D209" s="2" t="inlineStr">
+      <c r="D209" s="2" t="n"/>
+      <c r="E209" s="2" t="n"/>
+      <c r="F209" s="2" t="inlineStr">
         <is>
           <t>social grouping</t>
         </is>
       </c>
-      <c r="E209" s="2" t="n"/>
-      <c r="F209" s="2" t="n"/>
       <c r="G209" s="2" t="n"/>
       <c r="H209" s="2" t="n"/>
       <c r="I209" s="2" t="n"/>
@@ -12000,13 +12000,13 @@
           <t>A human population who share some common attribute that involves some form of social interaction.</t>
         </is>
       </c>
-      <c r="D210" s="2" t="inlineStr">
+      <c r="D210" s="2" t="n"/>
+      <c r="E210" s="2" t="n"/>
+      <c r="F210" s="2" t="inlineStr">
         <is>
           <t>human population</t>
         </is>
       </c>
-      <c r="E210" s="2" t="n"/>
-      <c r="F210" s="2" t="n"/>
       <c r="G210" s="2" t="n"/>
       <c r="H210" s="2" t="n"/>
       <c r="I210" s="2" t="n"/>
@@ -12051,13 +12051,13 @@
           <t>A personal role that is realised in human social processes.</t>
         </is>
       </c>
-      <c r="D211" s="2" t="inlineStr">
+      <c r="D211" s="2" t="n"/>
+      <c r="E211" s="2" t="n"/>
+      <c r="F211" s="2" t="inlineStr">
         <is>
           <t>personal role</t>
         </is>
       </c>
-      <c r="E211" s="2" t="n"/>
-      <c r="F211" s="2" t="n"/>
       <c r="G211" s="2" t="n"/>
       <c r="H211" s="2" t="n"/>
       <c r="I211" s="2" t="n"/>
@@ -12098,13 +12098,13 @@
           <t>A &lt;personal attribute&gt; that, together with other attributes, characterises a person’s position in society.</t>
         </is>
       </c>
-      <c r="D212" s="2" t="inlineStr">
+      <c r="D212" s="2" t="n"/>
+      <c r="E212" s="2" t="n"/>
+      <c r="F212" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E212" s="2" t="n"/>
-      <c r="F212" s="2" t="n"/>
       <c r="G212" s="2" t="n"/>
       <c r="H212" s="2" t="n"/>
       <c r="I212" s="2" t="n"/>
@@ -12149,13 +12149,13 @@
           <t>A personal attribute reflecting a person's economic and social position in relation to others</t>
         </is>
       </c>
-      <c r="D213" s="2" t="inlineStr">
+      <c r="D213" s="2" t="n"/>
+      <c r="E213" s="2" t="n"/>
+      <c r="F213" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E213" s="2" t="n"/>
-      <c r="F213" s="2" t="n"/>
       <c r="G213" s="2" t="inlineStr">
         <is>
           <t>OPMI:0000121</t>
@@ -12173,7 +12173,7 @@
       <c r="M213" s="2" t="n"/>
       <c r="N213" s="2" t="inlineStr">
         <is>
-          <t>attribute</t>
+          <t>attributes</t>
         </is>
       </c>
       <c r="O213" s="2" t="n"/>
@@ -12208,13 +12208,13 @@
           <t xml:space="preserve">A data item about a score on a measure of a person's socioeconomic position, calculated by combining information about the number of years of education completed, their individual or household income, their current occupation or the industry in which they work or family size or household. </t>
         </is>
       </c>
-      <c r="D214" s="2" t="inlineStr">
+      <c r="D214" s="2" t="n"/>
+      <c r="E214" s="2" t="n"/>
+      <c r="F214" s="2" t="inlineStr">
         <is>
           <t>data item</t>
         </is>
       </c>
-      <c r="E214" s="2" t="n"/>
-      <c r="F214" s="2" t="n"/>
       <c r="G214" s="2" t="n"/>
       <c r="H214" s="2" t="n"/>
       <c r="I214" s="2" t="n"/>
@@ -12267,20 +12267,20 @@
           <t xml:space="preserve">A  data item about a category assigned to a person based on an assessment of a score calculated from various measures of their income, education, occupation, family size or household. </t>
         </is>
       </c>
-      <c r="D215" s="3" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
+      <c r="D215" s="3" t="n"/>
       <c r="E215" s="3" t="n"/>
       <c r="F215" s="3" t="inlineStr">
         <is>
-          <t>Semi-routine and routine occupations, blue collar occupations</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="G215" s="3" t="n"/>
       <c r="H215" s="3" t="n"/>
-      <c r="I215" s="3" t="n"/>
+      <c r="I215" s="3" t="inlineStr">
+        <is>
+          <t>Semi-routine and routine occupations, blue collar occupations</t>
+        </is>
+      </c>
       <c r="J215" s="3" t="n"/>
       <c r="K215" s="3" t="inlineStr">
         <is>
@@ -12330,13 +12330,13 @@
           <t>A personal attribute inhering in a person by virtue of that person not bearing a role realised in an employment process, due to being a homemaker whose work includes caring for children.</t>
         </is>
       </c>
-      <c r="D216" s="2" t="inlineStr">
+      <c r="D216" s="2" t="n"/>
+      <c r="E216" s="2" t="n"/>
+      <c r="F216" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E216" s="2" t="n"/>
-      <c r="F216" s="2" t="n"/>
       <c r="G216" s="2" t="inlineStr">
         <is>
           <t>NCIT_C148253</t>
@@ -12389,13 +12389,13 @@
           <t>A parent in a parent-child relationship established by the parent's subsequent marriage to one of the child's original biological or legal parents.</t>
         </is>
       </c>
-      <c r="D217" s="2" t="inlineStr">
+      <c r="D217" s="2" t="n"/>
+      <c r="E217" s="2" t="n"/>
+      <c r="F217" s="2" t="inlineStr">
         <is>
           <t>parent</t>
         </is>
       </c>
-      <c r="E217" s="2" t="n"/>
-      <c r="F217" s="2" t="n"/>
       <c r="G217" s="2" t="inlineStr">
         <is>
           <t>NCIT:C166116</t>
@@ -12448,13 +12448,13 @@
           <t>A sibling who is the child of one's step-parent.</t>
         </is>
       </c>
-      <c r="D218" s="2" t="inlineStr">
+      <c r="D218" s="2" t="n"/>
+      <c r="E218" s="2" t="n"/>
+      <c r="F218" s="2" t="inlineStr">
         <is>
           <t>sibling</t>
         </is>
       </c>
-      <c r="E218" s="2" t="n"/>
-      <c r="F218" s="2" t="n"/>
       <c r="G218" s="2" t="n"/>
       <c r="H218" s="2" t="n"/>
       <c r="I218" s="2" t="n"/>
@@ -12503,13 +12503,13 @@
           <t>A step-sibling who is male gender.</t>
         </is>
       </c>
-      <c r="D219" s="2" t="inlineStr">
+      <c r="D219" s="2" t="n"/>
+      <c r="E219" s="2" t="n"/>
+      <c r="F219" s="2" t="inlineStr">
         <is>
           <t>step-sibling</t>
         </is>
       </c>
-      <c r="E219" s="2" t="n"/>
-      <c r="F219" s="2" t="n"/>
       <c r="G219" s="2" t="n"/>
       <c r="H219" s="2" t="n"/>
       <c r="I219" s="2" t="n"/>
@@ -12558,13 +12558,13 @@
           <t>A child relation in a parent-child relationship established by the parent's subsequent marriage to one of the child's original biological or legal parents.</t>
         </is>
       </c>
-      <c r="D220" s="2" t="inlineStr">
+      <c r="D220" s="2" t="n"/>
+      <c r="E220" s="2" t="n"/>
+      <c r="F220" s="2" t="inlineStr">
         <is>
           <t>child relation</t>
         </is>
       </c>
-      <c r="E220" s="2" t="n"/>
-      <c r="F220" s="2" t="n"/>
       <c r="G220" s="2" t="n"/>
       <c r="H220" s="2" t="n"/>
       <c r="I220" s="2" t="n"/>
@@ -12613,13 +12613,13 @@
           <t>A stepchild who is female gender.</t>
         </is>
       </c>
-      <c r="D221" s="2" t="inlineStr">
+      <c r="D221" s="2" t="n"/>
+      <c r="E221" s="2" t="n"/>
+      <c r="F221" s="2" t="inlineStr">
         <is>
           <t>stepchild</t>
         </is>
       </c>
-      <c r="E221" s="2" t="n"/>
-      <c r="F221" s="2" t="n"/>
       <c r="G221" s="2" t="n"/>
       <c r="H221" s="2" t="n"/>
       <c r="I221" s="2" t="n"/>
@@ -12668,13 +12668,13 @@
           <t>A step-parent who is male gender.</t>
         </is>
       </c>
-      <c r="D222" s="2" t="inlineStr">
+      <c r="D222" s="2" t="n"/>
+      <c r="E222" s="2" t="n"/>
+      <c r="F222" s="2" t="inlineStr">
         <is>
           <t>step-parent</t>
         </is>
       </c>
-      <c r="E222" s="2" t="n"/>
-      <c r="F222" s="2" t="n"/>
       <c r="G222" s="2" t="n"/>
       <c r="H222" s="2" t="n"/>
       <c r="I222" s="2" t="n"/>
@@ -12723,13 +12723,13 @@
           <t>A step-parent who is female gender.</t>
         </is>
       </c>
-      <c r="D223" s="2" t="inlineStr">
+      <c r="D223" s="2" t="n"/>
+      <c r="E223" s="2" t="n"/>
+      <c r="F223" s="2" t="inlineStr">
         <is>
           <t>step-parent</t>
         </is>
       </c>
-      <c r="E223" s="2" t="n"/>
-      <c r="F223" s="2" t="n"/>
       <c r="G223" s="2" t="n"/>
       <c r="H223" s="2" t="n"/>
       <c r="I223" s="2" t="n"/>
@@ -12778,13 +12778,13 @@
           <t>A step-sibling who is female gender.</t>
         </is>
       </c>
-      <c r="D224" s="2" t="inlineStr">
+      <c r="D224" s="2" t="n"/>
+      <c r="E224" s="2" t="n"/>
+      <c r="F224" s="2" t="inlineStr">
         <is>
           <t>step-sibling</t>
         </is>
       </c>
-      <c r="E224" s="2" t="n"/>
-      <c r="F224" s="2" t="n"/>
       <c r="G224" s="2" t="n"/>
       <c r="H224" s="2" t="n"/>
       <c r="I224" s="2" t="n"/>
@@ -12833,13 +12833,13 @@
           <t>A stepchild who is male gender.</t>
         </is>
       </c>
-      <c r="D225" s="2" t="inlineStr">
+      <c r="D225" s="2" t="n"/>
+      <c r="E225" s="2" t="n"/>
+      <c r="F225" s="2" t="inlineStr">
         <is>
           <t>stepchild</t>
         </is>
       </c>
-      <c r="E225" s="2" t="n"/>
-      <c r="F225" s="2" t="n"/>
       <c r="G225" s="2" t="n"/>
       <c r="H225" s="2" t="n"/>
       <c r="I225" s="2" t="n"/>
@@ -12888,13 +12888,13 @@
           <t>A role which inheres in a person and is realised by being enrolled in an educational institution or a formal programme of professional training.</t>
         </is>
       </c>
-      <c r="D226" s="2" t="inlineStr">
+      <c r="D226" s="2" t="n"/>
+      <c r="E226" s="2" t="n"/>
+      <c r="F226" s="2" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="E226" s="2" t="n"/>
-      <c r="F226" s="2" t="n"/>
       <c r="G226" s="2" t="n"/>
       <c r="H226" s="2" t="n"/>
       <c r="I226" s="2" t="n"/>
@@ -12943,7 +12943,7 @@
           <t>A person between 13 and 19 years of age.</t>
         </is>
       </c>
-      <c r="D227" t="inlineStr">
+      <c r="F227" t="inlineStr">
         <is>
           <t>person</t>
         </is>
@@ -12985,13 +12985,13 @@
           <t>A student or trainee role that is currently learning the curriculum material of vocational programme, normally in preparation for employment in a trade, job or profession.</t>
         </is>
       </c>
-      <c r="D228" s="2" t="inlineStr">
+      <c r="D228" s="2" t="n"/>
+      <c r="E228" s="2" t="n"/>
+      <c r="F228" s="2" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E228" s="2" t="n"/>
-      <c r="F228" s="2" t="n"/>
       <c r="G228" s="2" t="n"/>
       <c r="H228" s="2" t="n"/>
       <c r="I228" s="2" t="n"/>
@@ -13040,13 +13040,13 @@
           <t>A gender identity that differs from the person's assigned sex at birth.</t>
         </is>
       </c>
-      <c r="D229" s="2" t="inlineStr">
+      <c r="D229" s="2" t="n"/>
+      <c r="E229" s="2" t="n"/>
+      <c r="F229" s="2" t="inlineStr">
         <is>
           <t>gender identity</t>
         </is>
       </c>
-      <c r="E229" s="2" t="n"/>
-      <c r="F229" s="2" t="n"/>
       <c r="G229" s="2" t="inlineStr">
         <is>
           <t>GSSO:000096</t>
@@ -13099,13 +13099,13 @@
           <t xml:space="preserve">One of two siblings who resulted from the same pregnancy. </t>
         </is>
       </c>
-      <c r="D230" s="2" t="inlineStr">
+      <c r="D230" s="2" t="n"/>
+      <c r="E230" s="2" t="n"/>
+      <c r="F230" s="2" t="inlineStr">
         <is>
           <t>sibling</t>
         </is>
       </c>
-      <c r="E230" s="2" t="n"/>
-      <c r="F230" s="2" t="n"/>
       <c r="G230" s="2" t="n"/>
       <c r="H230" s="2" t="n"/>
       <c r="I230" s="2" t="n"/>
@@ -13154,13 +13154,13 @@
           <t>A situational personal attribute in which a person has not thought about enacting a behaviour.</t>
         </is>
       </c>
-      <c r="D231" s="2" t="inlineStr">
+      <c r="D231" s="2" t="n"/>
+      <c r="E231" s="2" t="n"/>
+      <c r="F231" s="2" t="inlineStr">
         <is>
           <t>situational personal attribute</t>
         </is>
       </c>
-      <c r="E231" s="2" t="n"/>
-      <c r="F231" s="2" t="n"/>
       <c r="G231" s="2" t="n"/>
       <c r="H231" s="2" t="n"/>
       <c r="I231" s="2" t="n"/>
@@ -13209,13 +13209,13 @@
           <t>A family member who is the brother of one's parent.</t>
         </is>
       </c>
-      <c r="D232" s="2" t="inlineStr">
+      <c r="D232" s="2" t="n"/>
+      <c r="E232" s="2" t="n"/>
+      <c r="F232" s="2" t="inlineStr">
         <is>
           <t>family member</t>
         </is>
       </c>
-      <c r="E232" s="2" t="n"/>
-      <c r="F232" s="2" t="n"/>
       <c r="G232" s="2" t="n"/>
       <c r="H232" s="2" t="n"/>
       <c r="I232" s="2" t="n"/>
@@ -13264,13 +13264,13 @@
           <t>A situational personal attribute in which the person has thought about a behaviour but not formed an intention regarding whether to enact it.</t>
         </is>
       </c>
-      <c r="D233" s="2" t="inlineStr">
+      <c r="D233" s="2" t="n"/>
+      <c r="E233" s="2" t="n"/>
+      <c r="F233" s="2" t="inlineStr">
         <is>
           <t>situational personal attribute</t>
         </is>
       </c>
-      <c r="E233" s="2" t="n"/>
-      <c r="F233" s="2" t="n"/>
       <c r="G233" s="2" t="n"/>
       <c r="H233" s="2" t="n"/>
       <c r="I233" s="2" t="n"/>
@@ -13319,13 +13319,13 @@
           <t>A higher education student role realised by currently studying for an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D234" s="3" t="inlineStr">
+      <c r="D234" s="3" t="n"/>
+      <c r="E234" s="3" t="n"/>
+      <c r="F234" s="3" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E234" s="3" t="n"/>
-      <c r="F234" s="3" t="n"/>
       <c r="G234" s="3" t="n"/>
       <c r="H234" s="3" t="n"/>
       <c r="I234" s="3" t="n"/>
@@ -13374,13 +13374,13 @@
           <t>A higher education student role realised by currently studying for an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D235" s="2" t="inlineStr">
+      <c r="D235" s="2" t="n"/>
+      <c r="E235" s="2" t="n"/>
+      <c r="F235" s="2" t="inlineStr">
         <is>
           <t>higher education student role</t>
         </is>
       </c>
-      <c r="E235" s="2" t="n"/>
-      <c r="F235" s="2" t="n"/>
       <c r="G235" s="2" t="n"/>
       <c r="H235" s="2" t="n"/>
       <c r="I235" s="2" t="n"/>
@@ -13429,13 +13429,13 @@
           <t>An employment status in which the person is not employed or self-employed, is looking for work and able to start in paid employment.</t>
         </is>
       </c>
-      <c r="D236" s="2" t="inlineStr">
+      <c r="D236" s="2" t="n"/>
+      <c r="E236" s="2" t="n"/>
+      <c r="F236" s="2" t="inlineStr">
         <is>
           <t>employment status</t>
         </is>
       </c>
-      <c r="E236" s="2" t="n"/>
-      <c r="F236" s="2" t="n"/>
       <c r="G236" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">SDGIO_00010026 </t>
@@ -13488,13 +13488,13 @@
           <t>A personal attribute inhering in a person by virtue of that person not bearing a role realised in an employment process, due to their primary occupation being caring, without receiving a wage for it, for an adult friend or family member who, due to illness or disability, requires support in their daily life activities.</t>
         </is>
       </c>
-      <c r="D237" s="2" t="inlineStr">
+      <c r="D237" s="2" t="n"/>
+      <c r="E237" s="2" t="n"/>
+      <c r="F237" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E237" s="2" t="n"/>
-      <c r="F237" s="2" t="n"/>
       <c r="G237" s="2" t="n"/>
       <c r="H237" s="2" t="n"/>
       <c r="I237" s="2" t="n"/>
@@ -13543,24 +13543,24 @@
           <t>An object aggregate under the control of some person or organisation which confers an economic benefit to that person or organisation in an economic system.</t>
         </is>
       </c>
-      <c r="D238" s="2" t="inlineStr">
-        <is>
-          <t>object aggregate</t>
-        </is>
-      </c>
+      <c r="D238" s="2" t="n"/>
       <c r="E238" s="2" t="n"/>
       <c r="F238" s="2" t="inlineStr">
         <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
+      <c r="G238" s="2" t="inlineStr">
+        <is>
+          <t>SDGIO:00010048</t>
+        </is>
+      </c>
+      <c r="H238" s="2" t="n"/>
+      <c r="I238" s="2" t="inlineStr">
+        <is>
           <t>farmland, jewellery, livestock</t>
         </is>
       </c>
-      <c r="G238" s="2" t="inlineStr">
-        <is>
-          <t>SDGIO:00010048</t>
-        </is>
-      </c>
-      <c r="H238" s="2" t="n"/>
-      <c r="I238" s="2" t="n"/>
       <c r="J238" s="2" t="n"/>
       <c r="K238" s="2" t="inlineStr">
         <is>
@@ -13598,20 +13598,20 @@
           <t>A data item about the monetary value of a valuable material resource possessed by a person.</t>
         </is>
       </c>
-      <c r="D239" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
+      <c r="D239" s="2" t="n"/>
       <c r="E239" s="2" t="n"/>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>$400, 3000 euros</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="G239" s="2" t="n"/>
       <c r="H239" s="2" t="n"/>
-      <c r="I239" s="2" t="n"/>
+      <c r="I239" s="2" t="inlineStr">
+        <is>
+          <t>$400, 3000 euros</t>
+        </is>
+      </c>
       <c r="J239" s="2" t="n"/>
       <c r="K239" s="2" t="inlineStr">
         <is>
@@ -13661,13 +13661,13 @@
           <t>A student or trainee role realised by currently learning the curriculum material of vocational programme, normally in preparation for employment in a trade, job or profession.</t>
         </is>
       </c>
-      <c r="D240" s="3" t="inlineStr">
+      <c r="D240" s="3" t="n"/>
+      <c r="E240" s="3" t="n"/>
+      <c r="F240" s="3" t="inlineStr">
         <is>
           <t>student or trainee role</t>
         </is>
       </c>
-      <c r="E240" s="3" t="n"/>
-      <c r="F240" s="3" t="n"/>
       <c r="G240" s="3" t="n"/>
       <c r="H240" s="3" t="n"/>
       <c r="I240" s="3" t="n"/>
@@ -13716,13 +13716,13 @@
           <t>A personal attribute inhering in a person by virtue of that person working or assisting at a workplace without receiving remuneration.</t>
         </is>
       </c>
-      <c r="D241" s="2" t="inlineStr">
+      <c r="D241" s="2" t="n"/>
+      <c r="E241" s="2" t="n"/>
+      <c r="F241" s="2" t="inlineStr">
         <is>
           <t>personal attribute</t>
         </is>
       </c>
-      <c r="E241" s="2" t="n"/>
-      <c r="F241" s="2" t="n"/>
       <c r="G241" s="2" t="n"/>
       <c r="H241" s="2" t="n"/>
       <c r="I241" s="2" t="n"/>
@@ -13775,13 +13775,13 @@
           <t xml:space="preserve">A relationship status where the individual is no longer in a legally formalised marriage or civil partnership due to the death of their spouse or partner. </t>
         </is>
       </c>
-      <c r="D242" s="2" t="inlineStr">
+      <c r="D242" s="2" t="n"/>
+      <c r="E242" s="2" t="n"/>
+      <c r="F242" s="2" t="inlineStr">
         <is>
           <t>relationship status</t>
         </is>
       </c>
-      <c r="E242" s="2" t="n"/>
-      <c r="F242" s="2" t="n"/>
       <c r="G242" s="2" t="n"/>
       <c r="H242" s="2" t="n"/>
       <c r="I242" s="2" t="n"/>

</xml_diff>

<commit_message>
Update employment status in BCIO_Population.xlsx
</commit_message>
<xml_diff>
--- a/Population/BCIO_Population.xlsx
+++ b/Population/BCIO_Population.xlsx
@@ -451,32 +451,32 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Parent</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Logical definition</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Examples</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Cross-reference</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Synonyms</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Informal definition</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Logical definition</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Parent</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Cross-reference</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Synonyms</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Examples</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -556,20 +556,20 @@
           <t>A linguistic capability that is realised by following and understanding speech in the intervention language.</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">linguistic capability </t>
+        </is>
+      </c>
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">linguistic capability </t>
+          <t>Comprehend the German language</t>
         </is>
       </c>
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Comprehend the German language</t>
-        </is>
-      </c>
+      <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -615,20 +615,20 @@
           <t>A linguistic capability that is realised by reading and understanding text in the intervention language.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">linguistic capability </t>
+        </is>
+      </c>
       <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">linguistic capability </t>
+          <t>The exclusion criteria were an inability to read English</t>
         </is>
       </c>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>The exclusion criteria were an inability to read English</t>
-        </is>
-      </c>
+      <c r="I3" s="2" t="n"/>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -674,20 +674,20 @@
           <t xml:space="preserve">A linguistic capability that is realised by producing speech  in the intervention language. </t>
         </is>
       </c>
-      <c r="D4" s="2" t="n"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">linguistic capability </t>
+        </is>
+      </c>
       <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">linguistic capability </t>
+          <t>Able to speak Chinese.</t>
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Able to speak Chinese.</t>
-        </is>
-      </c>
+      <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -733,20 +733,20 @@
           <t>A linguistic capability that is realised by generating written text in the intervention language.</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">linguistic capability </t>
+        </is>
+      </c>
       <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">linguistic capability </t>
+          <t>Fluency in written English.</t>
         </is>
       </c>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Fluency in written English.</t>
-        </is>
-      </c>
+      <c r="I5" s="2" t="n"/>
       <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="inlineStr">
         <is>
@@ -792,13 +792,13 @@
           <t>A highest level of formal education qualification achieved after participating in an education process intended to result in the acquisition and development of skills and knowledge in a specialised discipline that culminated in the award of an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>highest level of formal educational qualification achieved</t>
+        </is>
+      </c>
       <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>highest level of formal educational qualification achieved</t>
-        </is>
-      </c>
+      <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>OMRSE_00002048</t>
@@ -855,13 +855,13 @@
           <t xml:space="preserve">A highest level of formal educational qualification achieved after participating in an education process devoted to advanced study and original research that led to the award of a PhD or equivalent level qualification. </t>
         </is>
       </c>
-      <c r="D7" s="2" t="n"/>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>highest level of formal educational qualification achieved</t>
+        </is>
+      </c>
       <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>highest level of formal educational qualification achieved</t>
-        </is>
-      </c>
+      <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="n"/>
@@ -914,13 +914,13 @@
           <t xml:space="preserve">A highest level of formal educational qualification achieved after participating in an education process intended to introduce very young children to a school-type environment. </t>
         </is>
       </c>
-      <c r="D8" s="2" t="n"/>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>highest level of formal educational qualification achieved</t>
+        </is>
+      </c>
       <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>highest level of formal educational qualification achieved</t>
-        </is>
-      </c>
+      <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
@@ -973,13 +973,13 @@
           <t>A highest level of formal educational qualification achieved after participating in an education process intended to result in the acquisition and development of skills and knowledge in subject areas more specialised than basic reading, writing and mathematics, with the overall goal of laying the foundation for lifelong learning and human development on which education systems may systematically expand further educational opportunities.</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n"/>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>highest level of formal educational qualification achieved</t>
+        </is>
+      </c>
       <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>highest level of formal educational qualification achieved</t>
-        </is>
-      </c>
+      <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
           <t>OMRSE_00002036</t>
@@ -1036,13 +1036,13 @@
           <t>A highest level of formal educational qualification achieved after participating in an education process which has as a prerequisite an undergraduate degree and which is intended to result in the acquisition and development of advanced academic or professional skills and knowledge in a specialised discipline, that culminated in the award of a Master's or equivalent degree.</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>highest level of formal educational qualification achieved</t>
+        </is>
+      </c>
       <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>highest level of formal educational qualification achieved</t>
-        </is>
-      </c>
+      <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
@@ -1095,13 +1095,13 @@
           <t>A highest level of formal educational qualification achieved after participating in an education process intended to result in the acquisition of fundamental skills in reading, writing and mathematics.</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n"/>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>highest level of formal educational qualification achieved</t>
+        </is>
+      </c>
       <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>highest level of formal educational qualification achieved</t>
-        </is>
-      </c>
+      <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">OMRSE_00002035  </t>
@@ -1158,11 +1158,15 @@
           <t>A highest level of formal educational qualification achieved after participating in an education process intended to result in the acquisition and development of skills and knowledge that prepare participants for tertiary education or employment.</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>highest level of formal educational qualification achieved</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>highest level of formal educational qualification achieved</t>
+          <t>graduated high school, International Baccaulaureate, A Levels</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1171,11 +1175,7 @@
         </is>
       </c>
       <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>graduated high school, International Baccaulaureate, A Levels</t>
-        </is>
-      </c>
+      <c r="I12" s="2" t="n"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
           <t>A highest level of formal educational qualification achieved that corresponds to the final stage of secondary education in most OECD countries. Instruction is often more organised along subject-matter lines than at ISCED 2 level and teachers typically need to have a higher level, or more subject-specific, qualifications than at ISCED 2. The entrance age to this level is typically 15 or 16 years. There are substantial differences in the typical duration of ISCED 3 programmes both between and within countries, typically ranging from 2 to 5 years of schooling. ISCED 3 may either be “terminal” (i.e. preparing students for direct entry into working life) and/or “preparatory” (i.e. preparing students for tertiary education).</t>
@@ -1225,13 +1225,13 @@
           <t>An adoptive sibling who is male gender.</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>adoptive sibling</t>
+        </is>
+      </c>
       <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>adoptive sibling</t>
-        </is>
-      </c>
+      <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="n"/>
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="n"/>
@@ -1280,13 +1280,13 @@
           <t xml:space="preserve">A child relation in a parent-child relationship established by a legal adoption process. </t>
         </is>
       </c>
-      <c r="D14" s="2" t="n"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>child relation</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>child relation</t>
-        </is>
-      </c>
+      <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>NCIT:C166130</t>
@@ -1339,13 +1339,13 @@
           <t>An adoptive child who is female gender.</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>adoptive child</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>adoptive child</t>
-        </is>
-      </c>
+      <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="n"/>
@@ -1394,13 +1394,13 @@
           <t>An adoptive parent who is male gender.</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>adoptive parent</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>adoptive parent</t>
-        </is>
-      </c>
+      <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
@@ -1449,13 +1449,13 @@
           <t>An adoptive parent who is female gender.</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n"/>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>adoptive parent</t>
+        </is>
+      </c>
       <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>adoptive parent</t>
-        </is>
-      </c>
+      <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="n"/>
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="n"/>
@@ -1504,13 +1504,13 @@
           <t>A parent in a parent-child relationship established by a legal adoption process.</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n"/>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>parent</t>
+        </is>
+      </c>
       <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>parent</t>
-        </is>
-      </c>
+      <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>NCIT:C166129</t>
@@ -1563,13 +1563,13 @@
           <t>A sibling with whom the subject shares a parent through a parent-child relationship established by a legal adoption process.</t>
         </is>
       </c>
-      <c r="D19" s="2" t="n"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
       <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>sibling</t>
-        </is>
-      </c>
+      <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="n"/>
@@ -1618,13 +1618,13 @@
           <t>An adoptive sibling who is female gender.</t>
         </is>
       </c>
-      <c r="D20" s="2" t="n"/>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>adoptive sibling</t>
+        </is>
+      </c>
       <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>adoptive sibling</t>
-        </is>
-      </c>
+      <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
       <c r="I20" s="2" t="n"/>
@@ -1673,13 +1673,13 @@
           <t>An adoptive child who is male gender.</t>
         </is>
       </c>
-      <c r="D21" s="2" t="n"/>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>adoptive child</t>
+        </is>
+      </c>
       <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>adoptive child</t>
-        </is>
-      </c>
+      <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="n"/>
       <c r="I21" s="2" t="n"/>
@@ -1728,7 +1728,7 @@
           <t>A person who has reached maturity.</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>person</t>
         </is>
@@ -1775,13 +1775,13 @@
           <t>A rent-free occupier who lives in the residential facility with the agreement of the residential facility owner.</t>
         </is>
       </c>
-      <c r="D23" s="2" t="n"/>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>rent-free occupier</t>
+        </is>
+      </c>
       <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>rent-free occupier</t>
-        </is>
-      </c>
+      <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
       <c r="H23" s="2" t="n"/>
       <c r="I23" s="2" t="n"/>
@@ -1830,13 +1830,13 @@
           <t xml:space="preserve">A sexual orientation of an individual who does not experience sexual attraction. </t>
         </is>
       </c>
-      <c r="D24" s="2" t="n"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>sexual orientation</t>
+        </is>
+      </c>
       <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>sexual orientation</t>
-        </is>
-      </c>
+      <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
           <t>NCIT_C155696</t>
@@ -1889,13 +1889,13 @@
           <t>A family member who is the sister of one's parent.</t>
         </is>
       </c>
-      <c r="D25" s="2" t="n"/>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>family member</t>
+        </is>
+      </c>
       <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>family member</t>
-        </is>
-      </c>
+      <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="2" t="n"/>
@@ -1944,13 +1944,13 @@
           <t>An intervention participant who is exposed to a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D26" s="2" t="n"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>intervention participant</t>
+        </is>
+      </c>
       <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>intervention participant</t>
-        </is>
-      </c>
+      <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="n"/>
@@ -1995,13 +1995,13 @@
           <t>An intervention population who are exposed to a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D27" s="2" t="n"/>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>intervention population</t>
+        </is>
+      </c>
       <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>intervention population</t>
-        </is>
-      </c>
+      <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="2" t="n"/>
@@ -2042,13 +2042,13 @@
           <t>A data item that is about the rate of individual human behaviour change.</t>
         </is>
       </c>
-      <c r="D28" s="2" t="n"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
       <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
+      <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="n"/>
@@ -2093,13 +2093,13 @@
           <t>A person who has formed an intention to enact a specified behaviour, and has enacted that behaviour.</t>
         </is>
       </c>
-      <c r="D29" s="2" t="n"/>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -2149,13 +2149,13 @@
           <t>A person who has formed an intention to enact a specified behaviour, but has not acted on this intention.</t>
         </is>
       </c>
-      <c r="D30" s="2" t="n"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="2" t="n"/>
@@ -2201,13 +2201,13 @@
           <t>A person who has not formed an intention to enact a specified behaviour.</t>
         </is>
       </c>
-      <c r="D31" s="2" t="n"/>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">person </t>
+        </is>
+      </c>
       <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">person </t>
-        </is>
-      </c>
+      <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="n"/>
@@ -2255,18 +2255,18 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>The number of times a person performs a behaviour within a specific period.</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
+      <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="n"/>
       <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="n"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>The number of times a person performs a behaviour within a specific period.</t>
+        </is>
+      </c>
       <c r="J32" s="2" t="n"/>
       <c r="K32" s="2" t="inlineStr">
         <is>
@@ -2312,13 +2312,13 @@
           <t>A biological sibling who is male gender.</t>
         </is>
       </c>
-      <c r="D33" s="2" t="n"/>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>biological sibling</t>
+        </is>
+      </c>
       <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>biological sibling</t>
-        </is>
-      </c>
+      <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="n"/>
       <c r="H33" s="2" t="n"/>
       <c r="I33" s="2" t="n"/>
@@ -2367,13 +2367,13 @@
           <t>A child relation who is genetically related to their parent.</t>
         </is>
       </c>
-      <c r="D34" s="2" t="n"/>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>child relation</t>
+        </is>
+      </c>
       <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>child relation</t>
-        </is>
-      </c>
+      <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="n"/>
       <c r="H34" s="2" t="n"/>
       <c r="I34" s="2" t="n"/>
@@ -2422,13 +2422,13 @@
           <t>A biological child who is female gender.</t>
         </is>
       </c>
-      <c r="D35" s="2" t="n"/>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>biological child</t>
+        </is>
+      </c>
       <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>biological child</t>
-        </is>
-      </c>
+      <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="n"/>
       <c r="H35" s="2" t="n"/>
       <c r="I35" s="2" t="n"/>
@@ -2477,13 +2477,13 @@
           <t>A biological parent who provided the sperm.</t>
         </is>
       </c>
-      <c r="D36" s="2" t="n"/>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>biological parent</t>
+        </is>
+      </c>
       <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>biological parent</t>
-        </is>
-      </c>
+      <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="n"/>
       <c r="H36" s="2" t="n"/>
       <c r="I36" s="2" t="n"/>
@@ -2532,13 +2532,13 @@
           <t>A biological parent who provided an egg.</t>
         </is>
       </c>
-      <c r="D37" s="2" t="n"/>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>biological parent</t>
+        </is>
+      </c>
       <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>biological parent</t>
-        </is>
-      </c>
+      <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="n"/>
       <c r="H37" s="2" t="n"/>
       <c r="I37" s="2" t="n"/>
@@ -2587,13 +2587,13 @@
           <t>A parent who provided one of the gametes that resulted in one's conception.</t>
         </is>
       </c>
-      <c r="D38" s="2" t="n"/>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>parent</t>
+        </is>
+      </c>
       <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>parent</t>
-        </is>
-      </c>
+      <c r="F38" s="2" t="n"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
           <t>NCIT:C166114, GSSO:001986</t>
@@ -2646,13 +2646,13 @@
           <t>A bodily quality based on reproductive function or organs.</t>
         </is>
       </c>
-      <c r="D39" s="2" t="n"/>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>bodily quality</t>
+        </is>
+      </c>
       <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>bodily quality</t>
-        </is>
-      </c>
+      <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="n"/>
       <c r="H39" s="2" t="n"/>
       <c r="I39" s="2" t="n"/>
@@ -2701,13 +2701,13 @@
           <t>A sibling with whom the subject shares a biological parent.</t>
         </is>
       </c>
-      <c r="D40" s="2" t="n"/>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
       <c r="E40" s="2" t="n"/>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>sibling</t>
-        </is>
-      </c>
+      <c r="F40" s="2" t="n"/>
       <c r="G40" s="2" t="n"/>
       <c r="H40" s="2" t="n"/>
       <c r="I40" s="2" t="n"/>
@@ -2756,13 +2756,13 @@
           <t>A biological sibling who is female gender.</t>
         </is>
       </c>
-      <c r="D41" s="2" t="n"/>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>biological sibling</t>
+        </is>
+      </c>
       <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>biological sibling</t>
-        </is>
-      </c>
+      <c r="F41" s="2" t="n"/>
       <c r="G41" s="2" t="n"/>
       <c r="H41" s="2" t="n"/>
       <c r="I41" s="2" t="n"/>
@@ -2811,13 +2811,13 @@
           <t>A biological child who is male gender.</t>
         </is>
       </c>
-      <c r="D42" s="2" t="n"/>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>biological child</t>
+        </is>
+      </c>
       <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>biological child</t>
-        </is>
-      </c>
+      <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="n"/>
       <c r="H42" s="2" t="n"/>
       <c r="I42" s="2" t="n"/>
@@ -2866,13 +2866,13 @@
           <t>A sexual orientation of an individual who experiences sexual attraction to members of more than one sex.</t>
         </is>
       </c>
-      <c r="D43" s="2" t="n"/>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>sexual orientation</t>
+        </is>
+      </c>
       <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>sexual orientation</t>
-        </is>
-      </c>
+      <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
           <t>NCIT_C84364</t>
@@ -2925,7 +2925,7 @@
           <t>A quality that inheres in some extended organism.</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>quality</t>
         </is>
@@ -2957,13 +2957,13 @@
           <t>A role which inheres in a person and is realised by the person assuming responsibility for the physical and emotional needs of another who has difficulties with self care.</t>
         </is>
       </c>
-      <c r="D45" s="2" t="n"/>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
       <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
+      <c r="F45" s="2" t="n"/>
       <c r="G45" s="2" t="n"/>
       <c r="H45" s="2" t="n"/>
       <c r="I45" s="2" t="n"/>
@@ -3012,13 +3012,13 @@
           <t>A personal attribute as belonging to a group within a stratified system of categorisation based on a status conferred at birth based on descent, in which individuals have limited or no mobility due to custom or law.</t>
         </is>
       </c>
-      <c r="D46" s="2" t="n"/>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E46" s="2" t="n"/>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F46" s="2" t="n"/>
       <c r="G46" s="2" t="n"/>
       <c r="H46" s="2" t="n"/>
       <c r="I46" s="2" t="n"/>
@@ -3071,13 +3071,13 @@
           <t xml:space="preserve">A person who has not yet reached maturity. </t>
         </is>
       </c>
-      <c r="D47" s="2" t="n"/>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="n"/>
       <c r="H47" s="2" t="n"/>
       <c r="I47" s="2" t="n"/>
@@ -3130,13 +3130,13 @@
           <t>A family member who is a person's first generation offspring.</t>
         </is>
       </c>
-      <c r="D48" s="2" t="n"/>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>family member</t>
+        </is>
+      </c>
       <c r="E48" s="2" t="n"/>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>family member</t>
-        </is>
-      </c>
+      <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="n"/>
       <c r="H48" s="2" t="n"/>
       <c r="I48" s="2" t="n"/>
@@ -3185,13 +3185,13 @@
           <t>A gender identity that matches the person's assigned sex at birth.</t>
         </is>
       </c>
-      <c r="D49" s="2" t="n"/>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>gender identity</t>
+        </is>
+      </c>
       <c r="E49" s="2" t="n"/>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>gender identity</t>
-        </is>
-      </c>
+      <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
           <t>GSSO:004240</t>
@@ -3244,13 +3244,13 @@
           <t xml:space="preserve">A geographic location that is the country in which a person was born. </t>
         </is>
       </c>
-      <c r="D50" s="2" t="n"/>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>geographic location</t>
+        </is>
+      </c>
       <c r="E50" s="2" t="n"/>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>geographic location</t>
-        </is>
-      </c>
+      <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
           <t>GENEPIO_0001094</t>
@@ -3303,13 +3303,13 @@
           <t>A family member who is a child relation of one's aunt or uncle.</t>
         </is>
       </c>
-      <c r="D51" s="2" t="n"/>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>family member</t>
+        </is>
+      </c>
       <c r="E51" s="2" t="n"/>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>family member</t>
-        </is>
-      </c>
+      <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="n"/>
       <c r="H51" s="2" t="n"/>
       <c r="I51" s="2" t="n"/>
@@ -3358,13 +3358,13 @@
           <t>A personal attribute in which the person has impaired physical or mental functioning that has a notable effect on their ability to do typical daily activities.</t>
         </is>
       </c>
-      <c r="D52" s="2" t="n"/>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E52" s="2" t="n"/>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F52" s="2" t="n"/>
       <c r="G52" s="2" t="n"/>
       <c r="H52" s="2" t="n"/>
       <c r="I52" s="2" t="n"/>
@@ -3413,20 +3413,20 @@
           <t>An expertise discipline of the programme of study currently undertaken by the bearer of a student or trainee role.</t>
         </is>
       </c>
-      <c r="D53" s="2" t="n"/>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>expertise discipline</t>
+        </is>
+      </c>
       <c r="E53" s="2" t="n"/>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>expertise discipline</t>
+          <t>psychology, counselling, public health</t>
         </is>
       </c>
       <c r="G53" s="2" t="n"/>
       <c r="H53" s="2" t="n"/>
-      <c r="I53" s="2" t="inlineStr">
-        <is>
-          <t>psychology, counselling, public health</t>
-        </is>
-      </c>
+      <c r="I53" s="2" t="n"/>
       <c r="J53" s="2" t="inlineStr">
         <is>
           <t>The division of knowledge and practice into different disciplines or fields is complex and depends on historical, social and structural factors</t>
@@ -3476,20 +3476,20 @@
           <t>An expertise discipline of the highest level of formal educational qualification a person has achieved.</t>
         </is>
       </c>
-      <c r="D54" s="2" t="n"/>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>expertise discipline</t>
+        </is>
+      </c>
       <c r="E54" s="2" t="n"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>expertise discipline</t>
+          <t>Mathematics, English, hairdressing skills, vehicle engineering, nursing, astrophysics, accountancy</t>
         </is>
       </c>
       <c r="G54" s="2" t="n"/>
       <c r="H54" s="2" t="n"/>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>Mathematics, English, hairdressing skills, vehicle engineering, nursing, astrophysics, accountancy</t>
-        </is>
-      </c>
+      <c r="I54" s="2" t="n"/>
       <c r="J54" s="2" t="n"/>
       <c r="K54" s="2" t="inlineStr">
         <is>
@@ -3535,13 +3535,13 @@
           <t>A relationship status where the individual was previously in a legally formalised relationship and this relationship has now ended or dissolved.</t>
         </is>
       </c>
-      <c r="D55" s="2" t="n"/>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>relationship status</t>
+        </is>
+      </c>
       <c r="E55" s="2" t="n"/>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>relationship status</t>
-        </is>
-      </c>
+      <c r="F55" s="2" t="n"/>
       <c r="G55" s="2" t="n"/>
       <c r="H55" s="2" t="n"/>
       <c r="I55" s="2" t="n"/>
@@ -3590,13 +3590,13 @@
           <t>A higher education student  role realised by currently studying for a doctoral degree.</t>
         </is>
       </c>
-      <c r="D56" s="3" t="n"/>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>higher education student role</t>
+        </is>
+      </c>
       <c r="E56" s="3" t="n"/>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>higher education student role</t>
-        </is>
-      </c>
+      <c r="F56" s="3" t="n"/>
       <c r="G56" s="3" t="n"/>
       <c r="H56" s="3" t="n"/>
       <c r="I56" s="3" t="n"/>
@@ -3645,13 +3645,13 @@
           <t>A higher education student  role realised by currently studying for a doctoral degree.</t>
         </is>
       </c>
-      <c r="D57" s="2" t="n"/>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>higher education student role</t>
+        </is>
+      </c>
       <c r="E57" s="2" t="n"/>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
-          <t>higher education student role</t>
-        </is>
-      </c>
+      <c r="F57" s="2" t="n"/>
       <c r="G57" s="2" t="n"/>
       <c r="H57" s="2" t="n"/>
       <c r="I57" s="2" t="n"/>
@@ -3700,13 +3700,13 @@
           <t>A &lt;social group&gt; of two people who interact and influence each other.</t>
         </is>
       </c>
-      <c r="D58" s="2" t="n"/>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>social group</t>
+        </is>
+      </c>
       <c r="E58" s="2" t="n"/>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>social group</t>
-        </is>
-      </c>
+      <c r="F58" s="2" t="n"/>
       <c r="G58" s="2" t="n"/>
       <c r="H58" s="2" t="n"/>
       <c r="I58" s="2" t="n"/>
@@ -3747,13 +3747,13 @@
           <t>A planned process wherein knowledge and skills is imparted.</t>
         </is>
       </c>
-      <c r="D59" s="2" t="n"/>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>planned process</t>
+        </is>
+      </c>
       <c r="E59" s="2" t="n"/>
-      <c r="F59" s="2" t="inlineStr">
-        <is>
-          <t>planned process</t>
-        </is>
-      </c>
+      <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
           <t>education process in the Sustainable Development Goals Interface Ontology (SDGIO:00010001)</t>
@@ -3798,13 +3798,13 @@
           <t>An employment status realised by an individual being engaged in an activity or service for wages or salary.</t>
         </is>
       </c>
-      <c r="D60" s="2" t="n"/>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>employment status</t>
+        </is>
+      </c>
       <c r="E60" s="2" t="n"/>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>employment status</t>
-        </is>
-      </c>
+      <c r="F60" s="2" t="n"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
           <t>NCIT_C25172</t>
@@ -3857,13 +3857,13 @@
           <t>An employment status realised by an individual working a standard number of hours defined as full-time by their employer.</t>
         </is>
       </c>
-      <c r="D61" s="2" t="n"/>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>employment status</t>
+        </is>
+      </c>
       <c r="E61" s="2" t="n"/>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t>employment status</t>
-        </is>
-      </c>
+      <c r="F61" s="2" t="n"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
           <t>OPMI:0000123</t>
@@ -3916,13 +3916,13 @@
           <t>An employment status realised by an individual working for recurring periods in which different groups of workers do the same jobs in relay.</t>
         </is>
       </c>
-      <c r="D62" s="2" t="n"/>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>employment status</t>
+        </is>
+      </c>
       <c r="E62" s="2" t="n"/>
-      <c r="F62" s="2" t="inlineStr">
-        <is>
-          <t>employment status</t>
-        </is>
-      </c>
+      <c r="F62" s="2" t="n"/>
       <c r="G62" s="2" t="n"/>
       <c r="H62" s="2" t="n"/>
       <c r="I62" s="2" t="n"/>
@@ -3971,13 +3971,13 @@
           <t>An employment status realised by an individual whose working hours involving less than the standard or customary working time.</t>
         </is>
       </c>
-      <c r="D63" s="2" t="n"/>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>employment status</t>
+        </is>
+      </c>
       <c r="E63" s="2" t="n"/>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>employment status</t>
-        </is>
-      </c>
+      <c r="F63" s="2" t="n"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
           <t>NCIT_C75562</t>
@@ -4027,16 +4027,16 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>A quality inhering in a person by virtue of that person bearing a role realised in an employment process.</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="n"/>
+          <t>A personal attribute relating the bearer to an employment process.</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E64" s="2" t="n"/>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>quality</t>
-        </is>
-      </c>
+      <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
           <t>Sustainable Development Goals Interface Ontology (SDGIO:00010029)</t>
@@ -4094,13 +4094,13 @@
           <t>A self-identity as belonging to a social group or groups whose members have a common cultural or ancestral heritage.</t>
         </is>
       </c>
-      <c r="D65" s="2" t="n"/>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>self-identity</t>
+        </is>
+      </c>
       <c r="E65" s="2" t="n"/>
-      <c r="F65" s="2" t="inlineStr">
-        <is>
-          <t>self-identity</t>
-        </is>
-      </c>
+      <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
           <t>EFO:0001799</t>
@@ -4157,13 +4157,13 @@
           <t>An attribute that is a field of knowledge or practice.</t>
         </is>
       </c>
-      <c r="D66" s="2" t="n"/>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>specifically dependent continuant</t>
+        </is>
+      </c>
       <c r="E66" s="2" t="n"/>
-      <c r="F66" s="2" t="inlineStr">
-        <is>
-          <t>specifically dependent continuant</t>
-        </is>
-      </c>
+      <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="n"/>
       <c r="H66" s="2" t="n"/>
       <c r="I66" s="2" t="n"/>
@@ -4212,13 +4212,13 @@
           <t>A data item that is the extent to which the person’s past behaviour has reached or exceeded a standard.</t>
         </is>
       </c>
-      <c r="D67" s="2" t="n"/>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E67" s="2" t="n"/>
-      <c r="F67" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F67" s="2" t="n"/>
       <c r="G67" s="2" t="n"/>
       <c r="H67" s="2" t="n"/>
       <c r="I67" s="2" t="n"/>
@@ -4267,13 +4267,13 @@
           <t>A person who is a member of a group of persons united by blood, or by marriage or other legal arrangement, or by self-identity as belonging to the same family.</t>
         </is>
       </c>
-      <c r="D68" s="2" t="n"/>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E68" s="2" t="n"/>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
           <t>NCIT:C41256</t>
@@ -4326,13 +4326,13 @@
           <t>A parent who is male gender.</t>
         </is>
       </c>
-      <c r="D69" s="2" t="n"/>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>parent</t>
+        </is>
+      </c>
       <c r="E69" s="2" t="n"/>
-      <c r="F69" s="2" t="inlineStr">
-        <is>
-          <t>parent</t>
-        </is>
-      </c>
+      <c r="F69" s="2" t="n"/>
       <c r="G69" s="2" t="n"/>
       <c r="H69" s="2" t="n"/>
       <c r="I69" s="2" t="n"/>
@@ -4381,13 +4381,13 @@
           <t>A biological sex associated with the ability to produce female gametes.</t>
         </is>
       </c>
-      <c r="D70" s="2" t="n"/>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>biological sex</t>
+        </is>
+      </c>
       <c r="E70" s="2" t="n"/>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>biological sex</t>
-        </is>
-      </c>
+      <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="n"/>
       <c r="H70" s="2" t="n"/>
       <c r="I70" s="2" t="n"/>
@@ -4436,13 +4436,13 @@
           <t>A gender identity as being female.</t>
         </is>
       </c>
-      <c r="D71" s="2" t="n"/>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>gender identity</t>
+        </is>
+      </c>
       <c r="E71" s="2" t="n"/>
-      <c r="F71" s="2" t="inlineStr">
-        <is>
-          <t>gender identity</t>
-        </is>
-      </c>
+      <c r="F71" s="2" t="n"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
           <t>GSSO:000089</t>
@@ -4499,13 +4499,13 @@
           <t>A foster sibling who is male gender.</t>
         </is>
       </c>
-      <c r="D72" s="2" t="n"/>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>foster sibling</t>
+        </is>
+      </c>
       <c r="E72" s="2" t="n"/>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>foster sibling</t>
-        </is>
-      </c>
+      <c r="F72" s="2" t="n"/>
       <c r="G72" s="2" t="n"/>
       <c r="H72" s="2" t="n"/>
       <c r="I72" s="2" t="n"/>
@@ -4554,13 +4554,13 @@
           <t xml:space="preserve">A child relation in a parent-child relationship created by a foster care arrangement. </t>
         </is>
       </c>
-      <c r="D73" s="2" t="n"/>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>child relation</t>
+        </is>
+      </c>
       <c r="E73" s="2" t="n"/>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>child relation</t>
-        </is>
-      </c>
+      <c r="F73" s="2" t="n"/>
       <c r="G73" s="2" t="n"/>
       <c r="H73" s="2" t="n"/>
       <c r="I73" s="2" t="n"/>
@@ -4609,13 +4609,13 @@
           <t>A foster child who is female gender.</t>
         </is>
       </c>
-      <c r="D74" s="2" t="n"/>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>foster child</t>
+        </is>
+      </c>
       <c r="E74" s="2" t="n"/>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>foster child</t>
-        </is>
-      </c>
+      <c r="F74" s="2" t="n"/>
       <c r="G74" s="2" t="n"/>
       <c r="H74" s="2" t="n"/>
       <c r="I74" s="2" t="n"/>
@@ -4664,13 +4664,13 @@
           <t>A foster parent who is male gender.</t>
         </is>
       </c>
-      <c r="D75" s="2" t="n"/>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>foster parent</t>
+        </is>
+      </c>
       <c r="E75" s="2" t="n"/>
-      <c r="F75" s="2" t="inlineStr">
-        <is>
-          <t>foster parent</t>
-        </is>
-      </c>
+      <c r="F75" s="2" t="n"/>
       <c r="G75" s="2" t="n"/>
       <c r="H75" s="2" t="n"/>
       <c r="I75" s="2" t="n"/>
@@ -4719,13 +4719,13 @@
           <t>A foster parent who is female gender.</t>
         </is>
       </c>
-      <c r="D76" s="2" t="n"/>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>foster parent</t>
+        </is>
+      </c>
       <c r="E76" s="2" t="n"/>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>foster parent</t>
-        </is>
-      </c>
+      <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="n"/>
       <c r="H76" s="2" t="n"/>
       <c r="I76" s="2" t="n"/>
@@ -4774,13 +4774,13 @@
           <t>A parent who cares for a child who has been placed with them in a foster care arrangement.</t>
         </is>
       </c>
-      <c r="D77" s="2" t="n"/>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>parent</t>
+        </is>
+      </c>
       <c r="E77" s="2" t="n"/>
-      <c r="F77" s="2" t="inlineStr">
-        <is>
-          <t>parent</t>
-        </is>
-      </c>
+      <c r="F77" s="2" t="n"/>
       <c r="G77" s="2" t="inlineStr">
         <is>
           <t>GSSO:001987</t>
@@ -4833,13 +4833,13 @@
           <t>A sibling who shares a parent through a parent-child relationship created by a foster care agreement.</t>
         </is>
       </c>
-      <c r="D78" s="2" t="n"/>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
       <c r="E78" s="2" t="n"/>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>sibling</t>
-        </is>
-      </c>
+      <c r="F78" s="2" t="n"/>
       <c r="G78" s="2" t="n"/>
       <c r="H78" s="2" t="n"/>
       <c r="I78" s="2" t="n"/>
@@ -4888,13 +4888,13 @@
           <t>A foster sibling who is female gender.</t>
         </is>
       </c>
-      <c r="D79" s="2" t="n"/>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>foster sibling</t>
+        </is>
+      </c>
       <c r="E79" s="2" t="n"/>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t>foster sibling</t>
-        </is>
-      </c>
+      <c r="F79" s="2" t="n"/>
       <c r="G79" s="2" t="n"/>
       <c r="H79" s="2" t="n"/>
       <c r="I79" s="2" t="n"/>
@@ -4943,13 +4943,13 @@
           <t>A foster child who is male gender.</t>
         </is>
       </c>
-      <c r="D80" s="2" t="n"/>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>foster child</t>
+        </is>
+      </c>
       <c r="E80" s="2" t="n"/>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>foster child</t>
-        </is>
-      </c>
+      <c r="F80" s="2" t="n"/>
       <c r="G80" s="2" t="n"/>
       <c r="H80" s="2" t="n"/>
       <c r="I80" s="2" t="n"/>
@@ -4998,13 +4998,13 @@
           <t>A behavioural frequency about the number of times a person has enacted a behaviour per unit of time.</t>
         </is>
       </c>
-      <c r="D81" s="2" t="n"/>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>behavioural frequency</t>
+        </is>
+      </c>
       <c r="E81" s="2" t="n"/>
-      <c r="F81" s="2" t="inlineStr">
-        <is>
-          <t>behavioural frequency</t>
-        </is>
-      </c>
+      <c r="F81" s="2" t="n"/>
       <c r="G81" s="2" t="n"/>
       <c r="H81" s="2" t="n"/>
       <c r="I81" s="2" t="n"/>
@@ -5053,13 +5053,13 @@
           <t>A self-identity as having a particular gender, which may or may not correspond with sex assigned at birth.</t>
         </is>
       </c>
-      <c r="D82" s="2" t="n"/>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>self-identity</t>
+        </is>
+      </c>
       <c r="E82" s="2" t="n"/>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>self-identity</t>
-        </is>
-      </c>
+      <c r="F82" s="2" t="n"/>
       <c r="G82" s="2" t="n"/>
       <c r="H82" s="2" t="n"/>
       <c r="I82" s="2" t="n"/>
@@ -5108,13 +5108,13 @@
           <t>A higher education student role realised by currently studying for a more advanced degree after completing an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D83" s="3" t="n"/>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>higher education student role</t>
+        </is>
+      </c>
       <c r="E83" s="3" t="n"/>
-      <c r="F83" s="3" t="inlineStr">
-        <is>
-          <t>higher education student role</t>
-        </is>
-      </c>
+      <c r="F83" s="3" t="n"/>
       <c r="G83" s="3" t="n"/>
       <c r="H83" s="3" t="n"/>
       <c r="I83" s="3" t="n"/>
@@ -5163,13 +5163,13 @@
           <t>A higher education student role realised by currently studying for a more advanced degree after completing an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D84" s="2" t="n"/>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>higher education student role</t>
+        </is>
+      </c>
       <c r="E84" s="2" t="n"/>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>higher education student role</t>
-        </is>
-      </c>
+      <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="n"/>
       <c r="H84" s="2" t="n"/>
       <c r="I84" s="2" t="n"/>
@@ -5218,13 +5218,13 @@
           <t>A grandparent who is male gender.</t>
         </is>
       </c>
-      <c r="D85" s="2" t="n"/>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>grandparent</t>
+        </is>
+      </c>
       <c r="E85" s="2" t="n"/>
-      <c r="F85" s="2" t="inlineStr">
-        <is>
-          <t>grandparent</t>
-        </is>
-      </c>
+      <c r="F85" s="2" t="n"/>
       <c r="G85" s="2" t="n"/>
       <c r="H85" s="2" t="n"/>
       <c r="I85" s="2" t="n"/>
@@ -5273,13 +5273,13 @@
           <t>A grandparent who is female gender.</t>
         </is>
       </c>
-      <c r="D86" s="2" t="n"/>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>grandparent</t>
+        </is>
+      </c>
       <c r="E86" s="2" t="n"/>
-      <c r="F86" s="2" t="inlineStr">
-        <is>
-          <t>grandparent</t>
-        </is>
-      </c>
+      <c r="F86" s="2" t="n"/>
       <c r="G86" s="2" t="n"/>
       <c r="H86" s="2" t="n"/>
       <c r="I86" s="2" t="n"/>
@@ -5328,13 +5328,13 @@
           <t>A family member who is the parent of one's parent.</t>
         </is>
       </c>
-      <c r="D87" s="2" t="n"/>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>family member</t>
+        </is>
+      </c>
       <c r="E87" s="2" t="n"/>
-      <c r="F87" s="2" t="inlineStr">
-        <is>
-          <t>family member</t>
-        </is>
-      </c>
+      <c r="F87" s="2" t="n"/>
       <c r="G87" s="2" t="n"/>
       <c r="H87" s="2" t="n"/>
       <c r="I87" s="2" t="n"/>
@@ -5383,13 +5383,13 @@
           <t xml:space="preserve">A personal history part that includes previously performing a behaviour. </t>
         </is>
       </c>
-      <c r="D88" s="2" t="n"/>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>personal history part</t>
+        </is>
+      </c>
       <c r="E88" s="2" t="n"/>
-      <c r="F88" s="2" t="inlineStr">
-        <is>
-          <t>personal history part</t>
-        </is>
-      </c>
+      <c r="F88" s="2" t="n"/>
       <c r="G88" s="2" t="n"/>
       <c r="H88" s="2" t="n"/>
       <c r="I88" s="2" t="n"/>
@@ -5438,20 +5438,20 @@
           <t>A policy holder role that inheres in a person who participates in the creation of an insurance contract designed to cover some or all of the cost of treating the insured person's illnesses or injuries as well as possibly providing preventive health care.</t>
         </is>
       </c>
-      <c r="D89" s="2" t="n"/>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>policy holder role</t>
+        </is>
+      </c>
       <c r="E89" s="2" t="n"/>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>policy holder role</t>
+          <t>having Medicare, Medicaid, Blue Cross, BUPA, being eligible for NHS treatment</t>
         </is>
       </c>
       <c r="G89" s="2" t="n"/>
       <c r="H89" s="2" t="n"/>
-      <c r="I89" s="2" t="inlineStr">
-        <is>
-          <t>having Medicare, Medicaid, Blue Cross, BUPA, being eligible for NHS treatment</t>
-        </is>
-      </c>
+      <c r="I89" s="2" t="n"/>
       <c r="J89" s="2" t="n"/>
       <c r="K89" s="2" t="inlineStr">
         <is>
@@ -5497,11 +5497,15 @@
           <t>A personal attribute that is the state of an individual's mental or physical condition.</t>
         </is>
       </c>
-      <c r="D90" s="2" t="n"/>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E90" s="2" t="n"/>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>personal attribute</t>
+          <t>Having chicken pox, asthma, a heart attack</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -5510,11 +5514,7 @@
         </is>
       </c>
       <c r="H90" s="2" t="n"/>
-      <c r="I90" s="2" t="inlineStr">
-        <is>
-          <t>Having chicken pox, asthma, a heart attack</t>
-        </is>
-      </c>
+      <c r="I90" s="2" t="n"/>
       <c r="J90" s="2" t="n"/>
       <c r="K90" s="2" t="inlineStr">
         <is>
@@ -5560,13 +5560,13 @@
           <t>A sexual orientation of an individual who experiences sexual attraction exclusively or primarily to members of a different sex.</t>
         </is>
       </c>
-      <c r="D91" s="2" t="n"/>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>sexual orientation</t>
+        </is>
+      </c>
       <c r="E91" s="2" t="n"/>
-      <c r="F91" s="2" t="inlineStr">
-        <is>
-          <t>sexual orientation</t>
-        </is>
-      </c>
+      <c r="F91" s="2" t="n"/>
       <c r="G91" s="2" t="inlineStr">
         <is>
           <t>NCIT_C84362</t>
@@ -5619,13 +5619,13 @@
           <t>A frequency of past behaviour that is above a threshold.</t>
         </is>
       </c>
-      <c r="D92" s="2" t="n"/>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>frequency of past behaviour</t>
+        </is>
+      </c>
       <c r="E92" s="2" t="n"/>
-      <c r="F92" s="2" t="inlineStr">
-        <is>
-          <t>frequency of past behaviour</t>
-        </is>
-      </c>
+      <c r="F92" s="2" t="n"/>
       <c r="G92" s="2" t="n"/>
       <c r="H92" s="2" t="n"/>
       <c r="I92" s="2" t="n"/>
@@ -5670,13 +5670,13 @@
           <t xml:space="preserve">A student or trainee role realised by currently learning on an advanced educational programme in a university, college or professional school. For example, completing a university bachelor's or master's course of study, medical school or other professional school. </t>
         </is>
       </c>
-      <c r="D93" s="3" t="n"/>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>student or trainee role</t>
+        </is>
+      </c>
       <c r="E93" s="3" t="n"/>
-      <c r="F93" s="3" t="inlineStr">
-        <is>
-          <t>student or trainee role</t>
-        </is>
-      </c>
+      <c r="F93" s="3" t="n"/>
       <c r="G93" s="3" t="n"/>
       <c r="H93" s="3" t="n"/>
       <c r="I93" s="3" t="n"/>
@@ -5725,20 +5725,20 @@
           <t>A student or trainee role realised by currently learning on an advanced educational programme in a university, college or professional school.</t>
         </is>
       </c>
-      <c r="D94" s="2" t="n"/>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>student or trainee role</t>
+        </is>
+      </c>
       <c r="E94" s="2" t="n"/>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>student or trainee role</t>
+          <t>completing a university bachelor's or master's course of study, medical school or other professional school.</t>
         </is>
       </c>
       <c r="G94" s="2" t="n"/>
       <c r="H94" s="2" t="n"/>
-      <c r="I94" s="2" t="inlineStr">
-        <is>
-          <t>completing a university bachelor's or master's course of study, medical school or other professional school.</t>
-        </is>
-      </c>
+      <c r="I94" s="2" t="n"/>
       <c r="J94" s="2" t="n"/>
       <c r="K94" s="2" t="inlineStr">
         <is>
@@ -5784,13 +5784,13 @@
           <t>A personal attribute related to the highest level of education achieved.</t>
         </is>
       </c>
-      <c r="D95" s="2" t="n"/>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E95" s="2" t="n"/>
-      <c r="F95" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F95" s="2" t="n"/>
       <c r="G95" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">NCIT_C17953 </t>
@@ -5847,7 +5847,7 @@
           <t>A process that is the sum of the totality of processes taking place in the spatiotemporal region occupied by a material entity or site, including processes on the surface of the entity or within the cavities to which it serves as host.</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr">
+      <c r="D96" t="inlineStr">
         <is>
           <t>process</t>
         </is>
@@ -5879,20 +5879,20 @@
           <t>A personal history part that includes exposure to a potentially harmful agent as a result of one's occupation.</t>
         </is>
       </c>
-      <c r="D97" s="2" t="n"/>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>personal history part</t>
+        </is>
+      </c>
       <c r="E97" s="2" t="n"/>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>personal history part</t>
+          <t>history of exposure to asbestos due to one's job</t>
         </is>
       </c>
       <c r="G97" s="2" t="n"/>
       <c r="H97" s="2" t="n"/>
-      <c r="I97" s="2" t="inlineStr">
-        <is>
-          <t>history of exposure to asbestos due to one's job</t>
-        </is>
-      </c>
+      <c r="I97" s="2" t="n"/>
       <c r="J97" s="2" t="n"/>
       <c r="K97" s="2" t="inlineStr">
         <is>
@@ -5938,20 +5938,20 @@
           <t>A personal history part that includes experience of physical, sexual, or psychological maltreatment during the first 18 years of life.</t>
         </is>
       </c>
-      <c r="D98" s="2" t="n"/>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>personal history part</t>
+        </is>
+      </c>
       <c r="E98" s="2" t="n"/>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>personal history part</t>
+          <t>history of physical abuse by a parent</t>
         </is>
       </c>
       <c r="G98" s="2" t="n"/>
       <c r="H98" s="2" t="n"/>
-      <c r="I98" s="2" t="inlineStr">
-        <is>
-          <t>history of physical abuse by a parent</t>
-        </is>
-      </c>
+      <c r="I98" s="2" t="n"/>
       <c r="J98" s="2" t="n"/>
       <c r="K98" s="2" t="inlineStr">
         <is>
@@ -5997,13 +5997,13 @@
           <t>A person who does not own a residential facility and does not have an agreement with a residential facility owner that would enable them to live in a residential facility.</t>
         </is>
       </c>
-      <c r="D99" s="2" t="n"/>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E99" s="2" t="n"/>
-      <c r="F99" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F99" s="2" t="n"/>
       <c r="G99" s="2" t="n"/>
       <c r="H99" s="2" t="inlineStr">
         <is>
@@ -6056,13 +6056,13 @@
           <t>A personal attribute inhering in a person who does not bear a role realised in an employment process and who manages their home as their main daily activity.</t>
         </is>
       </c>
-      <c r="D100" s="2" t="n"/>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E100" s="2" t="n"/>
-      <c r="F100" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F100" s="2" t="n"/>
       <c r="G100" s="2" t="inlineStr">
         <is>
           <t>NCIT_C75560</t>
@@ -6115,13 +6115,13 @@
           <t>A sexual orientation of an individual who experiences sexual attraction exclusively or primarily to members of the same sex.</t>
         </is>
       </c>
-      <c r="D101" s="2" t="n"/>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>sexual orientation</t>
+        </is>
+      </c>
       <c r="E101" s="2" t="n"/>
-      <c r="F101" s="2" t="inlineStr">
-        <is>
-          <t>sexual orientation</t>
-        </is>
-      </c>
+      <c r="F101" s="2" t="n"/>
       <c r="G101" s="2" t="inlineStr">
         <is>
           <t>NCIT_C84363</t>
@@ -6174,7 +6174,7 @@
           <t>A human or collection of humans that occupies a housing unit by storing their possessions there and habitually sleeping there thereby participating in the realization of its residence function.</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr">
+      <c r="D102" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>
@@ -6211,13 +6211,13 @@
           <t>An aggregate of the individual incomes received by all the members of a household.</t>
         </is>
       </c>
-      <c r="D103" s="3" t="n"/>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
       <c r="E103" s="3" t="n"/>
-      <c r="F103" s="3" t="inlineStr">
-        <is>
-          <t>object aggregate</t>
-        </is>
-      </c>
+      <c r="F103" s="3" t="n"/>
       <c r="G103" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">EFO_0009695 </t>
@@ -6274,13 +6274,13 @@
           <t>A personal attribute that is a time quality inhering in a person by virtue of how long since the person was born.</t>
         </is>
       </c>
-      <c r="D104" s="2" t="n"/>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E104" s="2" t="n"/>
-      <c r="F104" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F104" s="2" t="n"/>
       <c r="G104" s="2" t="inlineStr">
         <is>
           <t>PATO:0000011</t>
@@ -6333,13 +6333,13 @@
           <t>An object aggregate that consists of two or more people.</t>
         </is>
       </c>
-      <c r="D105" s="2" t="n"/>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
       <c r="E105" s="2" t="n"/>
-      <c r="F105" s="2" t="inlineStr">
-        <is>
-          <t>object aggregate</t>
-        </is>
-      </c>
+      <c r="F105" s="2" t="n"/>
       <c r="G105" s="2" t="n"/>
       <c r="H105" s="2" t="n"/>
       <c r="I105" s="2" t="n"/>
@@ -6380,7 +6380,7 @@
           <t>A cognitive representation of themselves by a person or group.</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr">
+      <c r="D106" t="inlineStr">
         <is>
           <t>cognitive representation</t>
         </is>
@@ -6412,13 +6412,13 @@
           <t>A person who has previously been a resident of a country and is now resident in another country.</t>
         </is>
       </c>
-      <c r="D107" s="2" t="n"/>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E107" s="2" t="n"/>
-      <c r="F107" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F107" s="2" t="n"/>
       <c r="G107" s="2" t="n"/>
       <c r="H107" s="2" t="n"/>
       <c r="I107" s="2" t="n"/>
@@ -6467,13 +6467,13 @@
           <t xml:space="preserve">A relationship status where the individual is in a legally formalised marriage or civil partnership. </t>
         </is>
       </c>
-      <c r="D108" s="2" t="n"/>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>relationship status</t>
+        </is>
+      </c>
       <c r="E108" s="2" t="n"/>
-      <c r="F108" s="2" t="inlineStr">
-        <is>
-          <t>relationship status</t>
-        </is>
-      </c>
+      <c r="F108" s="2" t="n"/>
       <c r="G108" s="2" t="n"/>
       <c r="H108" s="2" t="n"/>
       <c r="I108" s="2" t="n"/>
@@ -6523,13 +6523,13 @@
           <t>A relationship status where the individual has had the same partner for a significant length of time but is not in a legal union.</t>
         </is>
       </c>
-      <c r="D109" s="2" t="n"/>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>relationship status</t>
+        </is>
+      </c>
       <c r="E109" s="2" t="n"/>
-      <c r="F109" s="2" t="inlineStr">
-        <is>
-          <t>relationship status</t>
-        </is>
-      </c>
+      <c r="F109" s="2" t="n"/>
       <c r="G109" s="2" t="n"/>
       <c r="H109" s="2" t="n"/>
       <c r="I109" s="2" t="n"/>
@@ -6582,13 +6582,13 @@
           <t>An employment status realised by an individual working for a company or other organisation without a pre-determined end date, with security of employment and known working conditions.</t>
         </is>
       </c>
-      <c r="D110" s="2" t="n"/>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>employment status</t>
+        </is>
+      </c>
       <c r="E110" s="2" t="n"/>
-      <c r="F110" s="2" t="inlineStr">
-        <is>
-          <t>employment status</t>
-        </is>
-      </c>
+      <c r="F110" s="2" t="n"/>
       <c r="G110" s="2" t="n"/>
       <c r="H110" s="2" t="n"/>
       <c r="I110" s="2" t="n"/>
@@ -6637,13 +6637,13 @@
           <t>An employment status realised by an individual working for a company or other organisation in a position that is of a known, fixed duration with security of employment for that duration and certain working conditions.</t>
         </is>
       </c>
-      <c r="D111" s="2" t="n"/>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>employment status</t>
+        </is>
+      </c>
       <c r="E111" s="2" t="n"/>
-      <c r="F111" s="2" t="inlineStr">
-        <is>
-          <t>employment status</t>
-        </is>
-      </c>
+      <c r="F111" s="2" t="n"/>
       <c r="G111" s="2" t="n"/>
       <c r="H111" s="2" t="n"/>
       <c r="I111" s="2" t="n"/>
@@ -6692,13 +6692,13 @@
           <t>An employment status realised by an individual working for a company or other organisation in a position with uncertain duration or hours with unknown or low security of working conditions or pay.</t>
         </is>
       </c>
-      <c r="D112" s="2" t="n"/>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>employment status</t>
+        </is>
+      </c>
       <c r="E112" s="2" t="n"/>
-      <c r="F112" s="2" t="inlineStr">
-        <is>
-          <t>employment status</t>
-        </is>
-      </c>
+      <c r="F112" s="2" t="n"/>
       <c r="G112" s="2" t="n"/>
       <c r="H112" s="2" t="n"/>
       <c r="I112" s="2" t="n"/>
@@ -6747,13 +6747,13 @@
           <t>Individual income that an individual otherwise of low-income receives as a payment made by the state or an insurance scheme in the form of housing vouchers,  credit or benefits.</t>
         </is>
       </c>
-      <c r="D113" s="3" t="n"/>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>individual income</t>
+        </is>
+      </c>
       <c r="E113" s="3" t="n"/>
-      <c r="F113" s="3" t="inlineStr">
-        <is>
-          <t>individual income</t>
-        </is>
-      </c>
+      <c r="F113" s="3" t="n"/>
       <c r="G113" s="3" t="n"/>
       <c r="H113" s="3" t="n"/>
       <c r="I113" s="3" t="n"/>
@@ -6802,13 +6802,13 @@
           <t>A personal attribute inhering in a person who does not bear a role realised in an employment process due to possessing enough wealth to not need financial support from another person or require income from employment.</t>
         </is>
       </c>
-      <c r="D114" s="2" t="n"/>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E114" s="2" t="n"/>
-      <c r="F114" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F114" s="2" t="n"/>
       <c r="G114" s="2" t="n"/>
       <c r="H114" s="2" t="n"/>
       <c r="I114" s="2" t="n"/>
@@ -6857,20 +6857,20 @@
           <t>A bodily process of a human that involves co-ordinated contraction of striated muscles controlled by the brain.</t>
         </is>
       </c>
-      <c r="D115" s="2" t="n"/>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>bodily process</t>
+        </is>
+      </c>
       <c r="E115" s="2" t="n"/>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>bodily process</t>
+          <t>walks for 15 mins/day, never eats meat, attends school daily</t>
         </is>
       </c>
       <c r="G115" s="2" t="n"/>
       <c r="H115" s="2" t="n"/>
-      <c r="I115" s="2" t="inlineStr">
-        <is>
-          <t>walks for 15 mins/day, never eats meat, attends school daily</t>
-        </is>
-      </c>
+      <c r="I115" s="2" t="n"/>
       <c r="J115" s="2" t="n"/>
       <c r="K115" s="2" t="inlineStr">
         <is>
@@ -6916,13 +6916,13 @@
           <t>A personal attribute reflecting a benefit the person receives  derived from their capital or labour, usually measured in money.</t>
         </is>
       </c>
-      <c r="D116" s="2" t="n"/>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E116" s="2" t="n"/>
-      <c r="F116" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F116" s="2" t="n"/>
       <c r="G116" s="2" t="inlineStr">
         <is>
           <t>OMRSE_00002061</t>
@@ -6975,13 +6975,13 @@
           <t>A social role that involves influencing other people to adopt new ideas or behaviours.</t>
         </is>
       </c>
-      <c r="D117" s="2" t="n"/>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>social role</t>
+        </is>
+      </c>
       <c r="E117" s="2" t="n"/>
-      <c r="F117" s="2" t="inlineStr">
-        <is>
-          <t>social role</t>
-        </is>
-      </c>
+      <c r="F117" s="2" t="n"/>
       <c r="G117" s="2" t="n"/>
       <c r="H117" s="2" t="n"/>
       <c r="I117" s="2" t="n"/>
@@ -7030,13 +7030,13 @@
           <t>A student or trainee role realised by  currently learning in a non-institutional setting.</t>
         </is>
       </c>
-      <c r="D118" s="3" t="n"/>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>student or trainee role</t>
+        </is>
+      </c>
       <c r="E118" s="3" t="n"/>
-      <c r="F118" s="3" t="inlineStr">
-        <is>
-          <t>student or trainee role</t>
-        </is>
-      </c>
+      <c r="F118" s="3" t="n"/>
       <c r="G118" s="3" t="n"/>
       <c r="H118" s="3" t="n"/>
       <c r="I118" s="3" t="n"/>
@@ -7085,13 +7085,13 @@
           <t>A student or trainee that is currently learning in a non-institutional setting.</t>
         </is>
       </c>
-      <c r="D119" s="2" t="n"/>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>student or trainee role</t>
+        </is>
+      </c>
       <c r="E119" s="2" t="n"/>
-      <c r="F119" s="2" t="inlineStr">
-        <is>
-          <t>student or trainee role</t>
-        </is>
-      </c>
+      <c r="F119" s="2" t="n"/>
       <c r="G119" s="2" t="n"/>
       <c r="H119" s="2" t="n"/>
       <c r="I119" s="2" t="n"/>
@@ -7140,13 +7140,13 @@
           <t>A patient role which inheres in a person and is realized by being under the care of a physician or health care provider and being admitted to a hospital or equivalent facility.</t>
         </is>
       </c>
-      <c r="D120" s="2" t="n"/>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>patient role</t>
+        </is>
+      </c>
       <c r="E120" s="2" t="n"/>
-      <c r="F120" s="2" t="inlineStr">
-        <is>
-          <t>patient role</t>
-        </is>
-      </c>
+      <c r="F120" s="2" t="n"/>
       <c r="G120" s="2" t="n"/>
       <c r="H120" s="2" t="n"/>
       <c r="I120" s="2" t="n"/>
@@ -7195,13 +7195,13 @@
           <t xml:space="preserve">A role that inheres in an organism that is able to receive benefits from an insurance policy. </t>
         </is>
       </c>
-      <c r="D121" s="3" t="n"/>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
       <c r="E121" s="3" t="n"/>
-      <c r="F121" s="3" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
+      <c r="F121" s="3" t="n"/>
       <c r="G121" s="3" t="inlineStr">
         <is>
           <t>OMRSE:00000092</t>
@@ -7258,7 +7258,7 @@
           <t xml:space="preserve">A role that inheres in an organism that is able to receive benefits from an insurance policy. </t>
         </is>
       </c>
-      <c r="F122" t="inlineStr">
+      <c r="D122" t="inlineStr">
         <is>
           <t>role</t>
         </is>
@@ -7310,13 +7310,13 @@
           <t>A role relating to personal relationships or association between an individual and other individuals, including kinship relations, romantic, business, and social interactions.</t>
         </is>
       </c>
-      <c r="D123" s="2" t="n"/>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
       <c r="E123" s="2" t="n"/>
-      <c r="F123" s="2" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
+      <c r="F123" s="2" t="n"/>
       <c r="G123" s="2" t="inlineStr">
         <is>
           <t>NCIT_C92454</t>
@@ -7369,13 +7369,13 @@
           <t>A person who is exposed to an intervention.</t>
         </is>
       </c>
-      <c r="D124" s="2" t="n"/>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E124" s="2" t="n"/>
-      <c r="F124" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F124" s="2" t="n"/>
       <c r="G124" s="2" t="n"/>
       <c r="H124" s="2" t="n"/>
       <c r="I124" s="2" t="n"/>
@@ -7416,13 +7416,13 @@
           <t>A human population who are exposed to an intervention.</t>
         </is>
       </c>
-      <c r="D125" s="2" t="n"/>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>human population</t>
+        </is>
+      </c>
       <c r="E125" s="2" t="n"/>
-      <c r="F125" s="2" t="inlineStr">
-        <is>
-          <t>human population</t>
-        </is>
-      </c>
+      <c r="F125" s="2" t="n"/>
       <c r="G125" s="2" t="n"/>
       <c r="H125" s="2" t="n"/>
       <c r="I125" s="2" t="n"/>
@@ -7463,20 +7463,20 @@
           <t>A linguistic capability that is realised by using a language accurately and appropriately in more than one setting.</t>
         </is>
       </c>
-      <c r="D126" s="2" t="n"/>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">linguistic capability </t>
+        </is>
+      </c>
       <c r="E126" s="2" t="n"/>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">linguistic capability </t>
+          <t xml:space="preserve">Callers eligible for the study were adult cigarette smokers able to communicate in English </t>
         </is>
       </c>
       <c r="G126" s="2" t="n"/>
       <c r="H126" s="2" t="n"/>
-      <c r="I126" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Callers eligible for the study were adult cigarette smokers able to communicate in English </t>
-        </is>
-      </c>
+      <c r="I126" s="2" t="n"/>
       <c r="J126" s="2" t="n"/>
       <c r="K126" s="2" t="inlineStr">
         <is>
@@ -7522,13 +7522,13 @@
           <t>A social role in which the holder is given or creates authority to exert influence on other members of a social group.</t>
         </is>
       </c>
-      <c r="D127" s="2" t="n"/>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>social role</t>
+        </is>
+      </c>
       <c r="E127" s="2" t="n"/>
-      <c r="F127" s="2" t="inlineStr">
-        <is>
-          <t>social role</t>
-        </is>
-      </c>
+      <c r="F127" s="2" t="n"/>
       <c r="G127" s="2" t="n"/>
       <c r="H127" s="2" t="n"/>
       <c r="I127" s="2" t="n"/>
@@ -7577,7 +7577,7 @@
           <t>A mental capability that is realised in processes of communication involving language or in expressions of language.</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr">
+      <c r="D128" t="inlineStr">
         <is>
           <t>mental capability</t>
         </is>
@@ -7619,13 +7619,13 @@
           <t>Disabled for at least 12 months.</t>
         </is>
       </c>
-      <c r="D129" s="2" t="n"/>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>disabled</t>
+        </is>
+      </c>
       <c r="E129" s="2" t="n"/>
-      <c r="F129" s="2" t="inlineStr">
-        <is>
-          <t>disabled</t>
-        </is>
-      </c>
+      <c r="F129" s="2" t="n"/>
       <c r="G129" s="2" t="n"/>
       <c r="H129" s="2" t="n"/>
       <c r="I129" s="2" t="n"/>
@@ -7679,13 +7679,13 @@
           <t>A frequency of past behaviour that is below a threshold.</t>
         </is>
       </c>
-      <c r="D130" s="2" t="n"/>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>frequency of past behaviour</t>
+        </is>
+      </c>
       <c r="E130" s="2" t="n"/>
-      <c r="F130" s="2" t="inlineStr">
-        <is>
-          <t>frequency of past behaviour</t>
-        </is>
-      </c>
+      <c r="F130" s="2" t="n"/>
       <c r="G130" s="2" t="n"/>
       <c r="H130" s="2" t="n"/>
       <c r="I130" s="2" t="n"/>
@@ -7730,13 +7730,13 @@
           <t>A biological sex associated with the ability to produce male gametes.</t>
         </is>
       </c>
-      <c r="D131" s="2" t="n"/>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>biological sex</t>
+        </is>
+      </c>
       <c r="E131" s="2" t="n"/>
-      <c r="F131" s="2" t="inlineStr">
-        <is>
-          <t>biological sex</t>
-        </is>
-      </c>
+      <c r="F131" s="2" t="n"/>
       <c r="G131" s="2" t="n"/>
       <c r="H131" s="2" t="n"/>
       <c r="I131" s="2" t="n"/>
@@ -7785,13 +7785,13 @@
           <t>A gender identity as being male.</t>
         </is>
       </c>
-      <c r="D132" s="2" t="n"/>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>gender identity</t>
+        </is>
+      </c>
       <c r="E132" s="2" t="n"/>
-      <c r="F132" s="2" t="inlineStr">
-        <is>
-          <t>gender identity</t>
-        </is>
-      </c>
+      <c r="F132" s="2" t="n"/>
       <c r="G132" s="2" t="inlineStr">
         <is>
           <t>GSSO:000090</t>
@@ -7848,13 +7848,13 @@
           <t>A higher education student  role realised by currently studying for a masters degree.</t>
         </is>
       </c>
-      <c r="D133" s="3" t="n"/>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>higher education student role</t>
+        </is>
+      </c>
       <c r="E133" s="3" t="n"/>
-      <c r="F133" s="3" t="inlineStr">
-        <is>
-          <t>higher education student role</t>
-        </is>
-      </c>
+      <c r="F133" s="3" t="n"/>
       <c r="G133" s="3" t="n"/>
       <c r="H133" s="3" t="n"/>
       <c r="I133" s="3" t="n"/>
@@ -7903,13 +7903,13 @@
           <t>A higher education student  role realised by currently studying for a masters degree.</t>
         </is>
       </c>
-      <c r="D134" s="2" t="n"/>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>higher education student role</t>
+        </is>
+      </c>
       <c r="E134" s="2" t="n"/>
-      <c r="F134" s="2" t="inlineStr">
-        <is>
-          <t>higher education student role</t>
-        </is>
-      </c>
+      <c r="F134" s="2" t="n"/>
       <c r="G134" s="2" t="n"/>
       <c r="H134" s="2" t="n"/>
       <c r="I134" s="2" t="n"/>
@@ -7958,20 +7958,20 @@
           <t>A health status attribute that is having been prescribed the use of one or more drugs to improve, maintain or protect one's health.</t>
         </is>
       </c>
-      <c r="D135" s="2" t="n"/>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>health status attribute</t>
+        </is>
+      </c>
       <c r="E135" s="2" t="n"/>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>health status attribute</t>
+          <t>prescribed at least one antihypertensive medication, taking asthma preventer inhalers</t>
         </is>
       </c>
       <c r="G135" s="2" t="n"/>
       <c r="H135" s="2" t="n"/>
-      <c r="I135" s="2" t="inlineStr">
-        <is>
-          <t>prescribed at least one antihypertensive medication, taking asthma preventer inhalers</t>
-        </is>
-      </c>
+      <c r="I135" s="2" t="n"/>
       <c r="J135" s="2" t="inlineStr">
         <is>
           <t>This entity reflects having been prescribed a medication.  Actual use of the medicine would be captured as a behaviour</t>
@@ -8021,13 +8021,13 @@
           <t>A person living in  a household with at least one other person.</t>
         </is>
       </c>
-      <c r="D136" s="2" t="n"/>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E136" s="2" t="n"/>
-      <c r="F136" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F136" s="2" t="n"/>
       <c r="G136" s="2" t="n"/>
       <c r="H136" s="2" t="n"/>
       <c r="I136" s="2" t="n"/>
@@ -8080,11 +8080,15 @@
           <t>A member of a multi-person household where all of the household members are related.</t>
         </is>
       </c>
-      <c r="D137" s="2" t="n"/>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>member of a multi-person household</t>
+        </is>
+      </c>
       <c r="E137" s="2" t="n"/>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>member of a multi-person household</t>
+          <t>1) Co-habitating couple and their socially recognised children and elderly parents. 2) Co habitating couple with child and grandchild.</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -8093,11 +8097,7 @@
         </is>
       </c>
       <c r="H137" s="2" t="n"/>
-      <c r="I137" s="2" t="inlineStr">
-        <is>
-          <t>1) Co-habitating couple and their socially recognised children and elderly parents. 2) Co habitating couple with child and grandchild.</t>
-        </is>
-      </c>
+      <c r="I137" s="2" t="n"/>
       <c r="J137" s="2" t="n"/>
       <c r="K137" s="2" t="inlineStr">
         <is>
@@ -8143,20 +8143,20 @@
           <t>A member of a multi-person household where none of the household members are related.</t>
         </is>
       </c>
-      <c r="D138" s="2" t="n"/>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>member of a multi-person household</t>
+        </is>
+      </c>
       <c r="E138" s="2" t="n"/>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>member of a multi-person household</t>
+          <t>1) Two unrelated couples (unmarried couples). 2) Students sharing living accommodation. 3) Single professionals renting a room in a shared house.</t>
         </is>
       </c>
       <c r="G138" s="2" t="n"/>
       <c r="H138" s="2" t="n"/>
-      <c r="I138" s="2" t="inlineStr">
-        <is>
-          <t>1) Two unrelated couples (unmarried couples). 2) Students sharing living accommodation. 3) Single professionals renting a room in a shared house.</t>
-        </is>
-      </c>
+      <c r="I138" s="2" t="n"/>
       <c r="J138" s="2" t="n"/>
       <c r="K138" s="2" t="inlineStr">
         <is>
@@ -8202,20 +8202,20 @@
           <t>A member of a multi-person household where some household members are related.</t>
         </is>
       </c>
-      <c r="D139" s="2" t="n"/>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>member of a multi-person household</t>
+        </is>
+      </c>
       <c r="E139" s="2" t="n"/>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>member of a multi-person household</t>
+          <t>1) Cohabiting couple plus son and girlfriend. 2) Two brothers and their partners</t>
         </is>
       </c>
       <c r="G139" s="2" t="n"/>
       <c r="H139" s="2" t="n"/>
-      <c r="I139" s="2" t="inlineStr">
-        <is>
-          <t>1) Cohabiting couple plus son and girlfriend. 2) Two brothers and their partners</t>
-        </is>
-      </c>
+      <c r="I139" s="2" t="n"/>
       <c r="J139" s="2" t="n"/>
       <c r="K139" s="2" t="inlineStr">
         <is>
@@ -8261,20 +8261,20 @@
           <t>A member of a multi-person household where some household members belong to different generations.</t>
         </is>
       </c>
-      <c r="D140" s="2" t="n"/>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>member of a multi-person household</t>
+        </is>
+      </c>
       <c r="E140" s="2" t="n"/>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>member of a multi-person household</t>
+          <t>1) A family unit of a pair of adults and their socially recognized children. 2) Co-habitating couples plus socially recognised children and elderly parents or grandchildren.</t>
         </is>
       </c>
       <c r="G140" s="2" t="n"/>
       <c r="H140" s="2" t="n"/>
-      <c r="I140" s="2" t="inlineStr">
-        <is>
-          <t>1) A family unit of a pair of adults and their socially recognized children. 2) Co-habitating couples plus socially recognised children and elderly parents or grandchildren.</t>
-        </is>
-      </c>
+      <c r="I140" s="2" t="n"/>
       <c r="J140" s="2" t="inlineStr">
         <is>
           <t>A member of a multi-generational household lives with other people that are from more than one generation. A generation is all the people of about the same age within a society or within a particular family</t>
@@ -8324,13 +8324,13 @@
           <t>A person living alone in a household.</t>
         </is>
       </c>
-      <c r="D141" s="2" t="n"/>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E141" s="2" t="n"/>
-      <c r="F141" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F141" s="2" t="n"/>
       <c r="G141" s="2" t="n"/>
       <c r="H141" s="2" t="n"/>
       <c r="I141" s="2" t="n"/>
@@ -8379,7 +8379,7 @@
           <t>A personal capability that includes mental processes in its realisation.</t>
         </is>
       </c>
-      <c r="F142" t="inlineStr">
+      <c r="D142" t="inlineStr">
         <is>
           <t>personal capability</t>
         </is>
@@ -8421,13 +8421,13 @@
           <t>A parent who is female gender.</t>
         </is>
       </c>
-      <c r="D143" s="2" t="n"/>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>parent</t>
+        </is>
+      </c>
       <c r="E143" s="2" t="n"/>
-      <c r="F143" s="2" t="inlineStr">
-        <is>
-          <t>parent</t>
-        </is>
-      </c>
+      <c r="F143" s="2" t="n"/>
       <c r="G143" s="2" t="n"/>
       <c r="H143" s="2" t="n"/>
       <c r="I143" s="2" t="n"/>
@@ -8476,13 +8476,13 @@
           <t xml:space="preserve">A family member who is a child relation of one's sibling and is male gender. </t>
         </is>
       </c>
-      <c r="D144" s="2" t="n"/>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>family member</t>
+        </is>
+      </c>
       <c r="E144" s="2" t="n"/>
-      <c r="F144" s="2" t="inlineStr">
-        <is>
-          <t>family member</t>
-        </is>
-      </c>
+      <c r="F144" s="2" t="n"/>
       <c r="G144" s="2" t="n"/>
       <c r="H144" s="2" t="n"/>
       <c r="I144" s="2" t="n"/>
@@ -8531,13 +8531,13 @@
           <t>A family member who is a child relation of one's sibling and is female gender.</t>
         </is>
       </c>
-      <c r="D145" s="2" t="n"/>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>family member</t>
+        </is>
+      </c>
       <c r="E145" s="2" t="n"/>
-      <c r="F145" s="2" t="inlineStr">
-        <is>
-          <t>family member</t>
-        </is>
-      </c>
+      <c r="F145" s="2" t="n"/>
       <c r="G145" s="2" t="n"/>
       <c r="H145" s="2" t="n"/>
       <c r="I145" s="2" t="n"/>
@@ -8586,13 +8586,13 @@
           <t>A self-identity as not having a particular gender.</t>
         </is>
       </c>
-      <c r="D146" s="2" t="n"/>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>self-identity</t>
+        </is>
+      </c>
       <c r="E146" s="2" t="n"/>
-      <c r="F146" s="2" t="inlineStr">
-        <is>
-          <t>self-identity</t>
-        </is>
-      </c>
+      <c r="F146" s="2" t="n"/>
       <c r="G146" s="2" t="inlineStr">
         <is>
           <t>GSSO:002331</t>
@@ -8645,13 +8645,13 @@
           <t>A gender identity as having a gender that is not well-described by the binary categories of male or female.</t>
         </is>
       </c>
-      <c r="D147" s="2" t="n"/>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>gender identity</t>
+        </is>
+      </c>
       <c r="E147" s="2" t="n"/>
-      <c r="F147" s="2" t="inlineStr">
-        <is>
-          <t>gender identity</t>
-        </is>
-      </c>
+      <c r="F147" s="2" t="n"/>
       <c r="G147" s="2" t="inlineStr">
         <is>
           <t>GSSO:002328</t>
@@ -8704,13 +8704,13 @@
           <t>A personal attribute inhering in a person by virtue of that person not having a paid job and not currently seeking to begin participating in an employment process.</t>
         </is>
       </c>
-      <c r="D148" s="2" t="n"/>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E148" s="2" t="n"/>
-      <c r="F148" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F148" s="2" t="n"/>
       <c r="G148" s="2" t="n"/>
       <c r="H148" s="2" t="n"/>
       <c r="I148" s="2" t="n"/>
@@ -8759,13 +8759,13 @@
           <t>A personal attribute inhering in a person by virtue of that person not bearing a role realised in an employment process, due to being unable to work due to illness or disability.</t>
         </is>
       </c>
-      <c r="D149" s="2" t="n"/>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E149" s="2" t="n"/>
-      <c r="F149" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F149" s="2" t="n"/>
       <c r="G149" s="2" t="n"/>
       <c r="H149" s="2" t="n"/>
       <c r="I149" s="2" t="n"/>
@@ -8814,13 +8814,13 @@
           <t>A data item about the number of people in a population.</t>
         </is>
       </c>
-      <c r="D150" s="2" t="n"/>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
       <c r="E150" s="2" t="n"/>
-      <c r="F150" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
+      <c r="F150" s="2" t="n"/>
       <c r="G150" s="2" t="n"/>
       <c r="H150" s="2" t="n"/>
       <c r="I150" s="2" t="n"/>
@@ -8861,13 +8861,13 @@
           <t>The number of years a person spent engaged in an education process.</t>
         </is>
       </c>
-      <c r="D151" s="2" t="n"/>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
       <c r="E151" s="2" t="n"/>
-      <c r="F151" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
+      <c r="F151" s="2" t="n"/>
       <c r="G151" s="2" t="n"/>
       <c r="H151" s="2" t="n"/>
       <c r="I151" s="2" t="n"/>
@@ -8920,13 +8920,13 @@
           <t>A personal role that is realised in a person by doing a specified type of work or working in a specified way.</t>
         </is>
       </c>
-      <c r="D152" s="2" t="n"/>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>personal role</t>
+        </is>
+      </c>
       <c r="E152" s="2" t="n"/>
-      <c r="F152" s="2" t="inlineStr">
-        <is>
-          <t>personal role</t>
-        </is>
-      </c>
+      <c r="F152" s="2" t="n"/>
       <c r="G152" s="2" t="n"/>
       <c r="H152" s="2" t="n"/>
       <c r="I152" s="2" t="n"/>
@@ -8975,13 +8975,13 @@
           <t>A person who lives in a residential facility they do not own  with the agreement of the residential facility owner, by virtue of the occupier bearing a role realised in an employment process.</t>
         </is>
       </c>
-      <c r="D153" s="2" t="n"/>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E153" s="2" t="n"/>
-      <c r="F153" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F153" s="2" t="n"/>
       <c r="G153" s="2" t="n"/>
       <c r="H153" s="2" t="n"/>
       <c r="I153" s="2" t="n"/>
@@ -9030,20 +9030,20 @@
           <t>A role which inheres in a person and is realised by performing the activities deemed appropriate for that particular role as specified in the organisation rules.</t>
         </is>
       </c>
-      <c r="D154" s="2" t="n"/>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
       <c r="E154" s="2" t="n"/>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>Scout leader, club chairperson</t>
         </is>
       </c>
       <c r="G154" s="2" t="n"/>
       <c r="H154" s="2" t="n"/>
-      <c r="I154" s="2" t="inlineStr">
-        <is>
-          <t>Scout leader, club chairperson</t>
-        </is>
-      </c>
+      <c r="I154" s="2" t="n"/>
       <c r="J154" s="2" t="n"/>
       <c r="K154" s="2" t="inlineStr">
         <is>
@@ -9089,13 +9089,13 @@
           <t>A sexual orientation of an individual who is sure of their sexual orientation and reports it as other than asexual, bisexual, heterosexual, homosexual, queer or questioning.</t>
         </is>
       </c>
-      <c r="D155" s="2" t="n"/>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>sexual orientation</t>
+        </is>
+      </c>
       <c r="E155" s="2" t="n"/>
-      <c r="F155" s="2" t="inlineStr">
-        <is>
-          <t>sexual orientation</t>
-        </is>
-      </c>
+      <c r="F155" s="2" t="n"/>
       <c r="G155" s="2" t="n"/>
       <c r="H155" s="2" t="n"/>
       <c r="I155" s="2" t="n"/>
@@ -9144,13 +9144,13 @@
           <t>A social group that is part of a person’s social environmental system and with which the person does not identify.</t>
         </is>
       </c>
-      <c r="D156" s="2" t="n"/>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>social group</t>
+        </is>
+      </c>
       <c r="E156" s="2" t="n"/>
-      <c r="F156" s="2" t="inlineStr">
-        <is>
-          <t>social group</t>
-        </is>
-      </c>
+      <c r="F156" s="2" t="n"/>
       <c r="G156" s="2" t="n"/>
       <c r="H156" s="2" t="n"/>
       <c r="I156" s="2" t="n"/>
@@ -9191,13 +9191,13 @@
           <t>A patient role which inheres in a person and is realized by coming to a healthcare facility for diagnosis or treatment but not being admitted for an overnight stay.</t>
         </is>
       </c>
-      <c r="D157" s="2" t="n"/>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>patient role</t>
+        </is>
+      </c>
       <c r="E157" s="2" t="n"/>
-      <c r="F157" s="2" t="inlineStr">
-        <is>
-          <t>patient role</t>
-        </is>
-      </c>
+      <c r="F157" s="2" t="n"/>
       <c r="G157" s="2" t="n"/>
       <c r="H157" s="2" t="n"/>
       <c r="I157" s="2" t="n"/>
@@ -9246,13 +9246,13 @@
           <t>A person or organization that participates in an ownership process wherein they realize their role as owner by exercising their right to use, sell, rent, or gift an object.</t>
         </is>
       </c>
-      <c r="D158" s="2" t="n"/>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
       <c r="E158" s="2" t="n"/>
-      <c r="F158" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="F158" s="2" t="n"/>
       <c r="G158" s="2" t="inlineStr">
         <is>
           <t>owner in the Sustainable Development Goals Interface Ontology (SDGIO:00010028)</t>
@@ -9309,13 +9309,13 @@
           <t>A person who lives in a residential facility of which they are the residential facility owner</t>
         </is>
       </c>
-      <c r="D159" s="2" t="n"/>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E159" s="2" t="n"/>
-      <c r="F159" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F159" s="2" t="n"/>
       <c r="G159" s="2" t="n"/>
       <c r="H159" s="2" t="n"/>
       <c r="I159" s="2" t="n"/>
@@ -9365,13 +9365,13 @@
           <t xml:space="preserve">A family member who is a key caretaker or immediate progenitor of a child. </t>
         </is>
       </c>
-      <c r="D160" s="2" t="n"/>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>family member</t>
+        </is>
+      </c>
       <c r="E160" s="2" t="n"/>
-      <c r="F160" s="2" t="inlineStr">
-        <is>
-          <t>family member</t>
-        </is>
-      </c>
+      <c r="F160" s="2" t="n"/>
       <c r="G160" s="2" t="inlineStr">
         <is>
           <t>GSSO:001953</t>
@@ -9424,13 +9424,13 @@
           <t>An interpersonal role that is realised through a process of promoting and supporting the physical, emotional, social, and intellectual development of a child from infancy to adulthood.</t>
         </is>
       </c>
-      <c r="D161" s="2" t="n"/>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>interpersonal role</t>
+        </is>
+      </c>
       <c r="E161" s="2" t="n"/>
-      <c r="F161" s="2" t="inlineStr">
-        <is>
-          <t>interpersonal role</t>
-        </is>
-      </c>
+      <c r="F161" s="2" t="n"/>
       <c r="G161" s="2" t="n"/>
       <c r="H161" s="2" t="n"/>
       <c r="I161" s="2" t="n"/>
@@ -9483,13 +9483,13 @@
           <t>A personal history part that includes a behaviour.</t>
         </is>
       </c>
-      <c r="D162" s="2" t="n"/>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>personal history part</t>
+        </is>
+      </c>
       <c r="E162" s="2" t="n"/>
-      <c r="F162" s="2" t="inlineStr">
-        <is>
-          <t>personal history part</t>
-        </is>
-      </c>
+      <c r="F162" s="2" t="n"/>
       <c r="G162" s="2" t="n"/>
       <c r="H162" s="2" t="n"/>
       <c r="I162" s="2" t="n"/>
@@ -9534,13 +9534,13 @@
           <t>A past behaviour that is the target of an intervention.</t>
         </is>
       </c>
-      <c r="D163" s="2" t="n"/>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">past behaviour </t>
+        </is>
+      </c>
       <c r="E163" s="2" t="n"/>
-      <c r="F163" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">past behaviour </t>
-        </is>
-      </c>
+      <c r="F163" s="2" t="n"/>
       <c r="G163" s="2" t="n"/>
       <c r="H163" s="2" t="n"/>
       <c r="I163" s="2" t="n"/>
@@ -9585,7 +9585,7 @@
           <t>A role which inheres in a person and is realized by being under the care of a physician or health care provider.</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr">
+      <c r="D164" t="inlineStr">
         <is>
           <t>role</t>
         </is>
@@ -9628,13 +9628,13 @@
           <t>A &lt;human population&gt; whose members are people with an intervention source role for a specified intervention.</t>
         </is>
       </c>
-      <c r="D165" s="2" t="n"/>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>human population</t>
+        </is>
+      </c>
       <c r="E165" s="2" t="n"/>
-      <c r="F165" s="2" t="inlineStr">
-        <is>
-          <t>human population</t>
-        </is>
-      </c>
+      <c r="F165" s="2" t="n"/>
       <c r="G165" s="2" t="n"/>
       <c r="H165" s="2" t="n"/>
       <c r="I165" s="2" t="n"/>
@@ -9675,7 +9675,7 @@
           <t>An extended organism that is a member of the species Homo sapiens.</t>
         </is>
       </c>
-      <c r="F166" t="inlineStr">
+      <c r="D166" t="inlineStr">
         <is>
           <t>extended organism</t>
         </is>
@@ -9707,13 +9707,13 @@
           <t>A &lt;person&gt; who is part of a social environmental system.</t>
         </is>
       </c>
-      <c r="D167" s="2" t="n"/>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E167" s="2" t="n"/>
-      <c r="F167" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F167" s="2" t="n"/>
       <c r="G167" s="2" t="n"/>
       <c r="H167" s="2" t="n"/>
       <c r="I167" s="2" t="n"/>
@@ -9754,13 +9754,13 @@
           <t>A specifically dependent continuant that inheres in a person.</t>
         </is>
       </c>
-      <c r="D168" s="2" t="n"/>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>specifically dependent continuant</t>
+        </is>
+      </c>
       <c r="E168" s="2" t="n"/>
-      <c r="F168" s="2" t="inlineStr">
-        <is>
-          <t>specifically dependent continuant</t>
-        </is>
-      </c>
+      <c r="F168" s="2" t="n"/>
       <c r="G168" s="2" t="n"/>
       <c r="H168" s="2" t="n"/>
       <c r="I168" s="2" t="n"/>
@@ -9811,12 +9811,12 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
+          <t>bodily disposition</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
           <t>The ability of someone to perform some useful and/or beneficial activity.</t>
-        </is>
-      </c>
-      <c r="F169" t="inlineStr">
-        <is>
-          <t>bodily disposition</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
@@ -9852,13 +9852,13 @@
           <t>A history that is of a person.</t>
         </is>
       </c>
-      <c r="D170" s="2" t="n"/>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>history</t>
+        </is>
+      </c>
       <c r="E170" s="2" t="n"/>
-      <c r="F170" s="2" t="inlineStr">
-        <is>
-          <t>history</t>
-        </is>
-      </c>
+      <c r="F170" s="2" t="n"/>
       <c r="G170" s="2" t="n"/>
       <c r="H170" s="2" t="n"/>
       <c r="I170" s="2" t="n"/>
@@ -9899,13 +9899,13 @@
           <t xml:space="preserve">A personal history part that includes a change from a less desired behaviour pattern to a more desired behaviour pattern followed by a temporary reversion to the previous behaviour pattern. </t>
         </is>
       </c>
-      <c r="D171" s="2" t="n"/>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>personal history part</t>
+        </is>
+      </c>
       <c r="E171" s="2" t="n"/>
-      <c r="F171" s="2" t="inlineStr">
-        <is>
-          <t>personal history part</t>
-        </is>
-      </c>
+      <c r="F171" s="2" t="n"/>
       <c r="G171" s="2" t="n"/>
       <c r="H171" s="2" t="n"/>
       <c r="I171" s="2" t="n"/>
@@ -9954,13 +9954,13 @@
           <t xml:space="preserve">A personal history part that includes experience of events that influence behaviour. </t>
         </is>
       </c>
-      <c r="D172" s="2" t="n"/>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>personal history part</t>
+        </is>
+      </c>
       <c r="E172" s="2" t="n"/>
-      <c r="F172" s="2" t="inlineStr">
-        <is>
-          <t>personal history part</t>
-        </is>
-      </c>
+      <c r="F172" s="2" t="n"/>
       <c r="G172" s="2" t="n"/>
       <c r="H172" s="2" t="n"/>
       <c r="I172" s="2" t="n"/>
@@ -10009,13 +10009,13 @@
           <t>A personal history part of exposure to an intervention targeting the same outcome as the current intervention.</t>
         </is>
       </c>
-      <c r="D173" s="2" t="n"/>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>personal history part</t>
+        </is>
+      </c>
       <c r="E173" s="2" t="n"/>
-      <c r="F173" s="2" t="inlineStr">
-        <is>
-          <t>personal history part</t>
-        </is>
-      </c>
+      <c r="F173" s="2" t="n"/>
       <c r="G173" s="2" t="n"/>
       <c r="H173" s="2" t="n"/>
       <c r="I173" s="2" t="n"/>
@@ -10064,13 +10064,13 @@
           <t>A personal history part  that includes exposure to a prior intervention targeting the same outcome behaviour as the current intervention.</t>
         </is>
       </c>
-      <c r="D174" s="2" t="n"/>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>personal history part</t>
+        </is>
+      </c>
       <c r="E174" s="2" t="n"/>
-      <c r="F174" s="2" t="inlineStr">
-        <is>
-          <t>personal history part</t>
-        </is>
-      </c>
+      <c r="F174" s="2" t="n"/>
       <c r="G174" s="2" t="n"/>
       <c r="H174" s="2" t="n"/>
       <c r="I174" s="2" t="n"/>
@@ -10119,13 +10119,13 @@
           <t>A personal history part that includes exposure to the same intervention as the current intervention.</t>
         </is>
       </c>
-      <c r="D175" s="2" t="n"/>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>personal history part</t>
+        </is>
+      </c>
       <c r="E175" s="2" t="n"/>
-      <c r="F175" s="2" t="inlineStr">
-        <is>
-          <t>personal history part</t>
-        </is>
-      </c>
+      <c r="F175" s="2" t="n"/>
       <c r="G175" s="2" t="n"/>
       <c r="H175" s="2" t="n"/>
       <c r="I175" s="2" t="n"/>
@@ -10178,17 +10178,17 @@
           <t>A process that is part of a personal history.</t>
         </is>
       </c>
-      <c r="D176" s="2" t="n"/>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
           <t>'process' and 'part of' some 'personal history'</t>
         </is>
       </c>
-      <c r="F176" s="2" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
+      <c r="F176" s="2" t="n"/>
       <c r="G176" s="2" t="n"/>
       <c r="H176" s="2" t="n"/>
       <c r="I176" s="2" t="n"/>
@@ -10229,13 +10229,13 @@
           <t xml:space="preserve">A personal history part  that includes exposure to one or more interventions. </t>
         </is>
       </c>
-      <c r="D177" s="2" t="n"/>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>personal history part</t>
+        </is>
+      </c>
       <c r="E177" s="2" t="n"/>
-      <c r="F177" s="2" t="inlineStr">
-        <is>
-          <t>personal history part</t>
-        </is>
-      </c>
+      <c r="F177" s="2" t="n"/>
       <c r="G177" s="2" t="n"/>
       <c r="H177" s="2" t="n"/>
       <c r="I177" s="2" t="n"/>
@@ -10284,20 +10284,20 @@
           <t>An attribute reflecting a person's mental dispositions, mental processes or capabilities.</t>
         </is>
       </c>
-      <c r="D178" s="2" t="n"/>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E178" s="2" t="n"/>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>personal attribute</t>
+          <t>low motivation to quit,  low self efficacy for physical activity, negative attitudes to healthy eating, contemplation stage of change, low numeracy</t>
         </is>
       </c>
       <c r="G178" s="2" t="n"/>
       <c r="H178" s="2" t="n"/>
-      <c r="I178" s="2" t="inlineStr">
-        <is>
-          <t>low motivation to quit,  low self efficacy for physical activity, negative attitudes to healthy eating, contemplation stage of change, low numeracy</t>
-        </is>
-      </c>
+      <c r="I178" s="2" t="n"/>
       <c r="J178" s="2" t="n"/>
       <c r="K178" s="2" t="inlineStr">
         <is>
@@ -10345,18 +10345,18 @@
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>A role can be assigned without being realised. A person realises a role by doing something.</t>
+          <t>role</t>
         </is>
       </c>
       <c r="E179" s="2" t="n"/>
-      <c r="F179" s="2" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
+      <c r="F179" s="2" t="n"/>
       <c r="G179" s="2" t="n"/>
       <c r="H179" s="2" t="n"/>
-      <c r="I179" s="2" t="n"/>
+      <c r="I179" s="2" t="inlineStr">
+        <is>
+          <t>A role can be assigned without being realised. A person realises a role by doing something.</t>
+        </is>
+      </c>
       <c r="J179" s="2" t="inlineStr">
         <is>
           <t>A role can be assigned without being realised. A person realises a role by doing something.</t>
@@ -10398,20 +10398,20 @@
           <t>A disposition to undergo undesirable change in response to exposure to another entity.</t>
         </is>
       </c>
-      <c r="D180" s="2" t="n"/>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>disposition</t>
+        </is>
+      </c>
       <c r="E180" s="2" t="n"/>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>disposition</t>
+          <t>susceptibility to addiction, vulnerability to depression</t>
         </is>
       </c>
       <c r="G180" s="2" t="n"/>
       <c r="H180" s="2" t="n"/>
-      <c r="I180" s="2" t="inlineStr">
-        <is>
-          <t>susceptibility to addiction, vulnerability to depression</t>
-        </is>
-      </c>
+      <c r="I180" s="2" t="n"/>
       <c r="J180" s="2" t="n"/>
       <c r="K180" s="2" t="inlineStr">
         <is>
@@ -10457,13 +10457,13 @@
           <t>A personal vulnerability towards performing a behaviour that causes net harm.</t>
         </is>
       </c>
-      <c r="D181" s="2" t="n"/>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>personal vulnerability</t>
+        </is>
+      </c>
       <c r="E181" s="2" t="n"/>
-      <c r="F181" s="2" t="inlineStr">
-        <is>
-          <t>personal vulnerability</t>
-        </is>
-      </c>
+      <c r="F181" s="2" t="n"/>
       <c r="G181" s="2" t="n"/>
       <c r="H181" s="2" t="inlineStr">
         <is>
@@ -10516,13 +10516,13 @@
           <t>A geographic location in which a person resides.</t>
         </is>
       </c>
-      <c r="D182" s="2" t="n"/>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>geographic location</t>
+        </is>
+      </c>
       <c r="E182" s="2" t="n"/>
-      <c r="F182" s="2" t="inlineStr">
-        <is>
-          <t>geographic location</t>
-        </is>
-      </c>
+      <c r="F182" s="2" t="n"/>
       <c r="G182" s="2" t="n"/>
       <c r="H182" s="2" t="n"/>
       <c r="I182" s="2" t="n"/>
@@ -10571,7 +10571,7 @@
           <t>An insured party role that inheres in a person who participates in the creation of the insurance contract and is eligible to receive benefits as specified by the insurance contract.</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr">
+      <c r="D183" t="inlineStr">
         <is>
           <t>insured party role</t>
         </is>
@@ -10613,21 +10613,21 @@
           <t xml:space="preserve">A data item that is about the number or extent of something in a population. </t>
         </is>
       </c>
-      <c r="D184" s="2" t="n"/>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
       <c r="E184" s="2" t="n"/>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>data item</t>
+          <t>Percentage of highly educated individuals in a population. 
+Mean age in a population.</t>
         </is>
       </c>
       <c r="G184" s="2" t="n"/>
       <c r="H184" s="2" t="n"/>
-      <c r="I184" s="2" t="inlineStr">
-        <is>
-          <t>Percentage of highly educated individuals in a population. 
-Mean age in a population.</t>
-        </is>
-      </c>
+      <c r="I184" s="2" t="n"/>
       <c r="J184" s="2" t="n"/>
       <c r="K184" s="2" t="n"/>
       <c r="L184" s="2" t="n"/>
@@ -10661,13 +10661,13 @@
           <t>A student or trainee role realised by  currently learning at an initial level of organised instruction, primarily to familiarise the bearer to the school-type environment.</t>
         </is>
       </c>
-      <c r="D185" s="2" t="n"/>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>student or trainee role</t>
+        </is>
+      </c>
       <c r="E185" s="2" t="n"/>
-      <c r="F185" s="2" t="inlineStr">
-        <is>
-          <t>student or trainee role</t>
-        </is>
-      </c>
+      <c r="F185" s="2" t="n"/>
       <c r="G185" s="2" t="n"/>
       <c r="H185" s="2" t="n"/>
       <c r="I185" s="2" t="n"/>
@@ -10716,13 +10716,13 @@
           <t>A &lt;disposition&gt; that decreases the likelihood of engaging with harmful behaviour.</t>
         </is>
       </c>
-      <c r="D186" s="2" t="n"/>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>disposition</t>
+        </is>
+      </c>
       <c r="E186" s="2" t="n"/>
-      <c r="F186" s="2" t="inlineStr">
-        <is>
-          <t>disposition</t>
-        </is>
-      </c>
+      <c r="F186" s="2" t="n"/>
       <c r="G186" s="2" t="n"/>
       <c r="H186" s="2" t="n"/>
       <c r="I186" s="2" t="n"/>
@@ -10771,7 +10771,7 @@
           <t>A specifically dependent continuant that, in contrast to roles and dispositions, does not require any further process in order to be realized.</t>
         </is>
       </c>
-      <c r="F187" t="inlineStr">
+      <c r="D187" t="inlineStr">
         <is>
           <t>specifically dependent continuant</t>
         </is>
@@ -10803,20 +10803,20 @@
           <t>A data item about the number of units of a valuable material resource possessed by a person.</t>
         </is>
       </c>
-      <c r="D188" s="2" t="n"/>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
       <c r="E188" s="2" t="n"/>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>data item</t>
+          <t>12 acres, a flock of 20 goats</t>
         </is>
       </c>
       <c r="G188" s="2" t="n"/>
       <c r="H188" s="2" t="n"/>
-      <c r="I188" s="2" t="inlineStr">
-        <is>
-          <t>12 acres, a flock of 20 goats</t>
-        </is>
-      </c>
+      <c r="I188" s="2" t="n"/>
       <c r="J188" s="2" t="n"/>
       <c r="K188" s="2" t="inlineStr">
         <is>
@@ -10866,13 +10866,13 @@
           <t>A sexual orientation that is not exclusively homosexual or heterosexual, or of a person who does not identify with heterosexual, homosexual or bisexual labels.</t>
         </is>
       </c>
-      <c r="D189" s="2" t="n"/>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>sexual orientation</t>
+        </is>
+      </c>
       <c r="E189" s="2" t="n"/>
-      <c r="F189" s="2" t="inlineStr">
-        <is>
-          <t>sexual orientation</t>
-        </is>
-      </c>
+      <c r="F189" s="2" t="n"/>
       <c r="G189" s="2" t="inlineStr">
         <is>
           <t>NCIT_C155691</t>
@@ -10925,13 +10925,13 @@
           <t xml:space="preserve">A self-identity as being in the process of exploring one's sexual orientation. </t>
         </is>
       </c>
-      <c r="D190" s="2" t="n"/>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>self-identity</t>
+        </is>
+      </c>
       <c r="E190" s="2" t="n"/>
-      <c r="F190" s="2" t="inlineStr">
-        <is>
-          <t>self-identity</t>
-        </is>
-      </c>
+      <c r="F190" s="2" t="n"/>
       <c r="G190" s="2" t="inlineStr">
         <is>
           <t>NCIT_C155692</t>
@@ -10984,13 +10984,13 @@
           <t>A personal attribute that is whether an individual is connected or associated with another through romantic attraction or marriage.</t>
         </is>
       </c>
-      <c r="D191" s="2" t="n"/>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E191" s="2" t="n"/>
-      <c r="F191" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F191" s="2" t="n"/>
       <c r="G191" s="2" t="n"/>
       <c r="H191" s="2" t="n"/>
       <c r="I191" s="2" t="n"/>
@@ -11039,11 +11039,15 @@
           <t xml:space="preserve">A personal attribute that is belonging to a group that is characterised by the practice of a common religion by the group members. </t>
         </is>
       </c>
-      <c r="D192" s="2" t="n"/>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E192" s="2" t="n"/>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>personal attribute</t>
+          <t xml:space="preserve"> Religion Baptist 157 (37.0%) 163 (40.3%) Catholic 54 (12.7%) 60 (14.9%) Muslim 39 (9.2%) </t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -11052,11 +11056,7 @@
         </is>
       </c>
       <c r="H192" s="2" t="n"/>
-      <c r="I192" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Religion Baptist 157 (37.0%) 163 (40.3%) Catholic 54 (12.7%) 60 (14.9%) Muslim 39 (9.2%) </t>
-        </is>
-      </c>
+      <c r="I192" s="2" t="n"/>
       <c r="J192" s="2" t="inlineStr">
         <is>
           <t>presented in aggregated form as proportion/percentage belonging to a specified religious group</t>
@@ -11106,13 +11106,13 @@
           <t>A person who lives in a residential facility they do not own without paying an agreed sum of money to the residential facility owner.</t>
         </is>
       </c>
-      <c r="D193" s="2" t="n"/>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E193" s="2" t="n"/>
-      <c r="F193" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F193" s="2" t="n"/>
       <c r="G193" s="2" t="n"/>
       <c r="H193" s="2" t="n"/>
       <c r="I193" s="2" t="n"/>
@@ -11161,20 +11161,20 @@
           <t>A rent-free occupier who lives in the residential facility without the agreement of the residential facility owner.</t>
         </is>
       </c>
-      <c r="D194" s="2" t="n"/>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>rent-free occupier</t>
+        </is>
+      </c>
       <c r="E194" s="2" t="n"/>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>rent-free occupier</t>
+          <t>squatters</t>
         </is>
       </c>
       <c r="G194" s="2" t="n"/>
       <c r="H194" s="2" t="n"/>
-      <c r="I194" s="2" t="inlineStr">
-        <is>
-          <t>squatters</t>
-        </is>
-      </c>
+      <c r="I194" s="2" t="n"/>
       <c r="J194" s="2" t="n"/>
       <c r="K194" s="2" t="inlineStr">
         <is>
@@ -11220,13 +11220,13 @@
           <t>A person who lives in a residential facility they do not own in return for paying an agreed sum of money to the residential facility owner</t>
         </is>
       </c>
-      <c r="D195" s="2" t="n"/>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E195" s="2" t="n"/>
-      <c r="F195" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F195" s="2" t="n"/>
       <c r="G195" s="2" t="n"/>
       <c r="H195" s="2" t="n"/>
       <c r="I195" s="2" t="n"/>
@@ -11275,20 +11275,20 @@
           <t>A renter who lives in a residential facility where the residential facility owner decides who can live in the residential facility based on their perceived social or economic needs.</t>
         </is>
       </c>
-      <c r="D196" s="2" t="n"/>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>renter</t>
+        </is>
+      </c>
       <c r="E196" s="2" t="n"/>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>renter</t>
+          <t>renters living in "public housing"[US], council housing [UK], housing association properties, non-profit organisation, alms house occupier</t>
         </is>
       </c>
       <c r="G196" s="2" t="n"/>
       <c r="H196" s="2" t="n"/>
-      <c r="I196" s="2" t="inlineStr">
-        <is>
-          <t>renters living in "public housing"[US], council housing [UK], housing association properties, non-profit organisation, alms house occupier</t>
-        </is>
-      </c>
+      <c r="I196" s="2" t="n"/>
       <c r="J196" s="2" t="n"/>
       <c r="K196" s="2" t="inlineStr">
         <is>
@@ -11334,13 +11334,13 @@
           <t>An owner of a residential facility.</t>
         </is>
       </c>
-      <c r="D197" s="2" t="n"/>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
       <c r="E197" s="2" t="n"/>
-      <c r="F197" s="2" t="inlineStr">
-        <is>
-          <t>owner</t>
-        </is>
-      </c>
+      <c r="F197" s="2" t="n"/>
       <c r="G197" s="2" t="n"/>
       <c r="H197" s="2" t="n"/>
       <c r="I197" s="2" t="n"/>
@@ -11389,13 +11389,13 @@
           <t>A personal attribute inhering in a person who previously bore a role realised in an employment process but has withdrawn from that employment process, having concluded their working or professional career.</t>
         </is>
       </c>
-      <c r="D198" s="2" t="n"/>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E198" s="2" t="n"/>
-      <c r="F198" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F198" s="2" t="n"/>
       <c r="G198" s="2" t="n"/>
       <c r="H198" s="2" t="n"/>
       <c r="I198" s="2" t="n"/>
@@ -11444,7 +11444,7 @@
           <t>b is a role means: b is a realizable entity and b exists because there is some single bearer that is in some special physical, social, or institutional set of circumstances in which this bearer does not have to beand b is not such that, if it ceases to exist, then the physical make-up of the bearer is thereby changed.</t>
         </is>
       </c>
-      <c r="F199" t="inlineStr">
+      <c r="D199" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
@@ -11476,13 +11476,13 @@
           <t xml:space="preserve">A student or trainee role realised by currently learning at a primary or secondary education level in an institutional, organised setting. </t>
         </is>
       </c>
-      <c r="D200" s="3" t="n"/>
+      <c r="D200" s="3" t="inlineStr">
+        <is>
+          <t>student or trainee role</t>
+        </is>
+      </c>
       <c r="E200" s="3" t="n"/>
-      <c r="F200" s="3" t="inlineStr">
-        <is>
-          <t>student or trainee role</t>
-        </is>
-      </c>
+      <c r="F200" s="3" t="n"/>
       <c r="G200" s="3" t="n"/>
       <c r="H200" s="3" t="n"/>
       <c r="I200" s="3" t="n"/>
@@ -11531,13 +11531,13 @@
           <t xml:space="preserve">A student or trainee role realised by currently learning at a primary or secondary education level in an institutional, organised setting. </t>
         </is>
       </c>
-      <c r="D201" s="2" t="n"/>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>student or trainee role</t>
+        </is>
+      </c>
       <c r="E201" s="2" t="n"/>
-      <c r="F201" s="2" t="inlineStr">
-        <is>
-          <t>student or trainee role</t>
-        </is>
-      </c>
+      <c r="F201" s="2" t="n"/>
       <c r="G201" s="2" t="n"/>
       <c r="H201" s="2" t="n"/>
       <c r="I201" s="2" t="n"/>
@@ -11586,13 +11586,13 @@
           <t>A person who has at least one parent who is an immigrant.</t>
         </is>
       </c>
-      <c r="D202" s="2" t="n"/>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
       <c r="E202" s="2" t="n"/>
-      <c r="F202" s="2" t="inlineStr">
-        <is>
-          <t>person</t>
-        </is>
-      </c>
+      <c r="F202" s="2" t="n"/>
       <c r="G202" s="2" t="n"/>
       <c r="H202" s="2" t="n"/>
       <c r="I202" s="2" t="n"/>
@@ -11641,13 +11641,13 @@
           <t>An employment status realised by a person earning income directly from customers, clients, or other organisations rather than as a specified salary or wages from an employer.</t>
         </is>
       </c>
-      <c r="D203" s="2" t="n"/>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>employment status</t>
+        </is>
+      </c>
       <c r="E203" s="2" t="n"/>
-      <c r="F203" s="2" t="inlineStr">
-        <is>
-          <t>employment status</t>
-        </is>
-      </c>
+      <c r="F203" s="2" t="n"/>
       <c r="G203" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">NCIT_C116000 </t>
@@ -11704,7 +11704,7 @@
           <t>An identity that a person has about themselves.</t>
         </is>
       </c>
-      <c r="F204" t="inlineStr">
+      <c r="D204" t="inlineStr">
         <is>
           <t>identity</t>
         </is>
@@ -11736,13 +11736,13 @@
           <t xml:space="preserve">A personal attribute that is the pattern of a person's emotional, romantic and/or sexual attractions. </t>
         </is>
       </c>
-      <c r="D205" s="2" t="n"/>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E205" s="2" t="n"/>
-      <c r="F205" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F205" s="2" t="n"/>
       <c r="G205" s="2" t="inlineStr">
         <is>
           <t>NCIT_C84361</t>
@@ -11795,13 +11795,13 @@
           <t>A family member with whom the subject shares a parent.</t>
         </is>
       </c>
-      <c r="D206" s="2" t="n"/>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>family member</t>
+        </is>
+      </c>
       <c r="E206" s="2" t="n"/>
-      <c r="F206" s="2" t="inlineStr">
-        <is>
-          <t>family member</t>
-        </is>
-      </c>
+      <c r="F206" s="2" t="n"/>
       <c r="G206" s="2" t="n"/>
       <c r="H206" s="2" t="n"/>
       <c r="I206" s="2" t="n"/>
@@ -11851,13 +11851,13 @@
           <t>A relationship status where the individual is not in a relationship with another person.</t>
         </is>
       </c>
-      <c r="D207" s="2" t="n"/>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>relationship status</t>
+        </is>
+      </c>
       <c r="E207" s="2" t="n"/>
-      <c r="F207" s="2" t="inlineStr">
-        <is>
-          <t>relationship status</t>
-        </is>
-      </c>
+      <c r="F207" s="2" t="n"/>
       <c r="G207" s="2" t="n"/>
       <c r="H207" s="2" t="n"/>
       <c r="I207" s="2" t="n"/>
@@ -11906,13 +11906,13 @@
           <t>A personal attribute that holds within a given situation.</t>
         </is>
       </c>
-      <c r="D208" s="2" t="n"/>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E208" s="2" t="n"/>
-      <c r="F208" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F208" s="2" t="n"/>
       <c r="G208" s="2" t="n"/>
       <c r="H208" s="2" t="n"/>
       <c r="I208" s="2" t="n"/>
@@ -11953,13 +11953,13 @@
           <t>A social grouping that identifies as such and sometimes acts collectively.</t>
         </is>
       </c>
-      <c r="D209" s="2" t="n"/>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>social grouping</t>
+        </is>
+      </c>
       <c r="E209" s="2" t="n"/>
-      <c r="F209" s="2" t="inlineStr">
-        <is>
-          <t>social grouping</t>
-        </is>
-      </c>
+      <c r="F209" s="2" t="n"/>
       <c r="G209" s="2" t="n"/>
       <c r="H209" s="2" t="n"/>
       <c r="I209" s="2" t="n"/>
@@ -12000,13 +12000,13 @@
           <t>A human population who share some common attribute that involves some form of social interaction.</t>
         </is>
       </c>
-      <c r="D210" s="2" t="n"/>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>human population</t>
+        </is>
+      </c>
       <c r="E210" s="2" t="n"/>
-      <c r="F210" s="2" t="inlineStr">
-        <is>
-          <t>human population</t>
-        </is>
-      </c>
+      <c r="F210" s="2" t="n"/>
       <c r="G210" s="2" t="n"/>
       <c r="H210" s="2" t="n"/>
       <c r="I210" s="2" t="n"/>
@@ -12051,13 +12051,13 @@
           <t>A personal role that is realised in human social processes.</t>
         </is>
       </c>
-      <c r="D211" s="2" t="n"/>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>personal role</t>
+        </is>
+      </c>
       <c r="E211" s="2" t="n"/>
-      <c r="F211" s="2" t="inlineStr">
-        <is>
-          <t>personal role</t>
-        </is>
-      </c>
+      <c r="F211" s="2" t="n"/>
       <c r="G211" s="2" t="n"/>
       <c r="H211" s="2" t="n"/>
       <c r="I211" s="2" t="n"/>
@@ -12098,13 +12098,13 @@
           <t>A &lt;personal attribute&gt; that, together with other attributes, characterises a person’s position in society.</t>
         </is>
       </c>
-      <c r="D212" s="2" t="n"/>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E212" s="2" t="n"/>
-      <c r="F212" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F212" s="2" t="n"/>
       <c r="G212" s="2" t="n"/>
       <c r="H212" s="2" t="n"/>
       <c r="I212" s="2" t="n"/>
@@ -12149,13 +12149,13 @@
           <t>A personal attribute reflecting a person's economic and social position in relation to others</t>
         </is>
       </c>
-      <c r="D213" s="2" t="n"/>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E213" s="2" t="n"/>
-      <c r="F213" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F213" s="2" t="n"/>
       <c r="G213" s="2" t="inlineStr">
         <is>
           <t>OPMI:0000121</t>
@@ -12208,13 +12208,13 @@
           <t xml:space="preserve">A data item about a score on a measure of a person's socioeconomic position, calculated by combining information about the number of years of education completed, their individual or household income, their current occupation or the industry in which they work or family size or household. </t>
         </is>
       </c>
-      <c r="D214" s="2" t="n"/>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
       <c r="E214" s="2" t="n"/>
-      <c r="F214" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
+      <c r="F214" s="2" t="n"/>
       <c r="G214" s="2" t="n"/>
       <c r="H214" s="2" t="n"/>
       <c r="I214" s="2" t="n"/>
@@ -12267,20 +12267,20 @@
           <t xml:space="preserve">A  data item about a category assigned to a person based on an assessment of a score calculated from various measures of their income, education, occupation, family size or household. </t>
         </is>
       </c>
-      <c r="D215" s="3" t="n"/>
+      <c r="D215" s="3" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
       <c r="E215" s="3" t="n"/>
       <c r="F215" s="3" t="inlineStr">
         <is>
-          <t>data item</t>
+          <t>Semi-routine and routine occupations, blue collar occupations</t>
         </is>
       </c>
       <c r="G215" s="3" t="n"/>
       <c r="H215" s="3" t="n"/>
-      <c r="I215" s="3" t="inlineStr">
-        <is>
-          <t>Semi-routine and routine occupations, blue collar occupations</t>
-        </is>
-      </c>
+      <c r="I215" s="3" t="n"/>
       <c r="J215" s="3" t="n"/>
       <c r="K215" s="3" t="inlineStr">
         <is>
@@ -12330,13 +12330,13 @@
           <t>A personal attribute inhering in a person by virtue of that person not bearing a role realised in an employment process, due to being a homemaker whose work includes caring for children.</t>
         </is>
       </c>
-      <c r="D216" s="2" t="n"/>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E216" s="2" t="n"/>
-      <c r="F216" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F216" s="2" t="n"/>
       <c r="G216" s="2" t="inlineStr">
         <is>
           <t>NCIT_C148253</t>
@@ -12389,13 +12389,13 @@
           <t>A parent in a parent-child relationship established by the parent's subsequent marriage to one of the child's original biological or legal parents.</t>
         </is>
       </c>
-      <c r="D217" s="2" t="n"/>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>parent</t>
+        </is>
+      </c>
       <c r="E217" s="2" t="n"/>
-      <c r="F217" s="2" t="inlineStr">
-        <is>
-          <t>parent</t>
-        </is>
-      </c>
+      <c r="F217" s="2" t="n"/>
       <c r="G217" s="2" t="inlineStr">
         <is>
           <t>NCIT:C166116</t>
@@ -12448,13 +12448,13 @@
           <t>A sibling who is the child of one's step-parent.</t>
         </is>
       </c>
-      <c r="D218" s="2" t="n"/>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
       <c r="E218" s="2" t="n"/>
-      <c r="F218" s="2" t="inlineStr">
-        <is>
-          <t>sibling</t>
-        </is>
-      </c>
+      <c r="F218" s="2" t="n"/>
       <c r="G218" s="2" t="n"/>
       <c r="H218" s="2" t="n"/>
       <c r="I218" s="2" t="n"/>
@@ -12503,13 +12503,13 @@
           <t>A step-sibling who is male gender.</t>
         </is>
       </c>
-      <c r="D219" s="2" t="n"/>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>step-sibling</t>
+        </is>
+      </c>
       <c r="E219" s="2" t="n"/>
-      <c r="F219" s="2" t="inlineStr">
-        <is>
-          <t>step-sibling</t>
-        </is>
-      </c>
+      <c r="F219" s="2" t="n"/>
       <c r="G219" s="2" t="n"/>
       <c r="H219" s="2" t="n"/>
       <c r="I219" s="2" t="n"/>
@@ -12558,13 +12558,13 @@
           <t>A child relation in a parent-child relationship established by the parent's subsequent marriage to one of the child's original biological or legal parents.</t>
         </is>
       </c>
-      <c r="D220" s="2" t="n"/>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>child relation</t>
+        </is>
+      </c>
       <c r="E220" s="2" t="n"/>
-      <c r="F220" s="2" t="inlineStr">
-        <is>
-          <t>child relation</t>
-        </is>
-      </c>
+      <c r="F220" s="2" t="n"/>
       <c r="G220" s="2" t="n"/>
       <c r="H220" s="2" t="n"/>
       <c r="I220" s="2" t="n"/>
@@ -12613,13 +12613,13 @@
           <t>A stepchild who is female gender.</t>
         </is>
       </c>
-      <c r="D221" s="2" t="n"/>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>stepchild</t>
+        </is>
+      </c>
       <c r="E221" s="2" t="n"/>
-      <c r="F221" s="2" t="inlineStr">
-        <is>
-          <t>stepchild</t>
-        </is>
-      </c>
+      <c r="F221" s="2" t="n"/>
       <c r="G221" s="2" t="n"/>
       <c r="H221" s="2" t="n"/>
       <c r="I221" s="2" t="n"/>
@@ -12668,13 +12668,13 @@
           <t>A step-parent who is male gender.</t>
         </is>
       </c>
-      <c r="D222" s="2" t="n"/>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>step-parent</t>
+        </is>
+      </c>
       <c r="E222" s="2" t="n"/>
-      <c r="F222" s="2" t="inlineStr">
-        <is>
-          <t>step-parent</t>
-        </is>
-      </c>
+      <c r="F222" s="2" t="n"/>
       <c r="G222" s="2" t="n"/>
       <c r="H222" s="2" t="n"/>
       <c r="I222" s="2" t="n"/>
@@ -12723,13 +12723,13 @@
           <t>A step-parent who is female gender.</t>
         </is>
       </c>
-      <c r="D223" s="2" t="n"/>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>step-parent</t>
+        </is>
+      </c>
       <c r="E223" s="2" t="n"/>
-      <c r="F223" s="2" t="inlineStr">
-        <is>
-          <t>step-parent</t>
-        </is>
-      </c>
+      <c r="F223" s="2" t="n"/>
       <c r="G223" s="2" t="n"/>
       <c r="H223" s="2" t="n"/>
       <c r="I223" s="2" t="n"/>
@@ -12778,13 +12778,13 @@
           <t>A step-sibling who is female gender.</t>
         </is>
       </c>
-      <c r="D224" s="2" t="n"/>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>step-sibling</t>
+        </is>
+      </c>
       <c r="E224" s="2" t="n"/>
-      <c r="F224" s="2" t="inlineStr">
-        <is>
-          <t>step-sibling</t>
-        </is>
-      </c>
+      <c r="F224" s="2" t="n"/>
       <c r="G224" s="2" t="n"/>
       <c r="H224" s="2" t="n"/>
       <c r="I224" s="2" t="n"/>
@@ -12833,13 +12833,13 @@
           <t>A stepchild who is male gender.</t>
         </is>
       </c>
-      <c r="D225" s="2" t="n"/>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>stepchild</t>
+        </is>
+      </c>
       <c r="E225" s="2" t="n"/>
-      <c r="F225" s="2" t="inlineStr">
-        <is>
-          <t>stepchild</t>
-        </is>
-      </c>
+      <c r="F225" s="2" t="n"/>
       <c r="G225" s="2" t="n"/>
       <c r="H225" s="2" t="n"/>
       <c r="I225" s="2" t="n"/>
@@ -12888,13 +12888,13 @@
           <t>A role which inheres in a person and is realised by being enrolled in an educational institution or a formal programme of professional training.</t>
         </is>
       </c>
-      <c r="D226" s="2" t="n"/>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
       <c r="E226" s="2" t="n"/>
-      <c r="F226" s="2" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
+      <c r="F226" s="2" t="n"/>
       <c r="G226" s="2" t="n"/>
       <c r="H226" s="2" t="n"/>
       <c r="I226" s="2" t="n"/>
@@ -12943,7 +12943,7 @@
           <t>A person between 13 and 19 years of age.</t>
         </is>
       </c>
-      <c r="F227" t="inlineStr">
+      <c r="D227" t="inlineStr">
         <is>
           <t>person</t>
         </is>
@@ -12985,13 +12985,13 @@
           <t>A student or trainee role that is currently learning the curriculum material of vocational programme, normally in preparation for employment in a trade, job or profession.</t>
         </is>
       </c>
-      <c r="D228" s="2" t="n"/>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>student or trainee role</t>
+        </is>
+      </c>
       <c r="E228" s="2" t="n"/>
-      <c r="F228" s="2" t="inlineStr">
-        <is>
-          <t>student or trainee role</t>
-        </is>
-      </c>
+      <c r="F228" s="2" t="n"/>
       <c r="G228" s="2" t="n"/>
       <c r="H228" s="2" t="n"/>
       <c r="I228" s="2" t="n"/>
@@ -13040,13 +13040,13 @@
           <t>A gender identity that differs from the person's assigned sex at birth.</t>
         </is>
       </c>
-      <c r="D229" s="2" t="n"/>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>gender identity</t>
+        </is>
+      </c>
       <c r="E229" s="2" t="n"/>
-      <c r="F229" s="2" t="inlineStr">
-        <is>
-          <t>gender identity</t>
-        </is>
-      </c>
+      <c r="F229" s="2" t="n"/>
       <c r="G229" s="2" t="inlineStr">
         <is>
           <t>GSSO:000096</t>
@@ -13099,13 +13099,13 @@
           <t xml:space="preserve">One of two siblings who resulted from the same pregnancy. </t>
         </is>
       </c>
-      <c r="D230" s="2" t="n"/>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
       <c r="E230" s="2" t="n"/>
-      <c r="F230" s="2" t="inlineStr">
-        <is>
-          <t>sibling</t>
-        </is>
-      </c>
+      <c r="F230" s="2" t="n"/>
       <c r="G230" s="2" t="n"/>
       <c r="H230" s="2" t="n"/>
       <c r="I230" s="2" t="n"/>
@@ -13154,13 +13154,13 @@
           <t>A situational personal attribute in which a person has not thought about enacting a behaviour.</t>
         </is>
       </c>
-      <c r="D231" s="2" t="n"/>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>situational personal attribute</t>
+        </is>
+      </c>
       <c r="E231" s="2" t="n"/>
-      <c r="F231" s="2" t="inlineStr">
-        <is>
-          <t>situational personal attribute</t>
-        </is>
-      </c>
+      <c r="F231" s="2" t="n"/>
       <c r="G231" s="2" t="n"/>
       <c r="H231" s="2" t="n"/>
       <c r="I231" s="2" t="n"/>
@@ -13209,13 +13209,13 @@
           <t>A family member who is the brother of one's parent.</t>
         </is>
       </c>
-      <c r="D232" s="2" t="n"/>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>family member</t>
+        </is>
+      </c>
       <c r="E232" s="2" t="n"/>
-      <c r="F232" s="2" t="inlineStr">
-        <is>
-          <t>family member</t>
-        </is>
-      </c>
+      <c r="F232" s="2" t="n"/>
       <c r="G232" s="2" t="n"/>
       <c r="H232" s="2" t="n"/>
       <c r="I232" s="2" t="n"/>
@@ -13264,13 +13264,13 @@
           <t>A situational personal attribute in which the person has thought about a behaviour but not formed an intention regarding whether to enact it.</t>
         </is>
       </c>
-      <c r="D233" s="2" t="n"/>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>situational personal attribute</t>
+        </is>
+      </c>
       <c r="E233" s="2" t="n"/>
-      <c r="F233" s="2" t="inlineStr">
-        <is>
-          <t>situational personal attribute</t>
-        </is>
-      </c>
+      <c r="F233" s="2" t="n"/>
       <c r="G233" s="2" t="n"/>
       <c r="H233" s="2" t="n"/>
       <c r="I233" s="2" t="n"/>
@@ -13319,13 +13319,13 @@
           <t>A higher education student role realised by currently studying for an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D234" s="3" t="n"/>
+      <c r="D234" s="3" t="inlineStr">
+        <is>
+          <t>higher education student role</t>
+        </is>
+      </c>
       <c r="E234" s="3" t="n"/>
-      <c r="F234" s="3" t="inlineStr">
-        <is>
-          <t>higher education student role</t>
-        </is>
-      </c>
+      <c r="F234" s="3" t="n"/>
       <c r="G234" s="3" t="n"/>
       <c r="H234" s="3" t="n"/>
       <c r="I234" s="3" t="n"/>
@@ -13374,13 +13374,13 @@
           <t>A higher education student role realised by currently studying for an undergraduate degree.</t>
         </is>
       </c>
-      <c r="D235" s="2" t="n"/>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>higher education student role</t>
+        </is>
+      </c>
       <c r="E235" s="2" t="n"/>
-      <c r="F235" s="2" t="inlineStr">
-        <is>
-          <t>higher education student role</t>
-        </is>
-      </c>
+      <c r="F235" s="2" t="n"/>
       <c r="G235" s="2" t="n"/>
       <c r="H235" s="2" t="n"/>
       <c r="I235" s="2" t="n"/>
@@ -13429,13 +13429,13 @@
           <t>An employment status in which the person is not employed or self-employed, is looking for work and able to start in paid employment.</t>
         </is>
       </c>
-      <c r="D236" s="2" t="n"/>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>employment status</t>
+        </is>
+      </c>
       <c r="E236" s="2" t="n"/>
-      <c r="F236" s="2" t="inlineStr">
-        <is>
-          <t>employment status</t>
-        </is>
-      </c>
+      <c r="F236" s="2" t="n"/>
       <c r="G236" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">SDGIO_00010026 </t>
@@ -13488,13 +13488,13 @@
           <t>A personal attribute inhering in a person by virtue of that person not bearing a role realised in an employment process, due to their primary occupation being caring, without receiving a wage for it, for an adult friend or family member who, due to illness or disability, requires support in their daily life activities.</t>
         </is>
       </c>
-      <c r="D237" s="2" t="n"/>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E237" s="2" t="n"/>
-      <c r="F237" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F237" s="2" t="n"/>
       <c r="G237" s="2" t="n"/>
       <c r="H237" s="2" t="n"/>
       <c r="I237" s="2" t="n"/>
@@ -13543,11 +13543,15 @@
           <t>An object aggregate under the control of some person or organisation which confers an economic benefit to that person or organisation in an economic system.</t>
         </is>
       </c>
-      <c r="D238" s="2" t="n"/>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
       <c r="E238" s="2" t="n"/>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>object aggregate</t>
+          <t>farmland, jewellery, livestock</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -13556,11 +13560,7 @@
         </is>
       </c>
       <c r="H238" s="2" t="n"/>
-      <c r="I238" s="2" t="inlineStr">
-        <is>
-          <t>farmland, jewellery, livestock</t>
-        </is>
-      </c>
+      <c r="I238" s="2" t="n"/>
       <c r="J238" s="2" t="n"/>
       <c r="K238" s="2" t="inlineStr">
         <is>
@@ -13598,20 +13598,20 @@
           <t>A data item about the monetary value of a valuable material resource possessed by a person.</t>
         </is>
       </c>
-      <c r="D239" s="2" t="n"/>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
       <c r="E239" s="2" t="n"/>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>data item</t>
+          <t>$400, 3000 euros</t>
         </is>
       </c>
       <c r="G239" s="2" t="n"/>
       <c r="H239" s="2" t="n"/>
-      <c r="I239" s="2" t="inlineStr">
-        <is>
-          <t>$400, 3000 euros</t>
-        </is>
-      </c>
+      <c r="I239" s="2" t="n"/>
       <c r="J239" s="2" t="n"/>
       <c r="K239" s="2" t="inlineStr">
         <is>
@@ -13661,13 +13661,13 @@
           <t>A student or trainee role realised by currently learning the curriculum material of vocational programme, normally in preparation for employment in a trade, job or profession.</t>
         </is>
       </c>
-      <c r="D240" s="3" t="n"/>
+      <c r="D240" s="3" t="inlineStr">
+        <is>
+          <t>student or trainee role</t>
+        </is>
+      </c>
       <c r="E240" s="3" t="n"/>
-      <c r="F240" s="3" t="inlineStr">
-        <is>
-          <t>student or trainee role</t>
-        </is>
-      </c>
+      <c r="F240" s="3" t="n"/>
       <c r="G240" s="3" t="n"/>
       <c r="H240" s="3" t="n"/>
       <c r="I240" s="3" t="n"/>
@@ -13716,13 +13716,13 @@
           <t>A personal attribute inhering in a person by virtue of that person working or assisting at a workplace without receiving remuneration.</t>
         </is>
       </c>
-      <c r="D241" s="2" t="n"/>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>personal attribute</t>
+        </is>
+      </c>
       <c r="E241" s="2" t="n"/>
-      <c r="F241" s="2" t="inlineStr">
-        <is>
-          <t>personal attribute</t>
-        </is>
-      </c>
+      <c r="F241" s="2" t="n"/>
       <c r="G241" s="2" t="n"/>
       <c r="H241" s="2" t="n"/>
       <c r="I241" s="2" t="n"/>
@@ -13775,13 +13775,13 @@
           <t xml:space="preserve">A relationship status where the individual is no longer in a legally formalised marriage or civil partnership due to the death of their spouse or partner. </t>
         </is>
       </c>
-      <c r="D242" s="2" t="n"/>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>relationship status</t>
+        </is>
+      </c>
       <c r="E242" s="2" t="n"/>
-      <c r="F242" s="2" t="inlineStr">
-        <is>
-          <t>relationship status</t>
-        </is>
-      </c>
+      <c r="F242" s="2" t="n"/>
       <c r="G242" s="2" t="n"/>
       <c r="H242" s="2" t="n"/>
       <c r="I242" s="2" t="n"/>

</xml_diff>

<commit_message>
Update Curation status of household income in BCIO_Population.xlsx
</commit_message>
<xml_diff>
--- a/Population/BCIO_Population.xlsx
+++ b/Population/BCIO_Population.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,11 @@
         <fgColor rgb="002f4f4f"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ffffff"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -60,11 +65,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6196,67 +6202,67 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="3" t="inlineStr">
+      <c r="A103" s="4" t="inlineStr">
         <is>
           <t>BCIO:015027</t>
         </is>
       </c>
-      <c r="B103" s="3" t="inlineStr">
+      <c r="B103" s="4" t="inlineStr">
         <is>
           <t>household income</t>
         </is>
       </c>
-      <c r="C103" s="3" t="inlineStr">
+      <c r="C103" s="4" t="inlineStr">
         <is>
           <t>An aggregate of the individual incomes received by all the members of a household.</t>
         </is>
       </c>
-      <c r="D103" s="3" t="inlineStr">
+      <c r="D103" s="4" t="inlineStr">
         <is>
           <t>object aggregate</t>
         </is>
       </c>
-      <c r="E103" s="3" t="n"/>
-      <c r="F103" s="3" t="n"/>
-      <c r="G103" s="3" t="inlineStr">
+      <c r="E103" s="4" t="n"/>
+      <c r="F103" s="4" t="n"/>
+      <c r="G103" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">EFO_0009695 </t>
         </is>
       </c>
-      <c r="H103" s="3" t="n"/>
-      <c r="I103" s="3" t="n"/>
-      <c r="J103" s="3" t="n"/>
-      <c r="K103" s="3" t="inlineStr">
-        <is>
-          <t>population</t>
-        </is>
-      </c>
-      <c r="L103" s="3" t="inlineStr">
+      <c r="H103" s="4" t="n"/>
+      <c r="I103" s="4" t="n"/>
+      <c r="J103" s="4" t="n"/>
+      <c r="K103" s="4" t="inlineStr">
+        <is>
+          <t>population</t>
+        </is>
+      </c>
+      <c r="L103" s="4" t="inlineStr">
         <is>
           <t>household</t>
         </is>
       </c>
-      <c r="M103" s="3" t="n"/>
-      <c r="N103" s="3" t="inlineStr">
+      <c r="M103" s="4" t="n"/>
+      <c r="N103" s="4" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="O103" s="3" t="n"/>
-      <c r="P103" s="3" t="n"/>
-      <c r="Q103" s="3" t="inlineStr">
+      <c r="O103" s="4" t="n"/>
+      <c r="P103" s="4" t="n"/>
+      <c r="Q103" s="4" t="inlineStr">
         <is>
           <t>Mean;Minimum;Maximum;Median; percentage; proportion</t>
         </is>
       </c>
-      <c r="R103" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S103" s="3" t="n"/>
-      <c r="T103" s="3" t="n"/>
-      <c r="U103" s="3" t="n"/>
+      <c r="R103" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="S103" s="4" t="n"/>
+      <c r="T103" s="4" t="n"/>
+      <c r="U103" s="4" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update income-related welfare benefit in BCIO_Population.xlsx
</commit_message>
<xml_diff>
--- a/Population/BCIO_Population.xlsx
+++ b/Population/BCIO_Population.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,11 @@
         <fgColor rgb="002f4f4f"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ffe4b5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -60,11 +65,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6732,59 +6738,59 @@
       <c r="U112" s="2" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="3" t="inlineStr">
+      <c r="A113" s="4" t="inlineStr">
         <is>
           <t>BCIO:015037</t>
         </is>
       </c>
-      <c r="B113" s="3" t="inlineStr">
+      <c r="B113" s="4" t="inlineStr">
         <is>
           <t>income-related welfare benefit</t>
         </is>
       </c>
-      <c r="C113" s="3" t="inlineStr">
+      <c r="C113" s="4" t="inlineStr">
         <is>
           <t>Individual income that an individual otherwise of low-income receives as a payment made by the state or an insurance scheme in the form of housing vouchers,  credit or benefits.</t>
         </is>
       </c>
-      <c r="D113" s="3" t="inlineStr">
+      <c r="D113" s="4" t="inlineStr">
         <is>
           <t>individual income</t>
         </is>
       </c>
-      <c r="E113" s="3" t="n"/>
-      <c r="F113" s="3" t="n"/>
-      <c r="G113" s="3" t="n"/>
-      <c r="H113" s="3" t="n"/>
-      <c r="I113" s="3" t="n"/>
-      <c r="J113" s="3" t="n"/>
-      <c r="K113" s="3" t="inlineStr">
-        <is>
-          <t>population</t>
-        </is>
-      </c>
-      <c r="L113" s="3" t="n"/>
-      <c r="M113" s="3" t="n"/>
-      <c r="N113" s="3" t="inlineStr">
+      <c r="E113" s="4" t="n"/>
+      <c r="F113" s="4" t="n"/>
+      <c r="G113" s="4" t="n"/>
+      <c r="H113" s="4" t="n"/>
+      <c r="I113" s="4" t="n"/>
+      <c r="J113" s="4" t="n"/>
+      <c r="K113" s="4" t="inlineStr">
+        <is>
+          <t>population</t>
+        </is>
+      </c>
+      <c r="L113" s="4" t="n"/>
+      <c r="M113" s="4" t="n"/>
+      <c r="N113" s="4" t="inlineStr">
         <is>
           <t>past behaviour</t>
         </is>
       </c>
-      <c r="O113" s="3" t="n"/>
-      <c r="P113" s="3" t="n"/>
-      <c r="Q113" s="3" t="inlineStr">
-        <is>
-          <t>percentage; proportion</t>
-        </is>
-      </c>
-      <c r="R113" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S113" s="3" t="n"/>
-      <c r="T113" s="3" t="n"/>
-      <c r="U113" s="3" t="n"/>
+      <c r="O113" s="4" t="n"/>
+      <c r="P113" s="4" t="n"/>
+      <c r="Q113" s="4" t="inlineStr">
+        <is>
+          <t>percentage; proportion</t>
+        </is>
+      </c>
+      <c r="R113" s="4" t="inlineStr">
+        <is>
+          <t>Discussed</t>
+        </is>
+      </c>
+      <c r="S113" s="4" t="n"/>
+      <c r="T113" s="4" t="n"/>
+      <c r="U113" s="4" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">

</xml_diff>